<commit_message>
Mark outreach emails as sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -563,7 +563,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -634,7 +638,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>United States</t>
@@ -710,7 +718,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Estonia</t>
@@ -785,7 +797,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -856,7 +872,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -928,7 +948,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -999,7 +1023,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1070,7 +1098,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1141,7 +1173,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Brazil</t>
@@ -1216,7 +1252,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Cyprus</t>
@@ -1296,7 +1336,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Montenegro</t>
@@ -1372,7 +1416,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Thailand</t>
@@ -1448,7 +1496,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>United States</t>
@@ -1523,7 +1575,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1654,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Benin</t>
@@ -1673,7 +1733,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1744,7 +1808,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -1815,7 +1883,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
@@ -1886,7 +1958,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
@@ -1957,7 +2033,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Brazil</t>
@@ -2032,7 +2112,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>India</t>
@@ -2107,7 +2191,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n"/>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -2182,7 +2270,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-28</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>United Kingdom</t>

</xml_diff>

<commit_message>
Update outreach status after resend from correct account
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -565,7 +565,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -640,7 +640,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Contacted 2026-09-26 from oseniibrahim845@gmail.com (not resent)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -874,7 +874,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Contacted 2026-09-26 from oseniibrahim845@gmail.com (not resent)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -950,7 +950,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Bounced (address undeliverable)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1418,7 +1418,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Contacted 2026-09-26 from oseniibrahim845@gmail.com (not resent)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28</t>
+          <t>Sent 2026-09-28 from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Record 6 bounces from batch 1; add MX pre-check to outreach runbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -2745,7 +2745,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28 14:35 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-28 15:23 UTC)</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28 14:35 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-28 15:23 UTC)</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28 14:35 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-28 15:23 UTC)</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3520,7 +3520,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28 14:35 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-28 15:23 UTC)</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28 14:35 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-28 15:23 UTC)</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Sent 2026-09-28 14:35 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-28 15:23 UTC)</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -4421,7 +4421,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Skipped no mail server (2026-09-28 15:24 UTC)</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Skipped no mail server (2026-09-28 15:24 UTC)</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Skipped no mail server (2026-09-28 15:24 UTC)</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Skipped no mail server (2026-09-28 15:24 UTC)</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">

</xml_diff>

<commit_message>
Outreach batch 2: 25 sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -4275,7 +4275,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4871,7 +4871,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -5247,7 +5247,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -5496,7 +5496,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -5735,7 +5735,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -5813,7 +5813,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -6052,7 +6052,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6135,7 +6135,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -6296,7 +6296,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -6452,7 +6452,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 16:39 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -9419,7 +9419,6 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" t="inlineStr"/>
       <c r="B116" t="inlineStr">
         <is>
           <t>AlphaTRADER</t>
@@ -9607,7 +9606,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
       <c r="I118" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -9645,7 +9643,6 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" t="inlineStr"/>
       <c r="B119" t="inlineStr">
         <is>
           <t>Bitbash</t>
@@ -9757,7 +9754,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -9831,7 +9827,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
       <c r="I121" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -9905,7 +9900,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
       <c r="I122" t="inlineStr">
         <is>
           <t>Fintech / blockchain development</t>
@@ -10099,7 +10093,6 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" t="inlineStr"/>
       <c r="B125" t="inlineStr">
         <is>
           <t>ByTamerFX</t>
@@ -10131,7 +10124,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -10205,7 +10197,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr">
         <is>
           <t>Software / trading tools</t>
@@ -10243,7 +10234,6 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr"/>
       <c r="B127" t="inlineStr">
         <is>
           <t>Nodalytics</t>
@@ -10275,7 +10265,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr">
         <is>
           <t>Proprietary quantitative trading</t>
@@ -10313,7 +10302,6 @@
       </c>
     </row>
     <row r="128">
-      <c r="A128" t="inlineStr"/>
       <c r="B128" t="inlineStr">
         <is>
           <t>Trade Vectors LLP</t>
@@ -10387,7 +10375,6 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr"/>
       <c r="B129" t="inlineStr">
         <is>
           <t>ProChart XAUUSD (kipli.net)</t>
@@ -10419,7 +10406,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
       <c r="I129" t="inlineStr">
         <is>
           <t>Trading tools / custom development</t>
@@ -10457,7 +10443,6 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr"/>
       <c r="B130" t="inlineStr">
         <is>
           <t>Copiix</t>
@@ -10531,7 +10516,6 @@
       </c>
     </row>
     <row r="131">
-      <c r="A131" t="inlineStr"/>
       <c r="B131" t="inlineStr">
         <is>
           <t>Fintechee</t>
@@ -10563,7 +10547,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
       <c r="I131" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10601,7 +10584,6 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr"/>
       <c r="B132" t="inlineStr">
         <is>
           <t>Fivitech</t>
@@ -10633,7 +10615,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
       <c r="I132" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10671,7 +10652,6 @@
       </c>
     </row>
     <row r="133">
-      <c r="A133" t="inlineStr"/>
       <c r="B133" t="inlineStr">
         <is>
           <t>MetaRPC</t>
@@ -10703,7 +10683,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10741,7 +10720,6 @@
       </c>
     </row>
     <row r="134">
-      <c r="A134" t="inlineStr"/>
       <c r="B134" t="inlineStr">
         <is>
           <t>LuxAlgo</t>
@@ -10893,7 +10871,6 @@
       </c>
     </row>
     <row r="136">
-      <c r="A136" t="inlineStr"/>
       <c r="B136" t="inlineStr">
         <is>
           <t>FxSocket</t>
@@ -10925,7 +10902,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
       <c r="I136" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10963,7 +10939,6 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr"/>
       <c r="B137" t="inlineStr">
         <is>
           <t>XBTFX</t>
@@ -10995,7 +10970,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
       <c r="I137" t="inlineStr">
         <is>
           <t>Forex brokerage technology</t>
@@ -11033,7 +11007,6 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" t="inlineStr"/>
       <c r="B138" t="inlineStr">
         <is>
           <t>Yuants (ntnl.io)</t>
@@ -11065,7 +11038,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
       <c r="I138" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -11103,7 +11075,6 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" t="inlineStr"/>
       <c r="B139" t="inlineStr">
         <is>
           <t>OrvaLabs</t>
@@ -11135,7 +11106,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
       <c r="I139" t="inlineStr">
         <is>
           <t>AI trading systems</t>
@@ -11287,7 +11257,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr">
         <is>
           <t>Trading systems</t>
@@ -11361,7 +11330,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
       <c r="I142" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -11747,7 +11715,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
       <c r="I147" t="inlineStr">
         <is>
           <t>Software development</t>
@@ -11821,7 +11788,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
       <c r="I148" t="inlineStr">
         <is>
           <t>Trading framework</t>
@@ -11859,7 +11825,6 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr"/>
       <c r="B149" t="inlineStr">
         <is>
           <t>DaedalusFX</t>
@@ -11891,7 +11856,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
       <c r="I149" t="inlineStr">
         <is>
           <t>MT5 trade management tools</t>
@@ -12085,7 +12049,6 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="inlineStr"/>
       <c r="B152" t="inlineStr">
         <is>
           <t>LoanXfer</t>
@@ -12117,7 +12080,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
       <c r="I152" t="inlineStr">
         <is>
           <t>Freelance trading software</t>
@@ -12233,7 +12195,6 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr"/>
       <c r="B154" t="inlineStr">
         <is>
           <t>Dewyndl</t>
@@ -12265,7 +12226,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
       <c r="I154" t="inlineStr">
         <is>
           <t>Freelance software development</t>
@@ -12339,7 +12299,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
       <c r="I155" t="inlineStr">
         <is>
           <t>Trading indicators</t>
@@ -12413,7 +12372,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
       <c r="I156" t="inlineStr">
         <is>
           <t>Trading education</t>
@@ -12565,7 +12523,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
       <c r="I158" t="inlineStr">
         <is>
           <t>MQL developer tooling</t>
@@ -12603,7 +12560,6 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr"/>
       <c r="B159" t="inlineStr">
         <is>
           <t>AtingMQL5</t>
@@ -12635,7 +12591,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
       <c r="I159" t="inlineStr">
         <is>
           <t>MQL5 libraries</t>
@@ -12709,7 +12664,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
       <c r="I160" t="inlineStr">
         <is>
           <t>Trading strategy development</t>
@@ -12783,7 +12737,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
       <c r="I161" t="inlineStr">
         <is>
           <t>Software development</t>
@@ -12857,7 +12810,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
       <c r="I162" t="inlineStr">
         <is>
           <t>Quant research</t>
@@ -12973,7 +12925,6 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr"/>
       <c r="B164" t="inlineStr">
         <is>
           <t>BigHeroAI</t>
@@ -13005,7 +12956,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
       <c r="I164" t="inlineStr">
         <is>
           <t>AI trading systems</t>
@@ -13043,7 +12993,6 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="inlineStr"/>
       <c r="B165" t="inlineStr">
         <is>
           <t>Ishaan Nasir</t>
@@ -13153,7 +13102,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
       <c r="I166" t="inlineStr">
         <is>
           <t>Algorithmic trading</t>
@@ -13269,7 +13217,6 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr"/>
       <c r="B168" t="inlineStr">
         <is>
           <t>Ahmed GoCode</t>
@@ -13343,7 +13290,6 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="inlineStr"/>
       <c r="B169" t="inlineStr">
         <is>
           <t>pixiu (tradepython)</t>
@@ -13376,7 +13322,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
       <c r="I169" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -13809,7 +13754,6 @@
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr"/>
       <c r="B175" t="inlineStr">
         <is>
           <t>Fuzzy Technologies</t>
@@ -13884,7 +13828,6 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="inlineStr"/>
       <c r="B176" t="inlineStr">
         <is>
           <t>xyz0217 (MT4 Position Helper)</t>
@@ -13917,7 +13860,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
       <c r="I176" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -14459,7 +14401,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
       <c r="I183" t="inlineStr">
         <is>
           <t>Trading software / fintech UI</t>
@@ -14767,7 +14708,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
       <c r="I187" t="inlineStr">
         <is>
           <t>Quantitative trading</t>
@@ -14883,7 +14823,6 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr"/>
       <c r="B189" t="inlineStr">
         <is>
           <t>marketprolab (NexoProyect)</t>
@@ -14915,7 +14854,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
       <c r="I189" t="inlineStr">
         <is>
           <t>Trading software / backtesting</t>
@@ -15223,7 +15161,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
       <c r="I193" t="inlineStr">
         <is>
           <t>Trading software framework</t>
@@ -15531,7 +15468,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
       <c r="I197" t="inlineStr">
         <is>
           <t>Quant trading tooling</t>
@@ -15605,7 +15541,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
       <c r="I198" t="inlineStr">
         <is>
           <t>Trading software framework</t>
@@ -15955,7 +15890,6 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr"/>
       <c r="B203" t="inlineStr">
         <is>
           <t>LogicCrafterDZ</t>
@@ -16065,7 +15999,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
       <c r="I204" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -16103,7 +16036,6 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr"/>
       <c r="B205" t="inlineStr">
         <is>
           <t>Multi-Pair Grid Trading Manager (IU Technical)</t>
@@ -16135,7 +16067,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
       <c r="I205" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -16173,7 +16104,6 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="inlineStr"/>
       <c r="B206" t="inlineStr">
         <is>
           <t>ALSHAHEEN</t>
@@ -16205,7 +16135,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
       <c r="I206" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -16435,7 +16364,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
       <c r="I209" t="inlineStr">
         <is>
           <t>MT5 indicator development</t>
@@ -16587,7 +16515,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
       <c r="I211" t="inlineStr">
         <is>
           <t>Algorithmic trading / AI</t>
@@ -16703,7 +16630,6 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr"/>
       <c r="B213" t="inlineStr">
         <is>
           <t>BotTrade Workspace (rangsarn)</t>
@@ -16891,7 +16817,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
       <c r="I215" t="inlineStr">
         <is>
           <t>EA development services</t>
@@ -16965,7 +16890,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
       <c r="I216" t="inlineStr">
         <is>
           <t>Algorithmic trading / AI</t>
@@ -17039,7 +16963,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
       <c r="I217" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -17113,7 +17036,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
       <c r="I218" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -17187,7 +17109,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
       <c r="I219" t="inlineStr">
         <is>
           <t>Algorithmic trading / ML</t>
@@ -17225,7 +17146,6 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" t="inlineStr"/>
       <c r="B220" t="inlineStr">
         <is>
           <t>MQ5 Copy Trading Bot (gold-mouse)</t>
@@ -17257,7 +17177,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
       <c r="I220" t="inlineStr">
         <is>
           <t>Trade copier software</t>
@@ -17331,7 +17250,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
       <c r="I221" t="inlineStr">
         <is>
           <t>MQL5 development</t>
@@ -17405,7 +17323,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
       <c r="I222" t="inlineStr">
         <is>
           <t>Signal distribution / trading technology</t>
@@ -17479,7 +17396,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
       <c r="I223" t="inlineStr">
         <is>
           <t>Algorithmic trading / software</t>
@@ -17517,7 +17433,6 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" t="inlineStr"/>
       <c r="B224" t="inlineStr">
         <is>
           <t>EA Punokawan</t>
@@ -17627,7 +17542,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
       <c r="I225" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -17665,7 +17579,6 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" t="inlineStr"/>
       <c r="B226" t="inlineStr">
         <is>
           <t>EA Perfect FX</t>
@@ -17775,7 +17688,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
       <c r="I227" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -17813,7 +17725,6 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" t="inlineStr"/>
       <c r="B228" t="inlineStr">
         <is>
           <t>TradeDash MT5 EA</t>
@@ -17845,7 +17756,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
       <c r="I228" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -17961,7 +17871,6 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" t="inlineStr"/>
       <c r="B230" t="inlineStr">
         <is>
           <t>MX Forex Trader</t>
@@ -17993,7 +17902,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
       <c r="I230" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -18145,7 +18053,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
       <c r="I232" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -18261,7 +18168,6 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" t="inlineStr"/>
       <c r="B234" t="inlineStr">
         <is>
           <t>Monarch Trades (Deriv Pro)</t>
@@ -18371,7 +18277,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
       <c r="I235" t="inlineStr">
         <is>
           <t>Trading education</t>
@@ -18601,7 +18506,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
       <c r="I238" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -18675,7 +18579,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
       <c r="I239" t="inlineStr">
         <is>
           <t>Trading account monitoring</t>
@@ -18749,7 +18652,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
       <c r="I240" t="inlineStr">
         <is>
           <t>Trade copier software</t>
@@ -19213,7 +19115,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
       <c r="I246" t="inlineStr">
         <is>
           <t>Automated trading infrastructure</t>
@@ -19287,7 +19188,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr">
         <is>
           <t>MQL5 tools</t>
@@ -19439,7 +19339,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
       <c r="I249" t="inlineStr">
         <is>
           <t>Forex EA / indicator vendor</t>
@@ -19477,7 +19376,6 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" t="inlineStr"/>
       <c r="B250" t="inlineStr">
         <is>
           <t>Madarik Trader Pro</t>
@@ -19509,7 +19407,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
       <c r="I250" t="inlineStr">
         <is>
           <t>Trading bot software</t>
@@ -19781,7 +19678,6 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" t="inlineStr"/>
       <c r="B254" t="inlineStr">
         <is>
           <t>MT5-Bridge-TradingView (mastermobdev)</t>
@@ -19813,7 +19709,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
       <c r="I254" t="inlineStr">
         <is>
           <t>TradingView to MT5 bridge</t>
@@ -19887,7 +19782,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
       <c r="I255" t="inlineStr">
         <is>
           <t>MT5 trade copier software</t>
@@ -19925,7 +19819,6 @@
       </c>
     </row>
     <row r="256">
-      <c r="A256" t="inlineStr"/>
       <c r="B256" t="inlineStr">
         <is>
           <t>Simple AlgoTrading Solutions (Gold Daily Breakout EA)</t>
@@ -19957,7 +19850,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
       <c r="I256" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -20031,7 +19923,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
       <c r="I257" t="inlineStr">
         <is>
           <t>Algorithmic trading / quant research</t>
@@ -20105,7 +19996,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
       <c r="I258" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -20221,7 +20111,6 @@
       </c>
     </row>
     <row r="260">
-      <c r="A260" t="inlineStr"/>
       <c r="B260" t="inlineStr">
         <is>
           <t>AI Backtester (R1CZ)</t>
@@ -20253,7 +20142,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
       <c r="I260" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -20291,7 +20179,6 @@
       </c>
     </row>
     <row r="261">
-      <c r="A261" t="inlineStr"/>
       <c r="B261" t="inlineStr">
         <is>
           <t>JIG BOT</t>
@@ -20323,7 +20210,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
       <c r="I261" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -20361,7 +20247,6 @@
       </c>
     </row>
     <row r="262">
-      <c r="A262" t="inlineStr"/>
       <c r="B262" t="inlineStr">
         <is>
           <t>Telegram Signal to MT5 Auto Trader (Shokh-akf)</t>
@@ -20393,7 +20278,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
       <c r="I262" t="inlineStr">
         <is>
           <t>Telegram signal copier software</t>
@@ -20431,7 +20315,6 @@
       </c>
     </row>
     <row r="263">
-      <c r="A263" t="inlineStr"/>
       <c r="B263" t="inlineStr">
         <is>
           <t>OrderFlow Core (kawacoline)</t>
@@ -20463,7 +20346,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
       <c r="I263" t="inlineStr">
         <is>
           <t>Algorithmic trading systems</t>
@@ -20501,7 +20383,6 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" t="inlineStr"/>
       <c r="B264" t="inlineStr">
         <is>
           <t>Ophireum (SYMMETRIX GOLD SMC)</t>
@@ -20611,7 +20492,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
       <c r="I265" t="inlineStr">
         <is>
           <t>MT5 EA development</t>
@@ -20727,7 +20607,6 @@
       </c>
     </row>
     <row r="267">
-      <c r="A267" t="inlineStr"/>
       <c r="B267" t="inlineStr">
         <is>
           <t>QuickTrade (iTrade.tools)</t>
@@ -20759,7 +20638,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
       <c r="I267" t="inlineStr">
         <is>
           <t>MT5 trading tools</t>
@@ -20833,7 +20711,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
       <c r="I268" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -20907,7 +20784,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
       <c r="I269" t="inlineStr">
         <is>
           <t>Trading platforms / MetaTrader integrations</t>
@@ -21101,7 +20977,6 @@
       </c>
     </row>
     <row r="272">
-      <c r="A272" t="inlineStr"/>
       <c r="B272" t="inlineStr">
         <is>
           <t>TRADIVO</t>
@@ -21133,7 +21008,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
       <c r="I272" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -21171,7 +21045,6 @@
       </c>
     </row>
     <row r="273">
-      <c r="A273" t="inlineStr"/>
       <c r="B273" t="inlineStr">
         <is>
           <t>6amdev (FxBoat Quant Engine)</t>
@@ -21245,7 +21118,6 @@
       </c>
     </row>
     <row r="274">
-      <c r="A274" t="inlineStr"/>
       <c r="B274" t="inlineStr">
         <is>
           <t>goodthebest (TradingView &amp; Pine Script services)</t>
@@ -21277,7 +21149,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
       <c r="I274" t="inlineStr">
         <is>
           <t>Trading automation services</t>
@@ -21429,7 +21300,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
       <c r="I276" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -21503,7 +21373,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr"/>
       <c r="I277" t="inlineStr">
         <is>
           <t>Broker technology</t>
@@ -21577,7 +21446,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr">
         <is>
           <t>MT5 indicators</t>
@@ -21651,7 +21519,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr">
         <is>
           <t>Algorithmic trading</t>
@@ -21725,7 +21592,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr"/>
       <c r="I280" t="inlineStr">
         <is>
           <t>Algorithmic trading</t>
@@ -21799,7 +21665,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H281" t="inlineStr"/>
       <c r="I281" t="inlineStr">
         <is>
           <t>Software / AI automation</t>
@@ -21951,7 +21816,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H283" t="inlineStr"/>
       <c r="I283" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -21989,7 +21853,6 @@
       </c>
     </row>
     <row r="284">
-      <c r="A284" t="inlineStr"/>
       <c r="B284" t="inlineStr">
         <is>
           <t>Contigion</t>
@@ -22021,7 +21884,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr"/>
       <c r="I284" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22059,7 +21921,6 @@
       </c>
     </row>
     <row r="285">
-      <c r="A285" t="inlineStr"/>
       <c r="B285" t="inlineStr">
         <is>
           <t>forex-mcp / mt5proxy (qicongsheng)</t>
@@ -22091,7 +21952,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H285" t="inlineStr"/>
       <c r="I285" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22129,7 +21989,6 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" t="inlineStr"/>
       <c r="B286" t="inlineStr">
         <is>
           <t>MetaTrader MCP Server (ariadng)</t>
@@ -22161,7 +22020,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr"/>
       <c r="I286" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22199,7 +22057,6 @@
       </c>
     </row>
     <row r="287">
-      <c r="A287" t="inlineStr"/>
       <c r="B287" t="inlineStr">
         <is>
           <t>mcp-mt5 (PHUICMT)</t>
@@ -22231,7 +22088,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H287" t="inlineStr"/>
       <c r="I287" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22305,7 +22161,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H288" t="inlineStr"/>
       <c r="I288" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22379,7 +22234,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H289" t="inlineStr"/>
       <c r="I289" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22495,7 +22349,6 @@
       </c>
     </row>
     <row r="291">
-      <c r="A291" t="inlineStr"/>
       <c r="B291" t="inlineStr">
         <is>
           <t>mt5-bridge (akivajp)</t>
@@ -22527,7 +22380,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H291" t="inlineStr"/>
       <c r="I291" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22601,7 +22453,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr"/>
       <c r="I292" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22675,7 +22526,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr"/>
       <c r="I293" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22749,7 +22599,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H294" t="inlineStr"/>
       <c r="I294" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22823,7 +22672,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H295" t="inlineStr"/>
       <c r="I295" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22897,7 +22745,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H296" t="inlineStr"/>
       <c r="I296" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -22971,7 +22818,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H297" t="inlineStr"/>
       <c r="I297" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23009,7 +22855,6 @@
       </c>
     </row>
     <row r="298">
-      <c r="A298" t="inlineStr"/>
       <c r="B298" t="inlineStr">
         <is>
           <t>MT5 Trading Library (paxelcool)</t>
@@ -23041,7 +22886,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23115,7 +22959,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H299" t="inlineStr"/>
       <c r="I299" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23189,7 +23032,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H300" t="inlineStr"/>
       <c r="I300" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23227,7 +23069,6 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" t="inlineStr"/>
       <c r="B301" t="inlineStr">
         <is>
           <t>Py2MQL5</t>
@@ -23259,7 +23100,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H301" t="inlineStr"/>
       <c r="I301" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23333,7 +23173,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H302" t="inlineStr"/>
       <c r="I302" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23371,7 +23210,6 @@
       </c>
     </row>
     <row r="303">
-      <c r="A303" t="inlineStr"/>
       <c r="B303" t="inlineStr">
         <is>
           <t>PythonMetaTrader5 (Akinzou)</t>
@@ -23403,7 +23241,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H303" t="inlineStr"/>
       <c r="I303" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23477,7 +23314,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H304" t="inlineStr"/>
       <c r="I304" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23593,7 +23429,6 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" t="inlineStr"/>
       <c r="B306" t="inlineStr">
         <is>
           <t>n8n-nodes-metatrader5 (BlackBull Markets)</t>
@@ -23667,7 +23502,6 @@
       </c>
     </row>
     <row r="307">
-      <c r="A307" t="inlineStr"/>
       <c r="B307" t="inlineStr">
         <is>
           <t>n8n-nodes-ohlcv-metatrader (newraal)</t>
@@ -23699,7 +23533,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H307" t="inlineStr"/>
       <c r="I307" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23737,7 +23570,6 @@
       </c>
     </row>
     <row r="308">
-      <c r="A308" t="inlineStr"/>
       <c r="B308" t="inlineStr">
         <is>
           <t>mt5cli</t>
@@ -23769,7 +23601,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H308" t="inlineStr"/>
       <c r="I308" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23843,7 +23674,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H309" t="inlineStr"/>
       <c r="I309" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -23917,7 +23747,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H310" t="inlineStr"/>
       <c r="I310" t="inlineStr">
         <is>
           <t>Market data</t>
@@ -23991,7 +23820,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H311" t="inlineStr"/>
       <c r="I311" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24065,7 +23893,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H312" t="inlineStr"/>
       <c r="I312" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24103,7 +23930,6 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" t="inlineStr"/>
       <c r="B313" t="inlineStr">
         <is>
           <t>TradeRail</t>
@@ -24135,7 +23961,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr"/>
       <c r="I313" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24173,7 +23998,6 @@
       </c>
     </row>
     <row r="314">
-      <c r="A314" t="inlineStr"/>
       <c r="B314" t="inlineStr">
         <is>
           <t>Synapse MT5</t>
@@ -24205,7 +24029,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H314" t="inlineStr"/>
       <c r="I314" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24243,7 +24066,6 @@
       </c>
     </row>
     <row r="315">
-      <c r="A315" t="inlineStr"/>
       <c r="B315" t="inlineStr">
         <is>
           <t>StrategyLab (kwasati)</t>
@@ -24275,7 +24097,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H315" t="inlineStr"/>
       <c r="I315" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24313,7 +24134,6 @@
       </c>
     </row>
     <row r="316">
-      <c r="A316" t="inlineStr"/>
       <c r="B316" t="inlineStr">
         <is>
           <t>mt5-quant forex panel</t>
@@ -24387,7 +24207,6 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" t="inlineStr"/>
       <c r="B317" t="inlineStr">
         <is>
           <t>Clawtrade</t>
@@ -24419,7 +24238,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H317" t="inlineStr"/>
       <c r="I317" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24493,7 +24311,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H318" t="inlineStr"/>
       <c r="I318" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24531,7 +24348,6 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" t="inlineStr"/>
       <c r="B319" t="inlineStr">
         <is>
           <t>mt5-analysis-mcp (0xrelogic)</t>
@@ -24563,7 +24379,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H319" t="inlineStr"/>
       <c r="I319" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24601,7 +24416,6 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" t="inlineStr"/>
       <c r="B320" t="inlineStr">
         <is>
           <t>mt5-mcp-super (herjarsa)</t>
@@ -24633,7 +24447,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H320" t="inlineStr"/>
       <c r="I320" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24671,7 +24484,6 @@
       </c>
     </row>
     <row r="321">
-      <c r="A321" t="inlineStr"/>
       <c r="B321" t="inlineStr">
         <is>
           <t>mql5-mcp (kikuchy)</t>
@@ -24703,7 +24515,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H321" t="inlineStr"/>
       <c r="I321" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24741,7 +24552,6 @@
       </c>
     </row>
     <row r="322">
-      <c r="A322" t="inlineStr"/>
       <c r="B322" t="inlineStr">
         <is>
           <t>MQL5 EA MCP Server (ductri-dev)</t>
@@ -24815,7 +24625,6 @@
       </c>
     </row>
     <row r="323">
-      <c r="A323" t="inlineStr"/>
       <c r="B323" t="inlineStr">
         <is>
           <t>IndexNano</t>
@@ -24847,7 +24656,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H323" t="inlineStr"/>
       <c r="I323" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -24921,7 +24729,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H324" t="inlineStr"/>
       <c r="I324" t="inlineStr">
         <is>
           <t>Developer tooling</t>
@@ -24959,7 +24766,6 @@
       </c>
     </row>
     <row r="325">
-      <c r="A325" t="inlineStr"/>
       <c r="B325" t="inlineStr">
         <is>
           <t>mql5-json / mql5-promise / mql5-timer (Senails)</t>
@@ -24991,7 +24797,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H325" t="inlineStr"/>
       <c r="I325" t="inlineStr">
         <is>
           <t>Developer tooling</t>
@@ -25065,7 +24870,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H326" t="inlineStr"/>
       <c r="I326" t="inlineStr">
         <is>
           <t>Developer tooling</t>
@@ -25103,7 +24907,6 @@
       </c>
     </row>
     <row r="327">
-      <c r="A327" t="inlineStr"/>
       <c r="B327" t="inlineStr">
         <is>
           <t>mql-interpreter</t>

</xml_diff>

<commit_message>
Add paid per-project note to all unsent outreach emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -6527,6 +6527,7 @@
           <t>Hi Breno,
 I read the MT5 Web Replicator README, with the Rails dashboard receiving and replicating MT5/MQL order data across accounts alongside the python-signal client, and saw that you are open to co-maintainers or partners.
 I am an MQL4/MQL5 developer who works on trade copiers and MetaTrader integrations, so the terminal side is where I could help most: the EA that reports and receives orders, symbol mapping and lot scaling between accounts, reconnect handling, and MT4 support if you ever want it. I am comfortable working inside an existing codebase and keeping changes small and documented.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still looking for someone to share the load, I would be glad to talk it through. Would it be useful if I sent over a few examples of my copier work first?
 Best regards,
 Oseni Ibrahim
@@ -6605,6 +6606,7 @@
           <t>Hi Felix,
 I came across your TradeMate showcase, the risk-first MT5 Expert Advisor with its Python monitor, six filter layers and daily loss halt. Presenting it with private source and a clear engineering write-up is a smart way to show clients what you build.
 I am an MQL4/MQL5 developer as well, focused on EAs, risk management, trade copiers and MT4 to MT5 conversion. Since you take on client projects, I thought collaboration could help both of us: I could cover MT4 versions of your EAs, take on smaller modules when your schedule is full, or handle Strategy Tester runs and VPS setup.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my work. Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -6688,6 +6690,7 @@
           <t>Hi Hưng,
 I came across ICT System EA v2.0, your MT5 Expert Advisor built on Inner Circle Trader concepts for The5%ers, with the backtest results laid out in the README.
 For prop-firm use, the pieces around the strategy often decide whether an account survives: a daily loss limit calculated exactly as the firm defines it, a pause around high-impact news, and equity checks that stop trading before the max loss is touched. I am an MQL5 developer and build these as modules that plug into an existing EA without changing entries.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are planning further versions or running the EA on more funded accounts, I would be glad to help. Would it be useful if I sent over a short example of such a module?
 Best regards,
 Oseni Ibrahim
@@ -6771,6 +6774,7 @@
           <t>Hi Jayadev,
 I came across your profile and the TradingView to MT5 webhook bridge with its queued, deduplicated order intake. I also saw that Pine-to-MQL5 ports, trade copiers and prop-firm rule logic are all part of what you deliver.
 I am an MQL4/MQL5 developer doing the same kind of work, and I wondered whether extra capacity on the MetaTrader side would ever help, for example taking a Pine-to-MQL5 port or an MT4 version of a client EA when your queue is full, delivered to your standards and under your name.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is something you would consider, I can send over a few examples of my MQL code so you can judge quality first. Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -6854,6 +6858,7 @@
           <t>Hi Noel,
 I came across TelegramSignalTrader, your EA for trading and managing accounts through Telegram, and noticed the setup guide centres on the MT4 file, TelegramSignalTrader.mq4.
 As more brokers and prop firms move clients to MT5, a maintained MQL5 version with the same Telegram commands can save you a lot of support questions. I am an MQL4/MQL5 developer and do MT4 to MT5 conversions regularly, including the parts that change the most: order handling moving to positions and deals, and WebRequest-based Telegram calls.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If an MT5 build or general maintenance of the EA would be useful to TradeAdviser, I would be glad to help. Would it be useful if I sent over a short example of a converted module?
 Best regards,
 Oseni Ibrahim
@@ -6932,6 +6937,7 @@
           <t>Hi Morteza,
 I came across tv-connector, your TradingView to MT5 bridge with HMAC-verified webhooks, a Redis queue and an MT5 EA that polls for orders. Clean design, and a good fit for traders who want something self-hosted.
 I am an MQL4/MQL5 developer and work on similar bridges, copiers and risk modules. Since you build trading systems for others, I thought there might be room to cooperate: I could write the MT4 version of your EA, add trade management features on the MQL side, or take on EA work when you have more projects than time.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my MQL code first. Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -7010,6 +7016,7 @@
           <t>Hi Pranay,
 I came across forex-mt5-strategies, your set of seven MQL5 Expert Advisors with Strategy Tester reports and design documents, including the custom oscillators built from parametric curves.
 Since you work across many venues, I thought an MQL-focused collaborator might be useful. I am an MQL4/MQL5 developer and handle the MetaTrader-specific parts that eat time: broker filling modes, stops-level checks, tester automation for multi-symbol runs, VPS deployment and MT4 versions when clients need them.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you take on client work involving MT5 EAs, I would be glad to support it. Would it be useful if I sent over a short example of my tester automation setup?
 Best regards,
 Oseni Ibrahim
@@ -7083,6 +7090,7 @@
           <t>Hi ArkoRisk team,
 I came across ArkoRisk, the open-source MT5 manager for position sizing, pending orders and prop-firm risk, with lot calculation by balance or equity percent and draggable Entry, SL and TP lines.
 Tools like this get a lot of requests once traders start using them: an MT4 edition, daily loss locks for prop accounts, partial close presets, or sizing across several positions at once. I am an MQL4/MQL5 developer who builds risk management panels and EAs, and I could help implement some of these or port the tool to MT4.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would welcome help with the backlog, I would be happy to contribute. Would it be useful if I sent over a short example of a daily loss lock module?
 Best regards,
 Oseni Ibrahim
@@ -7161,6 +7169,7 @@
           <t>Hi Sergio,
 I came across SignalReplicator and noticed that the Desktop plan only works with MT5 because the desktop expert advisor is written in MQL5, so MT4 users have to move to the Cloud plan.
 An MQL4 version of the desktop EA would let MT4 traders use the cheaper desktop option and reduce how much of your volume depends on MetaApi. I am an MQL4/MQL5 developer who works on Telegram copiers, and I could port the EA while keeping the same behaviour: multi-TP handling, break-even, trailing, partial closes and per-channel risk.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, I would be glad to help. Would it be useful if I sent over a short example of an MT4 receiver matching an MQL5 one?
 Best regards,
 Oseni Ibrahim
@@ -7239,6 +7248,7 @@
           <t>Hi FlowMetrix team,
 I came across FlowMetrix, your Windows app for managing several MT5 accounts and terminals from one dashboard with copy trading between them.
 A common request for multi-account tools is MT4 support, since many traders still hold MT4 accounts with prop firms and brokers. I am an MQL4/MQL5 developer who builds copier components, and I could write the MT4 side so those accounts appear in the same dashboard, along with symbol mapping, lot scaling rules and safeguards for partial closes and reconnects.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If widening platform support is on your list, I would be happy to help. Would it be useful if I sent over a short example of an MT4 to MT5 copy module?
 Best regards,
 Oseni Ibrahim
@@ -7312,6 +7322,7 @@
           <t>Hi ICT Library team,
 I came across ICT_Library_MQ5 and liked how it exposes SMC and ICT patterns as typed snapshots on closed candles, with the detection rules documented. Reaching over 200 stars for an MQL5 library is impressive.
 Popular libraries tend to get the same questions again and again: how to use it inside a full EA, and whether it runs on MT4. I am an MQL4/MQL5 developer and could help with both, for example a few reference EAs showing risk-managed entries built on the library, or an MQL4 port of the core detection.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would welcome a contributor or paid help for your own projects, I would be happy to talk. Would it be useful if I sent over a short example EA first?
 Best regards,
 Oseni Ibrahim
@@ -7395,6 +7406,7 @@
           <t>Hi Jason,
 I came across GGTH Predictor, where the Python side runs a five-model ensemble plus news sentiment and the MQL5 EA reads the results from shared JSON files to manage EURUSD trades.
 In setups like this, the EA usually needs the most defensive code: detecting stale or half-written prediction files, handling restarts without duplicate orders, and keeping risk limits independent of the model output. I am an MQL4/MQL5 developer and could help harden that side, extend it to more symbols, or set the whole system up on a VPS so both processes restart cleanly.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are continuing to develop GGTH, I would be glad to help. Would it be useful if I sent over a short example of a file-based signal reader?
 Best regards,
 Oseni Ibrahim
@@ -7468,6 +7480,7 @@
           <t>Hi DojiMonitorEA team,
 I came across DojiMonitorEA, the MT5 Expert Advisor that scans every Market Watch symbol for Doji candles and sends terminal or push notifications, and saw you invite people to get in touch about collaboration.
 A scanner like this is easy to grow into something traders will pay for: Telegram alerts with a chart snapshot, extra patterns such as engulfing or pin bars, multi-timeframe filters, or an MT4 edition. I am an MQL4/MQL5 developer and build scanners, alert systems and Telegram integrations for MetaTrader.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are open to developing it further, I would be glad to help. Would it be useful if I sent over a short example of a Telegram alert module in MQL5?
 Best regards,
 Oseni Ibrahim
@@ -7546,6 +7559,7 @@
           <t>Hi Chacha,
 I came across your AI Telegram Signal Copier backend, which filters Telegram messages, turns signals like 'BUY GOLD NOW SL 2330 TP 2360' into JSON with OpenAI, and hands them to an MT5 EA on Algo Forge.
 As signal channels get more varied, most of the work shifts to the EA: multiple take-profits, later edits to SL and TP, 'close half' messages, and avoiding duplicate orders after a restart. I am an MQL4/MQL5 developer who builds this kind of trade management, and I could also produce an MT4 version for users on that platform.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are taking the project further or using it for clients, I would be glad to help. Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -7629,6 +7643,7 @@
           <t>Hi Fortune,
 I came across your Triple-EA Prop-Firm Portfolio, with three MT5 EAs on US500 and USDJPY coordinated by a central PortfolioRiskManager. Sharing one risk budget across separate EAs is something most prop traders never get right.
 I am an MQL4/MQL5 developer who works on prop-firm risk management, multi-EA coordination and MT4 to MT5 ports. If you are extending the portfolio, adding firms with different daily loss definitions, or taking on clients who want something similar, I could help with the MQL side, testing across brokers, or VPS deployment.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If collaboration sounds useful, I would be glad to talk. Would it be useful if I sent over a short example of a shared-risk module?
 Best regards,
 Oseni Ibrahim
@@ -7707,6 +7722,7 @@
           <t>Hi QuantumEdgeProPlus team,
 I came across QuantumEdgeProPlus v11.0, your MT5 Expert Advisor with reinforcement learning and risk management, and saw that a professional edition is sold through Gumroad.
 Once an EA has paying users, a good share of the work becomes support: broker-specific errors, symbol suffixes, different contract sizes on gold and indices, and requests for an MT4 build. I am an MQL4/MQL5 developer and could take on part of that load, from fixing reported issues to preparing an MT4 edition and testing new versions before release.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If extra help would let you focus on the strategy itself, I would be glad to assist. Would it be useful if I sent over a few examples of my EA work?
 Best regards,
 Oseni Ibrahim
@@ -7785,6 +7801,7 @@
           <t>Hi Toki,
 I came across AI Trader for MT4, your framework that connects large language models to MetaTrader 4 with risk rules, a signal lifecycle and traceable execution.
 Since many brokers and prop firms now only offer MT5, an MQL5 bridge that speaks the same protocol as your MT4 side could widen the audience without changing the Python layer. I am an MQL4/MQL5 developer and have worked on this kind of bridge, including the MT4 to MT5 differences in order and position handling.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If adding MT5 support or hardening the MQL4 bridge is on your list, I would be glad to help. Would it be useful if I sent over a short example of an MQL5 bridge receiver?
 Best regards,
 Oseni Ibrahim
@@ -7864,6 +7881,7 @@
 I came across your Forex-Gold-Auto-Trader repository, the gold EA for MT4 and MT5 with configurable risk rules and a one-time license.
 Looking at your profile, you also take on a wide range of automation work outside trading, so keeping two MQL builds in sync, handling buyer customization requests and dealing with broker-specific issues can take a lot of time. I'm an MQL4/MQL5 developer who focuses only on MetaTrader work: EA fixes, MT4/MT5 parity, extra risk controls and Telegram notifications.
 If you ever want to pass on MQL tasks or client requests around the gold EA, I'd be happy to help as a subcontractor.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful? I can send over a few examples of my EA work.
 Best regards,
 Oseni Ibrahim
@@ -7943,6 +7961,7 @@
 I came across your GitHub profile and liked the line "Coding or Trading! Depending on the hour." I noticed you work in MQL4 and MQL5 next to your Next.js and TypeScript work at 1MF Ventures.
 When one person covers both the web stack and the trading side, MetaTrader projects often sit half-finished. I'm an MQL4/MQL5 developer who focuses only on MetaTrader: building Expert Advisors and indicators, fixing or porting MT4 code to MT5, and connecting EAs to web backends or Telegram.
 If you have a trading tool you'd like built or finished while you focus on the rest of 1MF Ventures, I'd be happy to help.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -8022,6 +8041,7 @@
 I came across your Gartal-Inc repository and the Decision Alpha Lab work, and the scale of the testing stood out: more than 9,700 documented tests with explicit quality gates.
 With that much research, the step from a validated idea to a reliable MetaTrader EA can become a bottleneck. I'm an MQL4/MQL5 developer and could help turn strategies that pass your gates into production Expert Advisors, with the same position sizing and risk rules, clean logging, and exports that match your Python analysis so live and backtest results can be compared.
 I'm also happy to build MT4 and MT5 versions of the same logic if you want both.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how I'd structure one of these EAs?
 Best regards,
 Oseni Ibrahim
@@ -8101,6 +8121,7 @@
 I came across TV2MT5 and liked the idea of charting on TradingView while the trades land in MetaTrader 5 from a local Windows machine.
 I noticed it targets MT5 only. A fair number of traders are still on MT4 accounts with their broker or prop firm, and they often ask for the same kind of copier. I'm an MQL4/MQL5 developer and could help build an MT4 receiver EA that plugs into your existing flow, or tidy up the MetaTrader side of the project, such as symbol mapping, partial closes and error handling for rejected orders.
 Happy to contribute through pull requests or as paid work, whichever suits you.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how the MT4 side could look?
 Best regards,
 Oseni Ibrahim
@@ -8180,6 +8201,7 @@
 I came across your MT5-SMC-trading-bot repository, with the Order Block, FVG and BOS modes, adaptive ATR filters and regime detection, and saw that you offer consulting to institutions.
 When an open-source EA gets attention, requests tend to follow: an MT4 version, broker-specific tweaks, extra risk rules or Telegram alerts for a particular desk. I'm an MQL4/MQL5 developer and could take on that kind of work as a subcontractor, so your consulting clients get what they need while you stay on the strategy and research side.
 An MT4 port of the SMC logic would be a natural first piece.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples of my MQL work.
 Best regards,
 Oseni Ibrahim
@@ -8264,6 +8286,7 @@
 I came across your mt5-trade-gateway repository, the order validation layer that blocks over-trading, invalid entries and trades around news events, with custom setups available on request.
 Custom setups usually mean new rule types, broker quirks and news-filter changes for each client. I'm an MQL4/MQL5 developer and could help with that side as a subcontractor, for example adding client-specific rules, building an MT4 version for traders still on MT4 accounts, or wiring alerts to Telegram when a trade is blocked.
 I'm happy to work under NDA since the code is proprietary.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples of similar risk tools.
 Best regards,
 Oseni Ibrahim
@@ -8342,6 +8365,7 @@
           <t>Hi Rafał,
 I came across your blessing-ea-optimizer repository. Optimizing all 134 Blessing EA parameters with Bayesian and genetic search on M1 tick data, then exporting .set files for MT4 and MT5, is a serious piece of work.
 You mention you're a domain expert rather than a traditional programmer, so I thought the MetaTrader side might be where some help is useful. I'm an MQL4/MQL5 developer and could, for example, automate Strategy Tester runs to validate your .set files, add logging to the EA so live results can be compared with your optimizer, or trim Blessing's logic into a cleaner EA based on what your tests show matters.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -8420,6 +8444,7 @@
           <t>Hi Simon,
 I came across the Botara 3.0 repository, with the Fisher Transform, RSI, volume oscillator and ATR logic, and saw that you mention MT4 and MT5 availability and offer custom bot development.
 Since most of the project is Python, I thought the MetaTrader builds might be where extra help is useful. I'm an MQL4/MQL5 developer and could implement or maintain the Botara logic as native Expert Advisors, keep the MT4 and MT5 versions matching your Python signals, and take on MetaTrader-specific requests from your clients as a subcontractor.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how I'd structure the EA?
 Best regards,
 Oseni Ibrahim
@@ -8494,6 +8519,7 @@
 I came across the AKG ALGO website repository and saw the range of MT4/MT5 robots you sell, from the entry license to the higher tiers, along with MQL source code access and a marketplace of EAs and indicators.
 Selling on both platforms means every robot needs two builds that behave the same way, and each MetaTrader update or broker quirk can create support work. I'm an MQL4/MQL5 developer and could help keep the MT4 and MT5 versions in sync, fix issues buyers report, add Telegram alerts or risk controls, or build new products for the marketplace.
 I'd be glad to start with one robot so you can judge the quality.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -8577,6 +8603,7 @@
           <t>Hi Mizhar,
 I came across your GitHub profile and the Forex Trading EA Scripts project, the MetaTrader 4 Expert Advisors with strategy logic, risk controls and backtesting.
 With your CTO role at Finovation Technologies and a long list of fintech and enterprise projects, I imagine the trading work gets less time than it deserves. I'm an MQL4/MQL5 developer and could help as a subcontractor: maintaining the MT4 EAs, porting them to MT5 so they run on newer broker and prop firm accounts, or handling MetaTrader requests from Finovation clients.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples of my MQL work.
 Best regards,
 Oseni Ibrahim
@@ -8660,6 +8687,7 @@
           <t>Hi Sage,
 I came across your GitHub profile and saw that you offer MetaTrader 4/5 Expert Advisor development that is spec-driven, backtested and walk-forward tested.
 That is the same kind of work I do. I'm an MQL4/MQL5 developer focused on building and fixing EAs, MT4-to-MT5 conversions, TradingView-to-MT5 ports and Telegram integrations. When client projects stack up or a job needs a second pair of hands, it can help to have someone reliable to share the load, and I'd be happy to work that way with you, either under your name or as a referral partner for jobs you can't take.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -8744,6 +8772,7 @@
 I came across your UT-Bot-Trading-System repository, with the UT Bot Alerts indicator and the UT Bot Phase EA, and noticed that most of your products, like the Multi-Symbol Trend Pullback EA and the RSI scanner, are built for MT4.
 A growing share of buyers now trade on MT5-only brokers and prop firms, so MT5 versions could open the products to more people. I'm an MQL4/MQL5 developer and could port the UT Bot tools to MQL5 while keeping the same inputs and signals, then check that both versions match in the Strategy Tester.
 I could also help when custom development requests come in faster than you can handle them.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of an MT4-to-MT5 port?
 Best regards,
 Oseni Ibrahim
@@ -8827,6 +8856,7 @@
           <t>Hi Abdiwahab,
 I came across your GitHub profile and saw that you build custom trading infrastructure for brokers, prop firms and serious traders, covering Expert Advisors, copy trading, APIs and Web3 integrations.
 Work like that often has an MQL-heavy part, such as EAs, copier endpoints inside MT4/MT5 or bridges to external APIs, that can hold up the rest of a project. I'm an MQL4/MQL5 developer focused on exactly those pieces, and I'd be glad to take them on as a subcontractor under NDA so you can stay on architecture and client work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples of my EA and bridge work.
 Best regards,
 Oseni Ibrahim
@@ -8905,6 +8935,7 @@
           <t>Hi Josias,
 I came across your profile and the Trade Pulse Technologies project, the automated forex EA platform with MT4/MT5 bots and Paystack and PayPal payments.
 A platform like this needs the MetaTrader side to be dependable: EAs that behave the same on MT4 and MT5, handle broker differences and report cleanly back to your cloud backend. Since you're also building AI, fleet and e-commerce projects, I thought extra MQL help might be useful. I'm an MQL4/MQL5 developer and could build or maintain the bots, add risk controls or Telegram notifications, and test them across brokers.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -8989,6 +9020,7 @@
 I came across your Custom-Indicators-MQL4 repository, with the RSI tools, trend validation, position sizing and correlation indicators that thousands of traders have downloaded on MQL5.com.
 They are written for MetaTrader 4, and many traders now use MT5 only, which limits who can use them on the Market. I'm an MQL4/MQL5 developer and could port your indicators to MQL5 with the same inputs, buffers and alerts, so you can publish MT5 versions alongside the originals.
 I could also take overflow work from your Fiverr or MQL5 freelance clients when you're busy.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of your indicators ported to MT5?
 Best regards,
 Oseni Ibrahim
@@ -9067,6 +9099,7 @@
           <t>Hi Vadim,
 I came across the TradingForge Terminal releases repository. Transpiling MQL4 Expert Advisors to C# so they can run on Binance Futures and other venues is an interesting approach, and I saw that MQL5 support is on the roadmap.
 MQL5 brings a different order model, handles for indicators and many small behaviour differences, so a solid set of reference EAs and test cases makes that step much easier. I'm an MQL4/MQL5 developer and could write MQL5 test EAs that cover those edge cases, compare their results in MetaTrader against your transpiled output, and help users port MQL4 strategies that don't transpile cleanly.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful? I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -9141,6 +9174,7 @@
 I came across your trading-bot-demo repository with demo versions of your Expert Advisors and indicators for MT4, MT5 and cTrader, and the full versions available for purchase.
 Selling the same tools on three platforms means every update has to be repeated and tested several times. I'm an MQL4/MQL5 developer and could take the MetaTrader side off your plate: keeping MT4 and MT5 builds in sync, fixing issues that buyers report, adding features such as Telegram alerts or extra risk settings, or building new products from your ideas.
 I'd be happy to begin with a single EA so you can see how I work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a few examples?
 Best regards,
 Oseni Ibrahim
@@ -9214,6 +9248,7 @@
           <t>Hi Helmsman Trade Manager team,
 I came across the helmsman-guide repository for Helmsman Trade Manager. A free trade panel for both MT4 and MT5, with no activation, no account limit and a 64-page user guide, is a generous piece of work.
 Keeping a panel like that working on two platforms, and answering feature requests from users, takes a lot of time. I'm an MQL4/MQL5 developer and could help maintain the MT4 and MT5 builds, fix bugs that users report, or build add-ons such as Telegram alerts or prop firm drawdown limits if you ever plan a paid edition.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples of panels and EAs I've worked on.
 Best regards,
 Oseni Ibrahim
@@ -9292,6 +9327,7 @@
           <t>Hi Viktor,
 I came across your GitHub profile and your background founding Forex Trader s.r.o. and RV-FX s.r.o., along with the custom bot architecture and MQL4/MQL5 Expert Advisor work you offer.
 When the architecture is yours, the MQL implementation, testing across brokers and MT4-to-MT5 ports can become the slow part of a project. I'm an MQL4/MQL5 developer who focuses on exactly that, and I'd be glad to act as a subcontractor under NDA, following your specifications and code standards.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short code sample first.
 Best regards,
 Oseni Ibrahim
@@ -9366,6 +9402,7 @@
 I came across your portfolio repository and the Swing Breakout V2.0 indicator you sell for TradingView through lynk.id.
 Many forex traders do their charting and execution in MetaTrader, so an MT4 or MT5 version of the indicator could reach buyers who don't use TradingView. I'm an MQL4/MQL5 developer and regularly convert Pine Script tools into MetaTrader indicators, keeping the same signals and alerts, and can also turn them into an EA if you want automated entries.
 I'd verify the MetaTrader output against your TradingView version bar by bar before handing it over.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of a Pine-to-MT5 conversion?
 Best regards,
 Oseni Ibrahim
@@ -9444,6 +9481,7 @@
           <t>Hi AlphaTRADER team,
 I noticed you publish both FuturePivots4 and FuturePivots5, along with FutureTargetsLite and AlphaRSI for MT5, plus an mt5linux setup behind your platform.
 Keeping MT4 and MT5 versions of the same indicator in step usually means every fix is done twice, and users of each platform tend to ask for alerts or an EA that trades the levels. I'm a trading bot developer who works in MQL4 and MQL5, and I could take on part of that maintenance: syncing both versions, adding alert and push notification options, or building a small EA wrapper around the pivot and target levels.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds helpful, I can send over a short example of how I would structure it.
 Best regards,
 Oseni Ibrahim
@@ -9522,6 +9560,7 @@
           <t>Hi Rodrigo,
 I came across LadinoBot, your open-source MQL5 robot, and saw it has passed 200 stars. The README's stop options (fixed, by candle and others) show how much thought went into the trade management.
 Projects like this tend to collect issues as MT5 builds and broker settings change, and forks often ask for features such as Telegram alerts or daily loss limits. I'm a trading bot developer working in MQL5, and I could help keep LadinoBot compiling cleanly on current builds, review open issues, or add a risk module if you want to extend it.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be helpful, I can send over a short example of similar maintenance work.
 Best regards,
 Oseni Ibrahim
@@ -9600,6 +9639,7 @@
           <t>Hi Moein,
 I noticed MetatraderMCP, which indexes 4,853 MQL4/MQL5 documentation entries, sitting next to PineMCP on your profile. Tooling that bridges TradingView and MetaTrader like that usually means you get requests to move strategies from one platform to the other.
 I'm a trading bot developer focused on MQL4/MQL5. Most of my work is Pine Script to MT5 conversions, MT4 to MT5 ports and EA fixes. If Fractalyst takes on client projects where the MetaTrader side is the bottleneck, I'd be happy to act as subcontract capacity, working to your specs and under your name if you prefer.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent a short sample, for example a small Pine strategy rebuilt as an MQL5 EA, so you can check the code quality first?
 Best regards,
 Oseni Ibrahim
@@ -9669,6 +9709,7 @@
 I saw your MT4 Python machine-learning trading bot deployment repo on GitHub. It's clear you're packaging MetaTrader automation for clients.
 In projects like that the Python and ML side usually goes smoothly, and the time goes into the MQL part: the bridge EA, order handling edge cases per broker, and clients who then ask for the same bot on MT5. That's where I work. I'm a trading bot developer handling MQL4/MQL5 EAs, MT4 to MT5 conversions and broker or Telegram integrations.
 If you ever need overflow capacity on the MetaTrader side, I'm happy to work white-label under your delivery process, with clear scopes and handover notes.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can also send over a few short code examples first.
 Best regards,
 Oseni Ibrahim
@@ -9748,6 +9789,7 @@
 I came across tradepostpro. It's a clever way to turn daily MT4/MT5 results into posts across X, Threads, Instagram and the other platforms. I saw that MT4 data comes in through an MQL4 EA writing CSV files, while MT5 goes through the Python API.
 Keeping those two paths consistent is usually where the small problems show up: different history fields, time zones or closed-trade detection. I'm a trading bot developer working in MQL4/MQL5, and I can write a matching MQL5 exporter EA, or tighten up the MQL4 one, so both terminals produce the same CSV format for your pipeline.
 If this is something you're working on, I can send over a short example exporter so you can check whether the output fits tradepostpro.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -9821,6 +9863,7 @@
           <t>Hi Bertin,
 I read the bbstrader README, especially the part on overcoming the MQL5 bottleneck with the C++/Python bridge to MetaTrader 5.
 Even with that approach, some users still want native pieces inside the terminal: an EA that mirrors a bbstrader strategy for the MT5 tester, custom indicators ported to MQL5, or a bridge EA for brokers where the Python API is not an option. That is the kind of MQL5 work I do as a trading bot developer.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you get requests like that from bbstrader users or clients, I could take them on as a subcontractor. Would it be useful if I sent a short example first?
 Best regards,
 Oseni Ibrahim
@@ -9894,6 +9937,7 @@
           <t>Hi Deco,
 I came across MT5 Strategy Analyzer and the feature that detects grid, scalping and other styles from a trader's history, then translates strategies between frameworks.
 When the target is MetaTrader 5, the translated strategy has to become a working MQL5 Expert Advisor, and that is where edge cases pile up: order filling modes, grid recovery logic, spread filters. I build MQL5 EAs and could help review generated code, or build the EA for your fintech clients once the analyzer has identified the strategy.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -9967,6 +10011,7 @@
           <t>Hi Umek,
 I came across QuantumBotX, the Windows-first MT5 bot and backtesting platform, and noticed the note that it is actively maintained but built in spare time.
 If the list of MetaTrader-side work is growing faster than your free hours, I could help. I build MQL5 Expert Advisors, and could write native EA versions of QuantumBotX strategies so users can run them on a VPS or in the MT5 Strategy Tester, or help with execution and deployment issues users report.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would take some load off, I can send a short example first. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -10045,6 +10090,7 @@
           <t>Hi Raphael,
 I came across your GitHub profile and Trady.chat, the trading assistant with a psychological focus, and saw that MQL5 Expert Advisors sit in your stack next to n8n, WebSockets and the OpenAI API.
 An assistant like that becomes much more useful when it can see what the trader actually did. I'm a MetaTrader developer and could build a small MT5 EA that streams positions, closed trades and account equity to Trady.chat over WebSockets or HTTP, so the assistant can comment on real behaviour such as revenge trading or oversizing, without asking users to log trades by hand.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, would it be useful if I sent over a short example of the MT5 side?
 Best regards,
 Oseni Ibrahim
@@ -10118,6 +10164,7 @@
           <t>Hi ByTamerFX team,
 I came across the ByTamerFX Pro showcase and read through the changelog. The pace of EA releases is impressive, and I noticed one entry where the server EA had stopped writing to the bytamer.com MT5 state endpoint until the URL was forced at init.
 I'm an MQL4/MQL5 developer, and links like that between an EA, a web API, a desktop terminal and a mobile app are the kind of plumbing I work on regularly: heartbeat checks, retry and queueing when the endpoint is unreachable, and alerts when data goes stale. If extra MQL5 capacity would help, whether for that layer, regression testing between releases or new EA modules, I would be glad to support your work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of a heartbeat and retry pattern?
 Best regards,
 Oseni Ibrahim
@@ -10191,6 +10238,7 @@
           <t>Hi Lachlan,
 I came across MicroQuant and liked the 'Micro Quant' idea behind it: a repeatable logic stack that pulls MT5 OHLC into PostgreSQL and adds AI, technical and news context before any decision is made.
 I'm an MQL4/MQL5 developer. If you're planning to let MicroQuant act on its trade plans, a small MQL5 EA is a reliable way to do it: it can read approved decisions from your WebSocket or database, apply position sizing and hard stops inside the terminal, and report fills back. I could build that and help with a stable VPS setup for the MT5 side, keeping to your existing stack.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that decision-to-EA handoff?
 Best regards,
 Oseni Ibrahim
@@ -10259,6 +10307,7 @@
           <t>Hi Nodalytics team,
 I came across nodalytics/metatrader-terminal and liked how clearly the README explains the reverse SSH tunnel and the WebSocket stream that pushes only the differences, since MT5 has no push API of its own.
 I'm an MQL4/MQL5 developer working on the MetaTrader side of setups like this: EAs and services that feed an external API, execution and risk modules, and keeping terminal bridges stable across builds and broker changes. If your team ever needs extra hands on the MT5 layer, such as an EA-side event publisher to complement the polling loop or help maintaining the container as you add accounts, I could take that on as a contractor.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is useful, I can send over a short example of an MQL5 event publisher.
 Best regards,
 Oseni Ibrahim
@@ -10327,6 +10376,7 @@
           <t>Hi Trade Vectors team,
 I came across your trading-strategy-templates-python repo and noticed that alongside the NSE/BSE and IBKR work, Trade Vectors lists MetaTrader broker integration and an MQL5 + Python bridge for MT5 forex and CFD clients.
 I'm a trading bot developer specialising in MQL4/MQL5. Agencies covering many markets sometimes prefer to hand the MetaTrader-specific parts to someone who works in MQL every day, so I wanted to offer myself as white-label capacity: Expert Advisors built from client specs, MQL5 sides of Python bridges, MT4 to MT5 conversions and fixes to existing EAs. You would keep the client relationship and I would deliver documented source code.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you'd consider, I can send over a few examples of recent MQL5 work.
 Best regards,
 Oseni Ibrahim
@@ -10400,6 +10450,7 @@
           <t>Hi Kipli team,
 I came across ProChart XAUUSD on GitHub, the FastAPI and MT5 chart app that alerts when gold nears Fibonacci entry areas, and saw that you offer custom versions, broker integrations and dashboards.
 Custom client requests like that often need work inside MetaTrader: an EA that places the trade when a Fibonacci zone triggers, a lighter MQL5 data feed instead of the Python MT5 package, or MT4 support for clients on older brokers. I'm a trading bot developer working in MQL4/MQL5, and I could take on that MetaTrader side for your custom projects.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can share examples first.
 Best regards,
 Oseni Ibrahim
@@ -10468,6 +10519,7 @@
           <t>Hi Copiix team,
 I came across the Copiix GitHub organization and saw that the copier handles MT4, MT5 and cTrader in any combination, free and without registration. Keeping MT4 and MT5 EAs in step across terminal updates and broker symbol differences is steady work, especially when every user is on a different setup.
 I'm an MQL4/MQL5 developer and could take on part of that load: fixing edge cases reported by users, adding features such as symbol mapping or lot rules, or reviewing the copier EAs for stability on both platforms. I work async and can start on a single small ticket so you can judge the fit.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of similar copier work?
 Best regards,
 Oseni Ibrahim
@@ -10541,6 +10593,7 @@
           <t>Hi Fintechee team,
 I noticed in the FiSDK README that Fintechee.io lets vendors sell C/C++/MQL-based EAs and indicators, and that Expert-Advisor-Studio runs EAs directly in the browser. That mix usually means someone has to translate MetaTrader logic into your runtime, or the other way around, for customers and white-label partners.
 I build and convert MT4/MT5 Expert Advisors and indicators, and I could help with ports from MQL4/MQL5 into your EA format, or with MetaTrader versions of strategies built in your studio. I can also handle smaller jobs such as indicator rewrites for your marketplace sellers.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -10609,6 +10662,7 @@
           <t>Hi Fivitech team,
 I came across fivitech-mt5-connector on PyPI, with its MT5Pool for connecting to and managing several MetaTrader 5 servers through manager and API credentials. That suggests you work close to brokers running their own MT5 infrastructure.
 Those clients often need terminal-side pieces too: expert advisors, custom indicators, equity-protection or risk tools for traders, or MT4-to-MT5 conversions of legacy code. I'm an MQL4/MQL5 developer and could act as extra capacity for that part of your projects, working to your specs and handing over clean, documented source.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you ever have MQL work queued up behind the server-side tasks, would you be open to me sending a few relevant examples?
 Best regards,
 Oseni Ibrahim
@@ -10677,6 +10731,7 @@
           <t>Hi MetaRPC team,
 I saw that you publish MetaRpcMT4 and MetaRpcMT5, gRPC Python clients for MetaTrader, and that both got fresh releases this week. Supporting two terminal generations in parallel is no small job.
 I'm an MQL4/MQL5 developer. For a gateway like yours, I could help with reference strategies built on your SDK for the documentation, test EAs that check order and position behaviour against the gRPC results, or porting client-side tools between MT4 and MT5. I'm happy to work as outside capacity under your specs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a couple of examples of related MetaTrader integration work.
 Best regards,
 Oseni Ibrahim
@@ -10745,6 +10800,7 @@
           <t>Hi LuxAlgo team,
 I came across @luxalgo/journal-importers on npm and saw that the new trade journal can import MetaTrader HTML statements. That tells me a good part of your users trade on MT4 and MT5.
 Statement imports are manual by nature. I'm an MQL4/MQL5 developer and could build a small MetaTrader EA that sends closed trades to the journal automatically, including screenshots, magic numbers and comments, so MT users get the same experience as API-connected brokers. I also port TradingView-style tools to MQL5 if that ever comes up.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the sync EA?
 Best regards,
 Oseni Ibrahim
@@ -10823,6 +10879,7 @@
           <t>Hi Simon,
 I came across the mt5-mcp-server package on npm, published under the afx-markets GitHub organisation, which gives AI assistants access to MetaTrader 5 symbol and trading data.
 If it's heading toward client-facing use, some features are easier from inside the terminal. Examples are an EA that enforces account-level risk rules whatever the assistant requests, streaming of trade events, or exporting custom indicator values. I'm an MQL4/MQL5 developer and could build those pieces or support the MetaTrader side generally, working to your specs and handing over documented source.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example?
 Best regards,
 Oseni Ibrahim
@@ -10896,6 +10953,7 @@
           <t>Hi FxSocket team,
 I came across the @fxsocket/sdk package, your typed Node.js client for MT4 and MT5 account management, trading and streaming, with automatic reconnect and subscription replay.
 API customers often come back with needs the API doesn't cover: a custom EA running beside their integration, indicator values the platform doesn't expose, or MT4 code that has to move to MT5. I'm an MQL4/MQL5 developer and could be the partner you point those requests to, or write example EAs that show FxSocket and in-terminal code working together.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's useful, I can send over a few examples of my work.
 Best regards,
 Oseni Ibrahim
@@ -10964,6 +11022,7 @@
           <t>Hi XBTFX team,
 I came across @xbtfx/mcp-trading, the MCP server that lets Claude, Codex and Cursor trade XBTFX MetaTrader 5 accounts through your Trading API.
 Traders coming in through AI agents often still want something running in the terminal itself. That could be an EA that enforces their own risk limits, trade management that runs while the agent is offline, or indicators that show what the agent did on the chart. I'm an MQL4/MQL5 developer and could build such tools for your clients or example EAs for the API documentation.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds relevant, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -11032,6 +11091,7 @@
           <t>Hi Yuants team,
 I came across @yuants/vendor-mt4 on npm, the MetaTrader 4 connector for the Yuants trading system.
 MT4 connectors usually depend on an MQL4 bridge running in the terminal, and many brokers now only open new accounts on MT5. I'm an MQL4/MQL5 developer and could help maintain the MT4 bridge side or build an MT5 equivalent with the same message format, so a vendor-mt5 package would need few changes in your TypeScript code. The EA would handle reconnection and report account state regularly.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's on your list, I can send over a short example of an MT5 bridge EA.
 Best regards,
 Oseni Ibrahim
@@ -11100,6 +11160,7 @@
           <t>Hi OrvaLabs team,
 I noticed orva-mt5-bridge, the MQL5 bridge that pushes MetaTrader 5 market data over HTTP and TCP into the Orva platform.
 Bridges like this usually work well in testing and then meet dropped connections, terminal restarts and brokers with odd symbol names once they run all day. I'm a trading bot developer working in MQL5, and I could help with reconnect and buffering logic, symbol mapping, or adding order execution endpoints so the AI side can act on its signals through the same bridge.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how I would handle reconnects in MQL5?
 Best regards,
 Oseni Ibrahim
@@ -11173,6 +11234,7 @@
           <t>Hi Cesar,
 I came across mql5-execution-components and your Castle Trade LLC profile, including the asynchronous execution framework work.
 Since you take contract work through Upwork, I thought it worth reaching out. I'm a trading bot developer working in MQL4/MQL5, mainly on EA fixes, MT4 to MT5 conversion, Telegram integration and trade copiers. When client work on the MetaTrader side piles up, I could take on defined pieces such as ports, broker compatibility fixes or testing harnesses so you can stay focused on the architecture.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of my MQL5 code?
 Best regards,
 Oseni Ibrahim
@@ -11251,6 +11313,7 @@
           <t>Hi Hossein,
 I came across WealthPole-Architecture-Demo, the modular MQL5 EA starter from Fintor AI, and the trend and risk engines you describe on your profile.
 Modular EA designs pay off, but every new engine still needs its inputs, tests and broker edge cases handled. I'm a trading bot developer working in MQL4/MQL5, and I could help build or test specific modules, for example the daily drawdown guard, exposure control, or a Telegram reporting layer, following the structure and naming you've already set up in the demo.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -11324,6 +11387,7 @@
           <t>Hi Sergei,
 I came across FinCore and XTradeServer, and noticed the README invites people to write about improvements, installation and support for a secured version.
 Both projects lean on MetaTrader 5 connectivity, and that part tends to need attention as MT5 builds and brokers change. I'm a trading bot developer working in MQL4/MQL5, and I could help on the MetaTrader side: the EA or script that reports deals and positions into FinCore, terminal management for XTradeServer, or updating older MQL code so it compiles cleanly on current builds.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example of similar work.
 Best regards,
 Oseni Ibrahim
@@ -11397,6 +11461,7 @@
           <t>Hi Pedro,
 I came across horizon5-mt, your MetaTrader framework with portfolio optimization, and it looks like a serious piece of engineering rather than a one-off EA.
 Frameworks like this usually reach a point where the core is solid but there's a backlog of strategy modules, reporting and small integrations to add. I'm a trading bot developer working in MQL4/MQL5, and I could help with that backlog, for example writing new strategy components against your interfaces, adding Telegram notifications for fills and drawdown, or building backtest export scripts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of similar work?
 Best regards,
 Oseni Ibrahim
@@ -11475,6 +11540,7 @@
           <t>Hi Nawfal,
 I came across mq5_skills, your AI skill for producing production-ready MT5 Expert Advisors, and the MT_MANAGER account tool alongside it.
 The quality of generated EAs depends heavily on the examples and rules the skill draws on, especially around order filling modes, stop levels and error handling that trip up new EAs. I'm a trading bot developer who writes MQL4/MQL5 daily, and I could contribute reviewed reference EAs and checklists, or help extend MT_MANAGER with risk limits and alerts. Everything would be written to match your conventions.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -11553,6 +11619,7 @@
           <t>Hi Ali,
 I came across metatrader-mcp and the Phoenix platform on your profile, the 21-service automated trading setup that includes MQL5 components.
 In platforms like that, the MetaTrader piece is often the one that needs the most care: terminals that disconnect, symbols that differ by broker, and EAs that must report state back cleanly. I'm a trading bot developer working in MQL4/MQL5, and I could help with the MT5 side, for example extending metatrader-mcp with order and position endpoints or hardening the EA that feeds Phoenix so it recovers cleanly after terminal restarts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -11631,6 +11698,7 @@
           <t>Hi Hemang,
 I came across Algotrading_Multi_account_Modern_UI, the web control panel for running trades across multiple accounts, and noticed it's tagged for MQL5.
 Multi-account tools get much more useful when MetaTrader 5 accounts can be driven the same way as the others, which usually means a small EA or bridge on each terminal that accepts commands and reports positions back. I'm a trading bot developer working in MQL4/MQL5, and I could build that connector, including reconnect handling, per-account risk limits and a simple status report your UI can display.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short outline of how I'd approach it?
 Best regards,
 Oseni Ibrahim
@@ -11709,6 +11777,7 @@
           <t>Hi Max,
 I came across mt5-device-fingerprint-tool and the MT-Indicator-Locker projects, which generate SHA-256 license codes to protect MT5 indicators.
 Vendors who try tools like these usually need help on the MQL5 side: wiring the license check into an existing EA or indicator without breaking it, handling offline cases and giving clear messages when a key fails. I'm a trading bot developer working in MQL4/MQL5, and I could write ready-to-use MQL5 include files and example integrations to sit alongside your tools, so vendors can adopt them in an afternoon rather than a week.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -11782,6 +11851,7 @@
           <t>Hi Tibor,
 I came across TradeForge, your Python framework for MetaTrader 5 with the live engine, Optuna optimisation and Telegram control.
 Python-driven MT5 setups often benefit from a small MQL5 companion running in the terminal, one that draws signals and levels on the chart and acts as a last safety check on order size and daily loss if the Python side misbehaves. I'm a trading bot developer working in MQL4/MQL5, and I could build that companion to fit TradeForge's config format and read the same parameters your optimiser produces.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -11850,6 +11920,7 @@
           <t>Hi Daedalus team,
 I came across your MetaTrader tools, advance-trade-management, GriffinATM and Lynxguard, the checker that compares tick data across brokers.
 Trade managers get a steady stream of requests once people use them: partial closes, basket breakeven, prop-firm daily limits, and fixes when a broker uses unusual stop levels. I'm a trading bot developer working in MQL4/MQL5, and I could help with those additions or with an MT4 version if your users ask for one. I'm used to working inside someone else's code without changing its style.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples of trade management code I've written.
 Best regards,
 Oseni Ibrahim
@@ -11923,6 +11994,7 @@
           <t>Hi Joao Pedro,
 I came across Connexus, your MQL5 HTTP library, and Logify for logging. Both solve problems I run into on almost every EA project.
 The most common things people build on top of an HTTP library in MQL5 are Telegram notifications, TradingView webhook receivers and small REST dashboards. I'm a trading bot developer working in MQL4/MQL5, and I'd be glad to contribute worked examples of those using Connexus, or help with client projects that need this kind of integration if you take on freelance work and want a hand with the MetaTrader side.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12001,6 +12073,7 @@
           <t>Hi Artem,
 I came across mt5-cloud-level-alerts, the service that syncs MT5 chart levels to the cloud and sends Telegram alerts.
 The MetaTrader client is usually the tricky part of a tool like this: catching every object change, surviving terminal restarts and WebRequest limits, and supporting MT4 users who ask for the same thing. I'm a trading bot developer working in MQL4/MQL5, and I could help with that client side, including an MT4 port, so you can keep your focus on the service and front end. I'd document the client so it is easy to maintain later.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -12074,6 +12147,7 @@
           <t>Hi LoanXfer team,
 I came across mt5-risk-reward-tool and mt5-economic-calendar, and saw on your profile that you take freelance work on trading bots and exchange backends.
 Clients who start on exchange bots often come back asking for the same logic in MetaTrader, and MQL has enough quirks that it can eat time. I'm a trading bot developer focused on MQL4/MQL5, and I could take on the MetaTrader pieces of your projects, such as EAs, trade copiers or TradingView to MT5 bridges, while you handle the backend work. I can work under your name and hand over documented source.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -12147,6 +12221,7 @@
           <t>Hi Sebastian,
 I came across your MT5 tools, especially mt5-panel-maestro with the kill switch and mt5-telegram-assistant for drawdown alerts.
 We seem to work on very similar things. I'm a trading bot developer working in MQL4/MQL5, mostly on EA fixes, Telegram integration, trade copiers and risk management. Freelance demand is rarely even, so I'm reaching out to suggest sharing overflow work: if you have a client project that needs an extra pair of hands, or an MT4 version of one of your tools, I could help, and I'd be glad to send work your way too.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -12220,6 +12295,7 @@
           <t>Hi Dewyndl team,
 I came across metatrader-automation-scripts-toolkit, with the trailing stop and grid EAs, and saw from your profile that you offer backend and integration services to clients in Europe and the CIS.
 When clients ask for MetaTrader work it is often more than a script: a full EA, a copier between accounts, or a bridge from TradingView. I'm a trading bot developer focused on MQL4/MQL5, and I could handle that side of your projects as a subcontractor while you keep the backend and API work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of my MQL5 code?
 Best regards,
 Oseni Ibrahim
@@ -12293,6 +12369,7 @@
           <t>Hi Khaleq,
 I came across your ICT_indicator repository and liked the closed-bar-only rule, where signals are only finalised after right-side confirmation. That is the part many SMC tools get wrong.
 Indicators with that much logic usually lead users to ask for two things: alerts they can trust and an EA that trades the signals with proper risk controls. I'm a trading bot developer working in MQL4/MQL5, and I could build an EA wrapper that reads the indicator buffers, adds position sizing and daily loss limits, and sends Telegram alerts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12366,6 +12443,7 @@
           <t>Hi Ali,
 I came across your MQL5 Programming for Traders course repository, the introduction to building trading robots and Expert Advisors in MQL5.
 Students of courses like this usually get stuck at the step after the basics: adding real risk management, sending alerts to Telegram, or converting an old MT4 indicator they already use. I'm a trading bot developer working in MQL4/MQL5, and I could prepare a few worked example EAs on those topics, or review student code if you run cohorts, to sit alongside your lessons.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful? I can send over a sample first.
 Best regards,
 Oseni Ibrahim
@@ -12439,6 +12517,7 @@
           <t>Hi Handiko,
 I came across Trading-Strategy-Development-Example and Improvement-to-an-existing-strategy, and liked how you walk through improving a strategy step by step instead of just posting final code.
 I'm a trading bot developer working in MQL4/MQL5, and your approach is close to how I handle client work. If you take on strategy projects or want help turning research into production EAs with proper risk handling, Telegram alerts and VPS deployment, I could help as a collaborator or subcontractor on the MetaTrader side.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of my code first.
 Best regards,
 Oseni Ibrahim
@@ -12517,6 +12596,7 @@
           <t>Hi Saymon,
 I came across mcp-metaeditor, your MCP server that runs MetaTrader 5's MetaEditor under Linux and Wine. Compiling MQL5 from outside Windows is something a lot of developers want.
 Tools like this get tested hardest on messy real projects: many include files, resources, DLL imports and strategy tester runs. I'm a trading bot developer working in MQL4/MQL5, and I could put mcp-metaeditor through its paces on real multi-file EAs, report where it breaks, and contribute test fixtures, or help your users with EA work if they ask.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example project to start with.
 Best regards,
 Oseni Ibrahim
@@ -12585,6 +12665,7 @@
           <t>Hi AtingMQL5 team,
 I came across AtingMQL5 and liked the automatic filling mode selection, since the wrong filling mode is one of the most common reasons an EA fails on a new broker.
 Libraries like this spread faster when there are complete example EAs showing the classes working together. I'm a trading bot developer working in MQL4/MQL5, and I could contribute a couple of example EAs built on AtingMQL5, for instance a session breakout using LimitsByTimeRange with CSV-filtered backtests, or help on bot projects if you take client work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -12658,6 +12739,7 @@
           <t>Hi Desmond,
 I came across MT5-EA-Project and saw in the README that you welcome collaboration on the collection, including the Power-Pivot strategy.
 Collections of EAs tend to grow uneven over time, with each one handling lot sizing, trailing and alerts a little differently. I'm a trading bot developer working in MQL4/MQL5, and I could help bring them onto a shared risk and notification module, add Telegram alerts, or write MT4 versions of the ones people ask for. I'd keep each strategy's logic untouched and only standardise the shared parts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -12731,6 +12813,7 @@
           <t>Hi Sajid,
 I came across grid-master-pro-mt5-ea and noticed it has picked up well over a hundred stars, which usually means plenty of people running it on different brokers.
 Grid EAs draw the most requests for protective features: equity stop, maximum open levels, news pauses and prop-firm daily loss rules. I'm a trading bot developer working in MQL4/MQL5, and I could help add those safeguards or handle broker compatibility issues users report, so the project keeps moving while you work on AlHarih's other products and client work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -12804,6 +12887,7 @@
           <t>Hi Duc Duy,
 I came across Algo-Trading-Lab, with the reinforcement learning agents (PPO, SAC, TD3 and others) alongside the indicator-based strategies.
 The step from a trained agent to live trading in MetaTrader is often where projects stall, because it needs a dependable bridge, order validation and account-level limits. I'm a trading bot developer working in MQL4/MQL5, and I could build the MT5 side: an EA that receives the model's actions, checks them against risk rules and reports fills back to Python, so live results can be compared fairly with your backtests.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12877,6 +12961,7 @@
           <t>Hi Joe,
 I came across MQL5-Bots, with the MACD and RSI strategies, and noticed your TrendBot work on Deriv's Volatility Index.
 Deriv's synthetic indices on MT5 have their own quirks, including large minimum lots, 24/7 sessions and fast spikes, so EAs written for forex often need changes to behave there. I'm a trading bot developer working in MQL4/MQL5, and I could help adapt the bots for synthetics with suitable sizing and a Telegram alert layer, or collaborate on client bots if you take that kind of work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12950,6 +13035,7 @@
           <t>Hi BigHeroAI team,
 I came across bigheroai-showcase and the BigHeroAI decision system for MetaTrader 5, along with your ICT/SMC Pine indicators.
 Two things usually follow a setup like this: the MQL5 bridge needs to survive disconnects and report state reliably, and users of the Pine indicators ask for MT5 versions. I'm a trading bot developer working in MQL4/MQL5, and I could help with either, hardening the bridge EA or converting the confirmed-bar ICT/SMC indicators to MQL5 with signals that match the TradingView versions bar for bar.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13018,6 +13104,7 @@
           <t>Hi Ishaan,
 I came across mt5-mac-python-bridge. Getting Python to drive MetaTrader 5 on a Mac is something I see traders struggle with often.
 Once the data side works, people usually want to place and manage orders through the same bridge and to know when the terminal has gone quiet. I'm a trading bot developer working in MQL4/MQL5, and I could build an MQL5 EA counterpart that executes orders with proper error codes, enforces basic risk limits and sends a regular heartbeat back to Python.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13096,6 +13183,7 @@
           <t>Hi Leeank,
 I came across Algorithmic-Trading-Bot, the Python bot you run on MetaTrader 5, and saw you're working on Inversiones Bloom.
 Python bots on MT5 usually hit the same practical issues in live use: the terminal disconnects, orders are rejected for broker-specific reasons, and nobody notices until the next morning. I'm a trading bot developer working in MQL4/MQL5, and I could add an MQL5 safety and monitoring layer with Telegram alerts, or help set up a stable VPS deployment for the bot.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -13169,6 +13257,7 @@
           <t>Hi Gilbran,
 I came across mt5-signal-copier-architecture, your Telegram to MT5 copier, and saw on your profile that it runs unattended with your other production services.
 Copiers like this tend to break on the execution side rather than the parsing side: signal edits that should move a stop, multiple take profits, duplicate messages and symbol suffixes that differ by broker. I'm a trading bot developer working in MQL4/MQL5, and I could help harden the MT5 EA for those cases and add a heartbeat so you know it is still trading.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13242,6 +13331,7 @@
           <t>Hi Ahmed,
 I came across forex-news-killer, your MT4 EA that protects accounts around news events.
 Since most brokers and prop firms have moved to MT5, I'd expect people in your Discord and YouTube audience to ask for an MT5 version. MQL5 also has a built-in economic calendar, which removes the need for outside news feeds. I'm a trading bot developer working in MQL4/MQL5, and I could convert the EA to MT5 using that calendar while keeping your existing inputs and behaviour, so current users can switch without relearning the settings.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13316,6 +13406,7 @@
 I came across pixiu, a Python backtesting tool built around MetaTrader 4 and 5. It's useful for people who don't want to live inside the Strategy Tester.
 A common question from MetaTrader users is whether a strategy backtested outside MT4/MT5 matches what their EA does in the terminal. I'm a trading bot developer working in MQL4/MQL5, and I could write reference EAs that mirror a few pixiu strategies. You could then compare fills, spreads and results against the MT4/MT5 tester and document any differences.
 If this is something you're working on, I can send over a short example, one simple strategy as both a pixiu script and an MQL5 EA, so you can judge whether it's worth doing more.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13390,6 +13481,7 @@
 I came across ubot-mt4, your MetaTrader 4 Expert Advisor. It stood out because of your backend and ML background, which shows in how the bot is laid out.
 Many traders now only get MT5 accounts from brokers and prop firms, so MT4-only EAs are harder to use. I'm a trading bot developer who does MT4 to MT5 conversions: rewriting order logic for MT5 positions and deals, checking indicator handles and validating both versions side by side in the Strategy Tester. I can also add Telegram trade notifications or a drawdown guard if that's useful.
 If you'd like, I can port a small part of ubot-mt4 to MQL5 and send it over as an example.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -13469,6 +13561,7 @@
 I came across your MT4 Manager REST API in ASP.NET Core. Exposing Manager functions over REST is exactly what broker back offices and CRMs ask for.
 Clients who start on MT4 usually ask for the same thing on MT5 soon after, along with terminal-side pieces such as EAs for reporting, risk checks or trade copying that the API alone can't cover. I'm a trading bot developer working in MQL4/MQL5 and MetaTrader integrations. If your .NET work brings in broker projects, I'd be glad to cover the MQL and MT5 parts as a collaborator.
 If this sounds relevant, I can send over a couple of short examples of EA-side components that would sit next to your API.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -13548,6 +13641,7 @@
 I came across your Automatic Setter Expert Advisor for MT4, which deploys up to 150 strategy instances per session. That saves a lot of time for anyone running strategy portfolios, for example from StrategyQuant-style generators.
 The same need exists on MT5, but charts, templates and EA inputs are handled differently there, so the MT4 tool can't just be recompiled. I'm a trading bot developer who works on MT4 to MT5 conversions and deployment tooling. I could build an MQL5 version with the same batch workflow.
 If that sounds interesting, I can send over a short example showing how the attach-and-configure step works on MT5.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -13627,6 +13721,7 @@
 I came across MetatraderSharp and the cookbook. A cleaner C# wrapper around MTsocketAPI for both MT4 and MT5 is useful for .NET developers who don't want to write MQL.
 Sooner or later, library users hit the terminal side: behaviour that differs between MT4 and MT5 accounts, custom indicators they want to read, or small EAs to run alongside the socket connection. I'm a trading bot developer working in MQL4/MQL5 and MetaTrader integrations, and I'd be happy to contribute cookbook examples or help with MQL work around the library.
 If this fits where you're taking the project, I can send over a short example of an MQL5 helper that exposes custom indicator values to a C# client.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13706,6 +13801,7 @@
 I came across AlgoExpertHub and saw that forex execution for MT4/MT5 goes through MetaApi and mtapi.io. That works well for getting started, but per-account cloud fees and an extra dependency tend to add up as subscribers grow.
 One option is a native MQL4/MQL5 receiver EA that polls or listens to your Laravel API and places trades directly in the subscriber's terminal, with lot sizing, symbol mapping and a daily loss limit. I'm a trading bot developer who builds signal executors, trade copiers and Telegram integrations for MetaTrader.
 If this is something you're working on, I can send over a short example of a receiver EA that reads signals from a JSON endpoint.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13780,6 +13876,7 @@
 I came across MT4ForexParser, which turns MetaTrader 4 .hst history into CSV and pandas. It fits nicely with PriceGenerator for strategy testing.
 Most brokers are moving users to MT5, where history is stored differently and is best exported from inside the terminal. I'm a trading bot developer working in MQL4/MQL5. I could write an MQL5 script or EA that exports bars and ticks in the same CSV layout your parser produces, so MT5 data drops straight into your existing pipeline.
 If that would help, I can send over a short example exporter so you can compare its output with an MT4ForexParser file.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13854,6 +13951,7 @@
 I came across MT4 Position Helper (MT4持仓助手). It looks like you support a real user group through QQ and keep the EA updated.
 As more brokers move clients to MT5, position-management tools like yours are often among the first things traders ask for on the new platform. The MT5 position and order model is different, so a direct recompile doesn't work. I'm a trading bot developer who does MT4 to MT5 conversions, and I could port the helper to MQL5 while keeping the same panel and behaviour your users already know.
 If you're interested, I can send over a short example of one feature, such as batch close or breakeven, running in MQL5.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13927,6 +14025,7 @@
           <t>Hi Gifari,
 I came across XAUBot AI and liked how the XGBoost model, SMC features and HMM regime detection are combined for XAUUSD on MetaTrader 5. I also saw SURGE-WSI following a similar path.
 Since the logic lives in Python, the terminal only acts on what the bridge sends. I build MQL5 Expert Advisors, and a small companion EA could keep the daily loss limit, session filter and trailing or breakeven rules running inside MT5 even if the Python side disconnects or restarts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits where the project is heading, I can send over a short example of how I usually structure that kind of guard EA. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -14005,6 +14104,7 @@
           <t>Hi Omega,
 I saw StrategyTester5 and the strategytester5.com docs. Bringing a proper backtesting layer to the MetaTrader 5 Python API is something a lot of Python traders have been missing.
 One thing that usually comes up with a tool like this is people wanting ST5 results to line up with the native MT5 Strategy Tester. I work on MQL5 Expert Advisors, and I could write mirror EAs for your example strategies so users can compare fills, order handling and report numbers side by side. I also take on overflow MQL5 work if clients ask you for EA versions of their Python strategies.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent over a small example of such a comparison EA?
 Best regards,
 Oseni Ibrahim
@@ -14083,6 +14183,7 @@
           <t>Hi José,
 I came across mt5-docker-api and your public trade journal at jose.ar. Running MT5 in Docker with VNC and a REST layer, then publishing 5,600+ trades openly, is a solid engineering setup.
 I build MQL5 Expert Advisors, and I thought there might be room for an in-terminal piece next to the container: an EA that handles execution checks, writes trade events in a format your journal can ingest, or enforces risk limits locally when the API is not reachable.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of that overlaps with what you are building next, I can send a short example of how I would structure it. Would you be open to that?
 Best regards,
 Oseni Ibrahim
@@ -14161,6 +14262,7 @@
           <t>Hi Bechara,
 I saw Claude Trader, with its 14 agents covering strategy, entries, capital management and position watching on MetaTrader 5, and TradeAI Gold on your profile.
 With agents deciding trades, it often helps to have a deterministic layer inside the terminal that does not depend on the API session. I develop MQL5 Expert Advisors and could build a compact guard EA that enforces max exposure, daily drawdown and hard stops, and reports state back to your system.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is on your list for the gold bot or client projects, I can send over a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -14239,6 +14341,7 @@
           <t>Hi Fredy,
 I came across mt5-arch-integration and the note that mt5linux/RPyC often hits IPC timeouts under Wine 11, which is why you went with the Mt5ArchBridge.mq5 file bridge.
 That EA ends up carrying the whole integration, so small things like command acknowledgements, retry handling and file locking make a big difference. I write MQL5 Expert Advisors and bridges, and could help extend the bridge with more order types and status reporting, or try a socket-based variant that still behaves under Wine.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are planning more work on it, I can send a short example of how I handle the file protocol side. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -14317,6 +14420,7 @@
           <t>Hi Elkhan,
 I saw ForexAiTrader and liked the principle that Claude proposes and the deterministic risk engine disposes. Routing execution through MetaApi keeps the Node side clean.
 One gap in cloud setups is that the terminal itself does not know the risk rules. I build MQL5 Expert Advisors and could write a small EA that enforces the same hard limits (max lots, daily loss, max open trades) inside MT5, so they hold even if the API link drops. A direct EA bridge is another option if you want to reduce dependence on the cloud service.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent a short example?
 Best regards,
 Oseni Ibrahim
@@ -14395,6 +14499,7 @@
           <t>Hi Amir,
 I came across TradingAgents, with the AI analyst team, the 25-strategy engine and MT5 streaming in one desktop app, and I saw you are also building Traders Royal.
 For a product like this, the MetaTrader side often decides how it feels: tick delivery, order confirmation and how the app recovers after a terminal restart. I build MQL5 Expert Advisors and bridges, and could write an EA that pushes ticks and account events to the app and handles execution requests with proper checks.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -14468,6 +14573,7 @@
           <t>Hi Prabal,
 I saw TradeLens and liked the idea of a calm, read-only companion that shows the risk story of an MT5 trade before the click.
 A natural extension could be an MQL5 panel or indicator that draws the same numbers on the chart itself: risk in money, margin after entry, stop distance compared with ATR. That way traders see it right where they place the order. I build MQL5 indicators and Expert Advisors and could put together that chart-side piece so it reads from the same assumptions.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is interesting, I can send over a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -14546,6 +14652,7 @@
           <t>Hi Kelvin,
 I saw your Deriv MT5 synthetic indices bot. The rules are clearly defined: 4H trend from fractal swings, the 4H order block, a 15M fair value gap entry and a structural target that must clear 1:3.
 Because the rules are so precise, they translate well into a native MQL5 Expert Advisor. That would let the strategy run on a VPS inside MT5, and you could test it in the MT5 Strategy Tester on Deriv's synthetic symbols. I build MQL5 EAs and have worked with this kind of swing and gap logic.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example of how I would structure it?
 Best regards,
 Oseni Ibrahim
@@ -14624,6 +14731,7 @@
           <t>Hi Zorion,
 I read the oas-execute-mcp README. Putting six independent checks and an audit log between a model and a broker order is a careful design, and running it against a live MetaTrader 5 terminal makes the stakes real.
 One layer you might find useful is a guard inside the terminal itself: an MQL5 Expert Advisor that checks every new position against hard limits and closes anything that slipped past, independent of the Python side. I build MQL5 EAs and could write that as a small, auditable component.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your approach, I can send over a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -14702,6 +14810,7 @@
           <t>Hi Thai,
 I came across mt5-python-bridge and the list of silent failure modes in the MetaTrader5 package that you wrote tests for. It is clear it came from running a real XAUUSD and FX system.
 Some of those problems are easier to close from inside the terminal: an MQL5 service or EA can confirm executions through OnTradeTransaction, keep protective stops on the broker side and export deal history with server time. I build MQL5 Expert Advisors and could write a small component that works alongside your bridge.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is useful for the production system, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -14775,6 +14884,7 @@
           <t>Hi Tej,
 I saw smc-ob-scanner, the Python port of the Volumetric Order Block script with a dashboard, CLI and an MQL5 expert advisor on top.
 Keeping Pine, Python and MQL5 versions in agreement is usually the tricky part, especially around how zones are invalidated and how bar indexing differs. I work on TradingView to MT5 conversions and MQL5 Expert Advisors, and could help with parity checks, an MQL5 indicator version that draws the zones on MT5 charts, or forex clients who want the MetaTrader side handled.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -14848,6 +14958,7 @@
           <t>Hi marketprolab team,
 I came across marketprolab and its starting premise: describe the instrument exactly as it appears in the MT5 Specification window and let the simulator behave accordingly.
 Two MQL5 pieces could support that. One is a script that exports symbol specifications (contract size, swap, margin, stops level) straight from the terminal into your format. The other is a set of reference Expert Advisors that run the example strategies in the MT5 Strategy Tester, so users can compare results side by side. I build MQL5 EAs and scripts like these.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -14921,6 +15032,7 @@
           <t>Hi Ezekiel,
 I came across your MT5 momentum trading platform, with the split between control plane and execution plane, the deterministic risk engine and the operator dashboard.
 When a platform like this goes from paper to several live accounts, running a Python terminal link per account gets heavy. An alternative is a lightweight MQL5 Expert Advisor in each terminal that receives instructions from the control plane, applies local checks and reports fills back idempotently. I build MQL5 EAs and bridges of that kind.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are heading toward live multi-account runs, I can send a short example. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -14999,6 +15111,7 @@
           <t>Hi Deepak,
 I came across TradePulse and the master-slave copier built on Redis Streams, including the note that MetaTrader5 only allows one terminal per Python process.
 That constraint is a common reason copier products move the capture and execution parts into MQL5. A master EA can publish trade events the moment they happen, and a slave EA can apply them with lot scaling and symbol mapping, while your Flask and Redis layer keeps the routing. I build MQL5 trade copiers and bridges like this.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are looking at scaling the copier, I can send a short example. Would that help?
 Best regards,
 Oseni Ibrahim
@@ -15077,6 +15190,7 @@
           <t>Hi Hans,
 I came across your XAUUSD scalper that combines CNN, LSTM and self-attention in PyTorch and trades through MetaTrader 5.
 For scalping, the round trip between Python and the terminal can matter. MQL5 can load ONNX models directly, so one option is exporting the network and running inference inside an Expert Advisor, with the EA handling entries, stops and spread filters locally. Another is keeping Python for inference and adding an MQL5 risk layer. I build MQL5 EAs and can help with either.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the ONNX route?
 Best regards,
 Oseni Ibrahim
@@ -15155,6 +15269,7 @@
           <t>Hi Daniel,
 I saw Unit8 and its goal of one strategy codebase across MetaTrader 5 and CCXT exchanges without rewrites.
 The MT5 side usually needs more care than exchanges: filling modes that differ per broker, netting versus hedging accounts, stop level limits and symbol suffixes. I build MQL5 Expert Advisors and bridges, and could help with a small in-terminal EA that handles these details and exposes a clean interface to your adapter, or review the adapter against a few real broker setups.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is useful for the project, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15228,6 +15343,7 @@
           <t>Hi Rahman,
 I came across your Telegram VIP signal auto-trader. Handling Arabic RTL text and invisible characters before parsing is a detail most copiers get wrong.
 On the execution side, an MQL5 Expert Advisor that receives the parsed signal can place orders and manage them natively: multiple take profits with partial closes, moving the stop to breakeven, and processing edits like 'close half' or 'move SL' reliably. I build Telegram-to-MT5 copiers and trade management EAs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want to extend the bot in that direction, I can send a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -15306,6 +15422,7 @@
           <t>Hi Leonardo,
 I saw MT5-Claude, the tool that reads candles and indicators from MetaTrader 5 and asks Claude for signals with key levels and risk management.
 A useful next step could be showing the answer where traders look: an MQL5 indicator that draws the entry, stop, target and key levels on the chart, or an Expert Advisor that places the trade after a confirmation click with lot size calculated from risk. I build MQL5 indicators and EAs and could write that piece so it reads the output your tool already produces.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent a short example?
 Best regards,
 Oseni Ibrahim
@@ -15384,6 +15501,7 @@
           <t>Hi Ishan,
 I came across TradeBridge, the MT5 to MCP bridge with regime detection, ATR sizing, bracket orders and trailing stops, small enough to fit on a 512 MB VPS.
 Trailing stops and brackets are one area where an in-terminal Expert Advisor helps: it reacts on every tick even if the Python services or the agent are busy or restarting. I build MQL5 EAs and could write a compact manager EA that your bridge configures through MCP, while the EA does the tick-level work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits the design, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15462,6 +15580,7 @@
           <t>Hi Alif,
 I came across nautilus_mt5, the MetaTrader 5 adapter for NautilusTrader with both data and execution clients.
 For an execution client, NautilusTrader expects accurate order and fill events, and polling the MT5 Python API can miss partial fills or modifications. An MQL5 Expert Advisor listening to OnTradeTransaction can push those events as they happen, which makes the adapter's state much easier to keep in sync. I build MQL5 EAs and bridges and could write that event feed.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would like to try it, I can send over a short example. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -15535,6 +15654,7 @@
           <t>Hi Kevin,
 I came across Tradetropy and its idea that engine differences are just a transport detail behind one Strategy API, with footprint analysis built in.
 For footprint work on MetaTrader 5, the Python package can be limiting on tick flags and market depth. An MQL5 Expert Advisor can subscribe to book events and every tick, then stream them to Tradetropy with low overhead and accept orders back. I build MQL5 EAs and data bridges and could write that transport component.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans for the MT5 side, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15608,6 +15728,7 @@
           <t>Hi Warren,
 I came across your MT5 MCP server that gives Claude access to prices, account state, positions and trade execution in MetaTrader 5.
 Two MQL5 additions could make it more useful. One is an EA that exposes values from custom indicators, which the Python package cannot read directly, so Claude can reason on the same signals a trader sees. The other is an in-terminal guard that caps risk on anything the assistant opens. I build MQL5 Expert Advisors and indicators.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either sounds interesting, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15686,6 +15807,7 @@
           <t>Hi Ruei-Ci,
 I came across Chip Whisperer, which computes volume profile levels such as POC and value area from MT5 data and answers questions through Claude and Telegram.
 It would be natural for traders to see those same levels on the MetaTrader chart. I build MQL5 indicators and Expert Advisors and could write a volume profile indicator that matches your calculation, draws the levels, and raises alerts when price reaches them, so the Telegram answers and the chart stay consistent.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is interesting, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15764,6 +15886,7 @@
           <t>Hi Agustin,
 I came across mt5-backtesting-toolkit and the way it separates experiment definitions from terminal details, with a fake runner for deterministic tests.
 The step from the fake runner to real terminals usually needs a couple of MQL5 pieces: an example EA whose inputs match your experiment schema, and OnTester or frame export code that writes results in a format your parser expects instead of scraping HTML reports. I build MQL5 Expert Advisors and testing hooks and could put together that reference pair.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -15842,6 +15965,7 @@
           <t>Hi Paul,
 I came across Forex Signal Bot, with its SMC market structure analysis, liquidity mapping, fair value gaps and Streamlit dashboard on top of MetaTrader 5.
 SMC logic is much easier to trust when you can see it on the chart. I build MQL5 indicators and Expert Advisors and could turn the structure, liquidity and FVG detection into an MT5 indicator that draws the zones, and optionally an EA that trades them on a VPS with the same risk rules as your Python version.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15915,6 +16039,7 @@
           <t>Hi LogicCrafterDZ team,
 I noticed your numbered MT5 strategy series on GitHub: SmartOrderBlocks, Liquidity Sweep Reversal, Gap Reversion Pro and Smart Scalp PA, alongside the Null Hypothesis research engine. It is a well organised way to test one idea per EA.
 When a series grows like this, the same risk sizing, session filters, trade management and logging code tends to get copied into each EA. I'm a MetaTrader developer and could help pull that into a shared MQL5 include library, so new strategies only contain their entry logic, and add optional Telegram reports for fills and daily results.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of how such a shared core is usually structured.
 Best regards,
 Oseni Ibrahim
@@ -15993,6 +16118,7 @@
           <t>Hi Harrison,
 I came across the Neuro Trading overview on GitHub and saw that MetaTrader 5 connectivity and structured risk management sit at the centre of the platform, with you as founder and lead developer.
 Integration layers like that tend to take a lot of maintenance: symbol naming differences between brokers, fill and requote handling, and keeping risk limits enforced even when the platform side is unavailable. I'm a MetaTrader developer and build MQL5 bridge EAs and broker-side risk modules that sit between a platform and the MT5 terminal.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want extra hands on the MT5 side while you focus on the AI and product work, would you be open to discussing it? I can also send over a short example of a bridge EA.
 Best regards,
 Oseni Ibrahim
@@ -16061,6 +16187,7 @@
           <t>Hi IU Technical team,
 I came across the Multi-Pair Grid Trading Manager on GitHub, a desktop app that runs grid strategies across several pairs through the MetaTrader 5 API with MySQL logging and a config panel for credentials.
 Grid systems carry most of their risk in the basket, so I wanted to suggest one addition: a small MQL5 companion EA that runs inside MT5 and enforces basket stop, equity drawdown and max-level limits even if the desktop app or its connection stops. It can also push grid status to Telegram. I'm a MetaTrader developer and build this kind of guard layer for Python-driven systems.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how the companion EA and the desktop app could share state?
 Best regards,
 Oseni Ibrahim
@@ -16129,6 +16256,7 @@
           <t>Hi ALSHAHEEN team,
 I came across the ALSHAHEEN documents on GitHub and saw that the app, distributed through the Microsoft Store, works on top of the user's own signed-in MetaTrader 5 terminal with Algo Trading enabled.
 Products built this way usually spend a lot of support time on the MT5 side: broker symbol suffixes, different filling modes, disabled algo trading and terminal builds that behave slightly differently. I'm a MetaTrader developer and can help with helper EAs or scripts that run diagnostics inside the terminal, normalise symbols and filling types, and report problems back to your app.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would take some load off your support queue, I can send over a short example of a diagnostics EA.
 Best regards,
 Oseni Ibrahim
@@ -16202,6 +16330,7 @@
           <t>Hi Chibuike,
 I came across your AI automation portfolio and the trading bot that connects MetaTrader 5, OpenAI and Telegram with daily loss limits and a live dashboard. I also saw you offer Telegram bots and API integrations on Fiverr.
 Clients who ask for a trading bot often end up needing native MetaTrader code as well: an MT4 or MT5 Expert Advisor, a custom indicator, or a TradingView alert converted into MQL5. I'm a MetaTrader developer and would be glad to work as a subcontract partner on those parts, while you keep the Python, AI and Telegram side.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could help you take on more trading jobs, I can send over a few examples of recent MQL5 work.
 Best regards,
 Oseni Ibrahim
@@ -16280,6 +16409,7 @@
           <t>Hi Samuel,
 I came across QUARSHFX Intelligence and your note on why v1 uses OANDA rather than MetaTrader: the MetaTrader5 Python package only runs on Windows with the terminal open, which does not fit a free Linux cloud host.
 There is another route for the MetaTrader bridge you mention for later. The signal engine stays on your Linux server, and a small MQL5 Expert Advisor inside the trader's own MT4 or MT5 terminal polls your API with WebRequest, then places and manages the trades locally. No Python on Windows is needed, and it works with any MetaTrader broker. I'm a MetaTrader developer and build this kind of signal-to-EA bridge.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send over a short example of the EA side.
 Best regards,
 Oseni Ibrahim
@@ -16358,6 +16488,7 @@
           <t>Hi André,
 I came across FXNews and was impressed by the discipline around it: composite scoring with MT5 calendar context, historical validation reports, and a build that fails on any MQL5 warning, not just errors.
 Since FXNews is deliberately chart-only, I wondered whether you have considered an optional layer on top. That could be a Telegram or push alert when a pair crosses a score threshold, or a separate EA that reads the scores and handles entries under fixed risk rules while the indicator stays untouched. I'm a MetaTrader developer and would follow the same zero-warning standard.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either idea interests you, I can send over a short example of how an EA can read an indicator's scores cleanly.
 Best regards,
 Oseni Ibrahim
@@ -16431,6 +16562,7 @@
           <t>Hi Maziar,
 I came across your GitHub profile and saw that AIOTA Trading Journal Pro syncs with MetaTrader 5 and is published on the MQL5 Market, alongside the Market Structure Suite and the other AIOTA products you are building.
 Selling on the Market brings its own MQL5 workload: passing automatic validation after each update, keeping MT4 and MT5 editions in step, and fixing edge cases buyers report on different brokers. I'm a MetaTrader developer and could take some of that off your plate, from new features in the sync component to Market-ready builds of new tools.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If extra MQL5 capacity would help, would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -16509,6 +16641,7 @@
           <t>Hi Daniel,
 I came across Helios and its self-learning setup that pairs a Python ML system with a MetaTrader 5 Expert Advisor. I noticed the troubleshooting section includes a case for the MT5 EA not receiving signals.
 That link between Python and the EA is where most hybrid systems get fragile. I'm a MetaTrader developer, and I usually handle it with a heartbeat between both sides, automatic reconnects, acknowledgements for every order and a safe mode in the EA that keeps stops managed if the signals stop. I can also add equity-based limits directly in MQL5.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still developing Helios, would it be useful if I sent over a short example of that bridge pattern?
 Best regards,
 Oseni Ibrahim
@@ -16582,6 +16715,7 @@
           <t>Hi Kukuh,
 I came across AI Forex Trading Assistant and its design where each user connects their own MT5 account through an isolated terminal and a private Python bridge, with Telegram as the interface. I noticed per-account worker provisioning, bridge verification and restart recovery on Windows VPS are still on the list.
 That is the part I work on most. I'm a MetaTrader developer and set up multi-terminal MT5 hosting on Windows VPS, with watchdogs that restart crashed terminals, health checks for each account, and a small MQL5 guard EA that keeps stops and daily limits enforced inside the terminal if the bridge drops.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want help getting that layer production-ready, would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -16655,6 +16789,7 @@
           <t>Hi BotTrade team,
 I came across your BotTrade workspace with the Lorentzian Classification and ML Kernel Regression EAs for MT5. I noticed the README points out two risks: stealth SL/TP orders are lost if the VPS or terminal goes down, and WebRequest calls to alert services can slow the EA.
 Both have practical fixes. A wide emergency stop can sit on the broker server while the stealth levels stay hidden, and alerts can move to a separate queue so the trading logic never waits for the network. I'm a MetaTrader developer and add this kind of protection and Telegram alerting to existing MQL5 EAs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would like, I can send over a short example of the emergency-stop pattern.
 Best regards,
 Oseni Ibrahim
@@ -16733,6 +16868,7 @@
           <t>Hi Osama,
 I came across your profile and the white-label MT5 copy-trading SaaS: multi-tenant control plane, Stripe billing, Discord and Telegram bots, and MetaTrader 5 master and follower Expert Advisors.
 In copy trading the EAs usually generate most of the support tickets: broker symbol suffixes, lot scaling between account sizes, partial closes, slippage limits and followers reconnecting after a restart. I'm a MetaTrader developer and could help on that layer, whether that means hardening the current EAs, adding MT4 followers or building per-tenant risk rules.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 With your full-stack and Web3 work also running, would extra MQL5 capacity be useful? I can send over a short example of a follower EA's sync logic.
 Best regards,
 Oseni Ibrahim
@@ -16811,6 +16947,7 @@
           <t>Hi Umair,
 I came across your case study on the live-vs-backtest divergence, where break-even and trailing were evaluated at bar close and the profit factor fell from 1.38 to 0.55. It is one of the clearest explanations of that problem I have read.
 I'm a MetaTrader developer focused on building and repairing MT4/MT5 EAs. Your diagnosis service and my work seem to fit together: once you find the cause, clients often need the trade management rewritten to tick level, an MT4 EA ported to MT5, or monitoring added so the issue does not come back. I would be glad to take on that implementation work as a partner, or refer clients who need a diagnosis to you.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -16884,6 +17021,7 @@
           <t>Hi Kenny,
 I came across your DRL XAUUSD bot and the walk-forward setup around the Soft Actor-Critic agent. I also read your honest note that the live mt5bridge.py does not mirror the backtest yet: it thresholds the action to long, short or flat, uses a fixed lot size, and places no per-trade stop loss or take profit.
 That live execution layer is my area. I'm a MetaTrader developer and could help map the agent's continuous action to position size, attach broker-side stops so trades stay protected if the script stops, and move the macro circuit breaker into a small MQL5 guard EA.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you plan to keep developing the project, I can send over a short example of how that bridge could look.
 Best regards,
 Oseni Ibrahim
@@ -16957,6 +17095,7 @@
           <t>Hi Sri Ram,
 I came across HydraPrime and the write-up behind it. Two years of solo iteration on a gold EA shows, especially in details like state recovery through terminal global variables after a VPS restart and the move to CPositionInfo and COrderInfo wrappers.
 I'm a MetaTrader developer, and the work that usually comes next for an EA at this stage is operational: Telegram reports for fills and drawdown, a watchdog on the VPS, and checks across brokers whose gold symbols, contract sizes and stop levels differ. I'd be glad to help with any of that, or be a second reviewer on the MQL5 code.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of the monitoring side first.
 Best regards,
 Oseni Ibrahim
@@ -17030,6 +17169,7 @@
           <t>Hi Mehdi,
 I came across GoldTraderEA and saw how much interest it has drawn, with around 145 stars for a gold EA that combines 14 weighted strategies with multi-layer confirmation.
 Open-source EAs that get popular usually collect the same kinds of requests: it does not trade on a certain broker because of symbol suffixes or stop levels, can it send Telegram alerts, is there an MT4 version. I'm a MetaTrader developer and would be glad to help with that maintenance, whether that means fixing broker compatibility, adding notifications or building a clean MT4 port, so you can keep working on the strategy side.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a short example of the kind of changes I mean.
 Best regards,
 Oseni Ibrahim
@@ -17103,6 +17243,7 @@
           <t>Hi Carlos,
 I came across your MQL5 Trading Bot and liked the engineering around it: an LSTM filter in front of four SMC setups, order retries with backoff, and daily drawdown protection. I noticed the model talks to the EA through a CSV file in MQL5/Files.
 File bridges work, but they tend to be where stale signals and silent stalls creep in. I'm a MetaTrader developer and could help move that link to a socket or HTTP channel with heartbeats and timestamps, so the EA knows when a prediction is fresh and falls back safely when it is not. I can add Telegram alerts for fills and errors at the same time.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that bridge?
 Best regards,
 Oseni Ibrahim
@@ -17171,6 +17312,7 @@
           <t>Hi gold-mouse team,
 I came across your MQL5 Copy Trading Bot, where the master writes trades to a binary file and several slave accounts read it to mirror positions. It is a clean, simple design, and I noticed the README already has a section on file operation errors.
 The file approach limits copying to terminals on the same machine. I'm a MetaTrader developer and have extended copiers like this with a small relay so masters and followers can run on different VPS servers, along with broker symbol mapping, lot scaling by balance and an MT4 follower for mixed setups.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still developing the bot, would it be useful if I sent over a short example of the relay approach?
 Best regards,
 Oseni Ibrahim
@@ -17244,6 +17386,7 @@
           <t>Hi Amon,
 I came across your MQL5 Projects repository with its collection of Expert Advisors, indicators and scripts, and saw that you work across MQL4, MQL5 and Python for traders who want automated solutions.
 I'm a MetaTrader developer doing similar work: MT4 and MT5 EAs, MT4-to-MT5 conversions, TradingView-to-MT5 integrations and Telegram alerts. Solo developers often get client requests in waves, so I wanted to suggest a simple partnership where we pass overflow or specialised jobs to each other, for example you keep the Python and analysis side while I take an MQL port or a copier module.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds reasonable, I can send over a few examples of my MQL5 code first.
 Best regards,
 Oseni Ibrahim
@@ -17317,6 +17460,7 @@
           <t>Hi Joel,
 I came across your Signal Service Platform, where a master Sender EA posts trades to the Express API and the dashboard handles subscriptions and flags disconnected MT5 accounts every hour.
 In setups like this the EAs decide what subscribers experience. A missed POST during a broker hiccup or a symbol with a different suffix on a follower account shows up as a missing trade. I'm a MetaTrader developer and could help harden that layer: a local retry queue and heartbeat in the Sender EA, symbol mapping and lot scaling in the receiving EA, and an MT4 receiver if some subscribers are still on MT4.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example first.
 Best regards,
 Oseni Ibrahim
@@ -17390,6 +17534,7 @@
           <t>Hi Faris,
 I came across your GitHub profile and saw that MT5 strategy development and automated trading infrastructure sit alongside your simulation engines and software platform work, including a trading signal management platform.
 I'm a MetaTrader developer focused on MQL4 and MQL5: Expert Advisors, indicators, risk modules, Telegram alerts and bridges between MT5 and Python or web backends. When the MQL side of a client project is the bottleneck, I can take that part as a subcontractor while you keep the architecture and the rest of the stack.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful for your pipeline, I can send over a few examples of recent MQL5 work.
 Best regards,
 Oseni Ibrahim
@@ -17458,6 +17603,7 @@
           <t>Hi Punokawan team,
 I came across EA Punokawan V.8_MA on GitHub, with its Dynamic Recovery Cycle, break-even projection, semi-manual buttons and hidden SL/TP.
 For averaging EAs, hidden stops are good against stop hunting, but they only exist while the terminal is running. If the VPS or connection drops, the account has no protection. I'm a MetaTrader developer and often add a wide broker-side safety stop behind the hidden levels, plus an equity guard. I can also build account-bound, time-limited trial licences, so the trial copies you send out stay under control.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either would help the next version, I can send over a short example of how the safety stop works alongside hidden SL/TP.
 Best regards,
 Oseni Ibrahim
@@ -17536,6 +17682,7 @@
           <t>Hi James,
 I came across JamesmariaEA, the MT5 Expert Advisor that trades EURUSD, EURGBP and gold with dynamic lot sizing and an equity-based stop, and saw you run it headless on Linux through Wine and Xvfb.
 With no screen to glance at, the weak points are usually visibility and combined risk: nobody notices when the terminal disconnects, and correlated EUR pairs can stack exposure. I'm a MetaTrader developer and can add Telegram reports for fills, errors and daily results, a heartbeat that warns you if the terminal goes quiet, and a cap on total exposure across the three symbols.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the monitoring module?
 Best regards,
 Oseni Ibrahim
@@ -17604,6 +17751,7 @@
           <t>Hi EA Perfect FX team,
 I came across your USDJPY M15 Expert Advisor for MT5 on GitHub, with its published Strategy Tester report and the 7-day free trial offered to anyone who sends their account number, one EA per account.
 Managing that by hand gets heavy as more traders ask for trials. I'm a MetaTrader developer and can build the account binding and trial expiry into the EA itself, with a small licence server so you can switch a trial to a paid licence or extend it without sending a new file. If you plan more pairs or an MT4 edition, I can help there too.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would save you time, I can send over a short example of the licence flow.
 Best regards,
 Oseni Ibrahim
@@ -17682,6 +17830,7 @@
           <t>Hi Sivaraman,
 I came across MT5-Dev and the ChartDrawBridge EA that fills a real gap: the official MetaTrader5 Python package cannot draw on charts, so your file-based command protocol lets Python place lines, labels and arrows.
 I'm a MetaTrader developer and have built similar bridges. If you want to take it further, a socket channel with acknowledgements removes the polling delay of files, and the same EA can also accept trade or alert commands, so one bridge covers drawing and execution. I could help with the MQL5 side of that, or with making it robust enough to share with other traders.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of the socket version first.
 Best regards,
 Oseni Ibrahim
@@ -17750,6 +17899,7 @@
           <t>Hi TradeDash team,
 I came across TradeDash MT5 EA, the on-chart dashboard for fast order entry, direct-price stop loss and take profit, trailing control and exit-all.
 Panels like this sell well to prop firm traders, and they usually ask for two things: lot size calculated from a risk percentage and stop distance, and a daily loss lock that closes everything and blocks new orders once a limit is hit. Many retail brokers also still run MT4. I'm a MetaTrader developer and could add those risk features and build a matching MT4 edition, so the dashboard reaches both groups.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of the daily loss lock.
 Best regards,
 Oseni Ibrahim
@@ -17823,6 +17973,7 @@
           <t>Hi Mykhailo,
 I came across your profile and TradeHub, with eight years of MQL4 and MQL5 work across Expert Advisors, trade copiers and risk management systems, and the BbRsi EA you published.
 I'm a MetaTrader developer doing similar work, mainly MT4 and MT5 EAs, MT4-to-MT5 conversions, TradingView-to-MT5 integrations and Telegram alerts. Busy freelance periods usually bring more good projects than one person can take, so I wanted to offer myself as a subcontractor for overflow work, delivered to your standards and under your name with the client.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could be useful, I can send over a few samples of my MQL5 code so you can judge the quality first.
 Best regards,
 Oseni Ibrahim
@@ -17896,6 +18047,7 @@
           <t>Hi MX Forex Trader team,
 I came across your Admin Panel v11 and saw that clients are managed in the cloud with PostgreSQL and JWT auth, but the MT5 EA still gets its licence list through MX_Clients.csv, downloaded and copied into MQL5/Files every time a client is added.
 Since the API is already online, the EA could check the licence itself. I'm a MetaTrader developer and can add a WebRequest call to your API at start-up and at intervals, with a cached result and a grace period so a short outage does not stop trading. New clients would work the moment you add them, and expired ones stop automatically.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that licence check?
 Best regards,
 Oseni Ibrahim
@@ -17969,6 +18121,7 @@
           <t>Hi Pranav,
 I came across your Trading Journal MT5 to Google Sheets EA, which posts each trade to a Google Apps Script URL through WebRequest. It is a simple, practical way to keep a journal without paid software.
 The weak point with Apps Script is that a timeout or quota limit can drop a trade without anyone noticing. I'm a MetaTrader developer and could add a small local queue in the EA that retries failed posts, marks trades as sent to avoid duplicates, and backfills history after the terminal restarts. An MT4 version would also let traders on MT4 brokers use it.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still improving the tool, would it be useful if I sent over a short example of the retry queue?
 Best regards,
 Oseni Ibrahim
@@ -18047,6 +18200,7 @@
           <t>Hi Badal,
 I came across the Lite version of your Trend-Following EA v2 and saw that the full version is licensed by email, with prop-firm-style risk management and a five-year NAS100 test on MT5 tick data.
 Once licences start selling, two requests tend to follow: locking each copy to the buyer's account with an expiry date, and ready-made presets for each prop firm's daily loss and maximum drawdown rules. I'm a MetaTrader developer and can build both into the EA, along with a simple way for you to extend or revoke licences without sending new files.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of the licence and preset logic first.
 Best regards,
 Oseni Ibrahim
@@ -18120,6 +18274,7 @@
           <t>Hi Andrés,
 I came across Atoms para MQL5 on your profile and liked the approach: new-bar detection, indicators, risk management and order execution as small decoupled units instead of one large EA file.
 I'm a MetaTrader developer, and libraries like this are exactly what I use when building EAs for clients. If you would like to grow Atoms, I could contribute modules that most EAs end up needing, such as session and news filters, trailing and break-even managers or a Telegram notifier, following your naming and coupling rules. I would also be open to passing along EA projects that could be built on it.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds interesting, would it be useful if I sent over a short example module first?
 Best regards,
 Oseni Ibrahim
@@ -18193,6 +18348,7 @@
           <t>Hi Monarch Trades team,
 I came across your MT4/MT5 indicators collection on GitHub, with tick movement, last-digit and candle pattern tools, and saw that you offer premium indicators and one-to-one mentorship.
 When indicators are sold, two requests usually follow. Students ask for an EA that trades the signals automatically with fixed risk rules, and paid files need protecting so they do not spread through Telegram groups. I'm a MetaTrader developer and can turn indicator logic into MT4 and MT5 Expert Advisors and add account-number licensing with expiry dates to premium tools.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either would help your offer, would you be open to discussing it? I can send over a short example first.
 Best regards,
 Oseni Ibrahim
@@ -18271,6 +18427,7 @@
           <t>Hi Dr. Khodakarami,
 I came across MT-Core-Lib and the way each YouTube session on YourTradeMaster has its own example Experts and Indicators in the TMCoreTest folders. It is a practical way to teach MQL5.
 Preparing and testing those examples for every video takes a lot of time. I'm a MetaTrader developer, and I could help build and test example projects on top of your library, including more advanced ones students often ask for, such as a trade manager panel, Telegram alerts or a TradingView-to-MT5 bridge. You would keep full control of the teaching and the code style.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you plan more sessions, would it be useful if I sent over a short example built on MT-Core-Lib?
 Best regards,
 Oseni Ibrahim
@@ -18344,6 +18501,7 @@
           <t>Hi Brent,
 I came across Pythology on GitHub and saw that you develop and optimise strategies for clients, whether they start in Python or as MT5 Expert Advisors, and that your USD Strength Index and regime dashboard update live from MT5.
 Once a strategy is optimised, clients often want it delivered as a clean MT5 EA they can run on a VPS or prop account. I'm a MetaTrader developer and could work as your MQL5 implementation partner, turning the final parameters into a robust EA with proper order handling and risk limits, and building MT5 data exports for your dashboards when needed.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of my MQL5 work first.
 Best regards,
 Oseni Ibrahim
@@ -18422,6 +18580,7 @@
           <t>Hi Andreas,
 I came across your GitHub profile and saw that, next to your web work for clients, you build algorithmic trading bots in C# for MetaTrader and cTrader.
 I'm a MetaTrader developer focused on MQL4 and MQL5. Clients who start on cTrader often later ask for the same bot on MT4 or MT5 because their broker or prop firm only offers MetaTrader, and the port to native MQL5 can take more time than expected. I would be glad to act as a subcontractor on those parts, or on any MetaTrader-specific work such as risk modules, trade copiers or Telegram alerts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could be useful, I can send over a few examples of my MQL5 code.
 Best regards,
 Oseni Ibrahim
@@ -18500,6 +18659,7 @@
           <t>Hi Naphat,
 I came across Vortex Prime and the two-year GBPUSD H1 dataset you published with it. I also liked that the README asks users to start in dry-run mode before risking real money.
 With grid and martingale logic, most of the risk sits in the basket rather than any single trade. I'm a MetaTrader developer and often add three things to EAs like this: an equity-based basket stop, a hard cap on grid levels and lot size, and Telegram alerts when the basket passes set drawdown levels. Together they give users a clear safety net when they move from dry-run to live.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still developing the EA, would it be useful if I sent over a short example of the basket guard?
 Best regards,
 Oseni Ibrahim
@@ -18573,6 +18733,7 @@
           <t>Hi Uğur,
 I came across MT4 Monitor v2 and its setup that syncs MT4 account data into SQLite and Google Sheets for the mt4pool project. It is a practical way to keep an eye on several accounts in one sheet.
 Most brokers and prop firms now push new accounts to MT5, so at some point the pool will likely mix both platforms. I'm a MetaTrader developer and could build an MT5 export EA that writes the same fields your pipeline already expects, so MT5 accounts appear next to the MT4 ones without changes to the Node side. I can also add Telegram alerts for drawdown limits or accounts that stop reporting.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the MT5 export EA?
 Best regards,
 Oseni Ibrahim
@@ -18646,6 +18807,7 @@
           <t>Hi Ratna,
 I came across your MT5 to MatchTrader Trade Copier, which mirrors MT5 trades onto MatchTrader prop firm accounts from a Python app.
 Copiers built on the MetaTrader5 Python package usually poll the terminal, so fast modifications or partial closes can arrive late, and nothing is sent if the script pauses. I'm a MetaTrader developer and could add a small MQL5 master EA that pushes every trade event to your copier the moment it happens through OnTradeTransaction, with a sequence number so nothing is missed after a restart. Symbol mapping and lot scaling per prop account can live in the same layer.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would strengthen the copier, would it be useful if I sent over a short example of the event-push EA?
 Best regards,
 Oseni Ibrahim
@@ -18719,6 +18881,7 @@
           <t>Hi Saif,
 I came across your GitHub profile and saw that you build custom indicators, Expert Advisors and forex bots on MetaTrader 4 and 5 for clients worldwide through Upwork.
 I'm a MetaTrader developer doing the same kind of work, with a focus on MT4-to-MT5 conversions, TradingView-to-MT5 bridges, trade copiers and Telegram integrations. Freelance work tends to come in waves, so I wanted to suggest a simple arrangement: when you have more jobs than time, or a client needs a module outside your usual scope, I can build it as a subcontractor and you stay the client's point of contact.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my MQL5 work first.
 Best regards,
 Oseni Ibrahim
@@ -18797,6 +18960,7 @@
           <t>Hi Massimo,
 I came across PipLock AI and liked the idea of a killswitch that makes traders stick to their own rules, with EA_PipLock sending heartbeats and account data to your Supabase webhook.
 One thing that would make it stronger is letting the EA enforce the core rules itself: closing positions and blocking new orders inside MT5 when the daily loss or trade count is reached, even if the phone or webhook is offline. I'm a MetaTrader developer and could add that, along with a queue for failed webhook posts and an MT4 version for traders on MT4 brokers.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of in-terminal rule enforcement?
 Best regards,
 Oseni Ibrahim
@@ -18875,6 +19039,7 @@
           <t>Hi Muhammad,
 I came across your profile and the 15+ funded-trader applications you have shipped, with challenge flows, leaderboards and live MT5, MatchTrader and TradeLocker account sync.
 On prop-firm projects, the MetaTrader side often needs pieces a full-stack team does not usually build: an EA that checks daily loss and drawdown on every tick, tools that export trade history in the exact format the dashboard expects, or checks for EA and copy-trading rules. I'm a MetaTrader developer and could be your MQL5 partner for those parts, so you can quote and deliver complete platforms.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of MT5 rule-monitoring code.
 Best regards,
 Oseni Ibrahim
@@ -18953,6 +19118,7 @@
           <t>Hi Jeh,
 I came across your JehKTech profile and the MetaTrader 5 copier architecture you run across funded accounts at firms like GoatFunded, AlphaCapital and FundedNext.
 Copying across prop firms gets tricky because every firm has its own daily loss rule, drawdown type and symbol names. I'm a MetaTrader developer and often build MQL5 receivers for copiers like this, where each follower account has its own rule guard that blocks or scales a trade before it breaks that firm's limits, with symbol and lot mapping per account. Native receivers also cut the delay compared with Python polling.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits where your copier is heading, would it be useful if I sent over a short example of the rule guard?
 Best regards,
 Oseni Ibrahim
@@ -19031,6 +19197,7 @@
           <t>Hi Nancy,
 I came across your profile and the multi-broker platform you built at Naxfront, with an async engine routing signals over ZeroMQ to NinjaTrader, MT5/FTMO, Interactive Brokers and Tradovate.
 Of those four, the MT5 leg usually needs the most care: the EA on the terminal side has to reconnect cleanly, confirm every fill back to the engine and respect FTMO's daily loss and max drawdown rules even when the engine sends something it should not. I'm a MetaTrader developer and build ZeroMQ and socket endpoint EAs for exactly this kind of setup.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want a second pair of hands on the MT5 side, would you be open to discussing it? I can send over a short example first.
 Best regards,
 Oseni Ibrahim
@@ -19109,6 +19276,7 @@
           <t>Hi Svenn,
 I came across your profile and the stonedesk-harness work: a per-book risk state machine, firm-aware drawdown, a watchdog and an execution-quality ledger, with nautilus-mt5-bridge connecting it all to MetaTrader 5. The focus on systems that fail safely is refreshing.
 One layer that fits your philosophy is a small MQL5 companion EA on the terminal side of the bridge. It would enforce the firm's hard drawdown limit inside MT5 even if the engine or bridge stops, and report fill prices, slippage and server timestamps straight from OnTradeTransaction for your ledger and reconciliation. I'm a MetaTrader developer and build this kind of in-terminal guard.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -19182,6 +19350,7 @@
           <t>Hi Sergio,
 I came across your NewsFilter library for MT5 and liked how small it keeps things: one WebRequest per day to the Forex Factory feed, cached and parsed with JAson.mqh, ready to drop into prop-firm EAs.
 Two additions come up often with news filters like this. The first is a fallback to MT5's built-in economic calendar when the feed is unreachable or the URL is not whitelisted. The second is Strategy Tester support, where WebRequest is not available, by loading a stored history of past events, so traders can backtest with the filter switched on. I'm a MetaTrader developer and could help with either, or with an MT4 port.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the calendar fallback?
 Best regards,
 Oseni Ibrahim
@@ -19255,6 +19424,7 @@
           <t>Hi Francisco,
 I came across your profile and the trading-ea-mql5 workspace template, with its risk-first, feature-driven structure, and saw you use it for an S&amp;P 500 highs and lows EA on prop firm accounts in MetaTrader 5.
 Combining that with a medical career cannot leave much spare time. I'm a MetaTrader developer and could take on parts of the EA work that are easy to get wrong on prop accounts: guards for each firm's daily loss and drawdown rules, a news filter around US data releases, and Telegram reports so you can check the account between shifts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, would it be useful if I sent over a short example built on your template's structure?
 Best regards,
 Oseni Ibrahim
@@ -19333,6 +19503,7 @@
           <t>Hi Javad,
 I came across JR MQL5 Market and RiskCockpit in particular: a prop-firm risk manager covering FundedNext, FTMO, E8 and The5ers rules is useful, and I noticed the .ex5 files are bound to each user's account number and sent out by hand within 24-48 hours.
 I'm an MQL4/MQL5 developer. Two things I could help with if they are on your list: MT4 versions of RiskCockpit and ProSessionBox, since many prop traders are still on MT4, and a simple automated way to issue account-bound builds so requests don't depend on your inbox. I'm also happy to take on new tools under your brand while you keep the design decisions.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of how I would handle the account binding.
 Best regards,
 Oseni Ibrahim
@@ -19401,6 +19572,7 @@
           <t>Hi Madarik Trader Pro team,
 I came across Madarik Trader Pro on GitHub and saw that it connects Deriv, Binance, MetaTrader 5 and TradingView webhooks in one bot, with a licence key per device.
 I'm an MQL4/MQL5 developer. For MT5 users, a small native Expert Advisor can make execution sturdier than driving the terminal only from Python: it can receive your bot's signals, apply lot sizing and stop rules inside MT5, and keep managing open trades if the phone or PC running the bot disconnects. I could build that companion EA to match your licence system, or add an MT4 version for users on older brokers.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're considering, I can send over a short example of how the EA would receive signals.
 Best regards,
 Oseni Ibrahim
@@ -19474,6 +19646,7 @@
           <t>Hi Neo,
 I came across your CRT Turtle Soup EAs and noticed the README says they are alert-only by default, with no auto-trading yet. The wick validation and the multi-symbol scanning across 60+ instruments from one chart are a solid base for that next step.
 I'm an MQL4/MQL5 developer, and adding execution to detection logic like this is work I do often: optional auto-entry with the existing Entry/SL/TP1/TP2 levels, partial closes at TP1, per-symbol risk limits and Telegram notifications, all switchable by inputs so the alert-only mode stays the default. The same approach could apply to the Ichimoku and gold scalper EAs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're planning, I can send over a short example of how I'd structure it.
 Best regards,
 Oseni Ibrahim
@@ -19552,6 +19725,7 @@
           <t>Hi Abdurrahman,
 I came across Traxovia AI and the 7-gate ICT engine: order blocks, fair value gaps and CHoCH confirmation, then an XGBoost confidence layer before live MT5 execution on five pairs.
 I'm an MQL4/MQL5 developer focused on the MetaTrader side of platforms like this. Once signals leave the FastAPI stack, a small MQL5 execution EA can take care of broker-specific lot and stop rounding, spread checks at entry, partial closes and trailing, and keep managing trades if the API container restarts. I could also help set up the terminal on a Windows VPS with basic health alerts so the live side runs unattended.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send over a short example of the signal-to-EA handoff.
 Best regards,
 Oseni Ibrahim
@@ -19630,6 +19804,7 @@
           <t>Hi Brayan,
 I came across your Order Blocks EA repo, the Pine Script v6 to MQL5 conversion with indicator parity checked over 12 years of EURUSD M30 data, and saw that you take freelance MQL5 and conversion projects.
 I'm a trading bot developer doing similar work: MT4/MT5 Expert Advisors, MT4 to MT5 conversion, TradingView integration and EA maintenance. When projects stack up, it can help to have another developer to pass overflow to, or to split a larger job, for example you handle the Pine logic and I cover MT4 builds, risk modules or Telegram alerts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing a simple overflow arrangement? I can send a few examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -19703,6 +19878,7 @@
           <t>Hi there,
 I came across MT5-Bridge-TradingView, the open-source bridge that picks up trades from the TradingView Strategy Tester and executes them on MetaTrader 5, and saw that you offer commercial support for custom features and installs.
 Requests on bridges like this tend to cluster around the MT5 side: partial closes, pending order types, broker symbol suffixes, lot rounding and an MT4 receiver for clients still on MT4. I'm a trading bot developer working in MQL4/MQL5 and TradingView integrations, and I could take on some of those custom jobs as a subcontractor when your queue fills up.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing that? I can send over a few examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -19776,6 +19952,7 @@
           <t>Hi Freedom,
 I came across MT5 Reverse Trader on GitHub, the PyQt5 copier that watches MT5 investor accounts and mirrors their positions to a master account, with the option to reverse direction.
 One limit of copiers built only on the Python MetaTrader5 package is that each process talks to one terminal and has to poll for changes. A small MQL5 EA on each source terminal can push trade events as they happen and handle modifications and partial closes more cleanly. I'm a trading bot developer working in MQL4/MQL5, and I could build that EA layer, or an MT4 version, to sit alongside your app.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -19844,6 +20021,7 @@
           <t>Hi Simple AlgoTrading Solutions team,
 I came across the Gold Daily Breakout EA documentation hub on GitHub and saw that you sell MINI and PRO versions on Gumroad, with prop firm settings for FTMO, BlueGuardian and others.
 Keeping two builds and several prop presets in step each time the breakout logic changes takes time, and buyers tend to ask for MT4 versions or extra protections like daily loss locks. I'm a trading bot developer working in MQL4/MQL5, and I could help maintain both builds from one codebase, add firm-specific guards, or produce an MT4 edition of the EA.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of that would help, I can send over a few examples of similar EA work.
 Best regards,
 Oseni Ibrahim
@@ -19917,6 +20095,7 @@
           <t>Hi Sadegh,
 I came across your profile and the NeuronAlgo portfolio, where research from Qlib and ML pipelines ends up deployed as MQL5 Expert Advisors on MT5, with live EAs running for over a year on prop-firm accounts.
 For small quant teams, turning a validated idea into a clean production EA with drawdown limits and allocation logic is often where time disappears. I'm a trading bot developer working in MQL4/MQL5, and I could take on that implementation step, or maintain existing EAs as brokers and prop rules change, so your time stays on research.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -19990,6 +20169,7 @@
           <t>Hi Rana,
 I came across the gold-trade-advanced-bot repo and IntradayAurumPulsePro, and saw that you offer a premium version with multi-pair support and commercial licensing for clients and prop firms.
 Once a premium EA is sold to different clients, requests pile up: account-locked licenses, custom risk settings, prop-firm daily loss guards, or an MT4 build. I'm a trading bot developer working in MQL4/MQL5, and I could help as extra capacity on those client-specific builds so you can keep focus on the core strategy.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a few examples of similar work.
 Best regards,
 Oseni Ibrahim
@@ -20063,6 +20243,7 @@
           <t>Hi Vipin,
 I came across your GitHub profile and saw that you build live algorithmic trading systems for clients, including MT5/MQL5 strategies and broker API integrations, alongside your Python work.
 When a client project needs deep MQL work, such as a full Expert Advisor, an MT4 to MT5 conversion, or an MQL5 bridge to a Python backend, it can pull time away from the rest of the build. I'm a trading bot developer focused on MQL4/MQL5, and I'd be happy to take on those parts as a subcontractor while you keep the client relationship and the Python side.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing a simple arrangement? I can share examples first.
 Best regards,
 Oseni Ibrahim
@@ -20136,6 +20317,7 @@
           <t>Hi there,
 I came across AI Backtester on GitHub, the web platform for testing and optimizing Python trading bots against real MetaTrader 5 market data.
 A natural next step for users is taking a strategy that passed your tests and running it natively inside MT5, or pulling cleaner tick and bar history straight from the terminal. I'm a trading bot developer working in MQL4/MQL5, and I could help with an MQL5 exporter EA for data, or a template that turns tested Python logic into an Expert Advisor with the same risk settings.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -20204,6 +20386,7 @@
           <t>Hi JIG BOT team,
 I came across the JIG BOT v1 page on GitHub, the XAUUSD M1 engine for MT5 with VWAP take-profit, a 10-level recovery multiplier, cent account support and SHA-256 machine verification behind a 7-day trial.
 EAs sold this way usually need steady upkeep: license checks that survive terminal reinstalls, fixes for brokers with unusual gold symbols or stop levels, and extra safeguards buyers ask for. I'm a trading bot developer working in MQL4/MQL5, and I could help maintain those parts, or build an MT4 edition if your users request one.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a few examples of similar EA work.
 Best regards,
 Oseni Ibrahim
@@ -20272,6 +20455,7 @@
           <t>Hi there,
 I came across your Telegram Signal to MT5 Auto Trader on GitHub and noticed the Future Updates list: more signal formats, custom lot sizing, advanced position management and additional platforms.
 Several of those are easier and more reliable inside the terminal. A small MQL5 companion EA can handle partial take-profits, breakeven and trailing stops even if the Python side is briefly offline, and an MT4 version covers users on older brokers. I'm a trading bot developer working in MQL4/MQL5, and I could build those pieces to plug into your existing signal reader.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -20340,6 +20524,7 @@
           <t>Hi Kawacoline,
 I came across OrderFlow Core, the Auction Market Theory system that pairs a native MQL5 Expert Advisor with a Python state machine and Telegram control, and also saw Airstrike-BTC-Engine running on MetaTrader 5.
 Two MT5 engines at once means a lot of MQL5 work: execution handling, volume profile calculations inside the terminal, and the testing that keeps the EA and Python side in agreement. I'm a trading bot developer working in MQL4/MQL5, and I could act as extra capacity on the EA side of either project.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -20408,6 +20593,7 @@
           <t>Hi Ophireum team,
 I came across the SYMMETRIX GOLD SMC document on GitHub and noticed it is marked as a production-candidate specification, with validation and broker-specific integration still required, and written for MQL5 developers among others.
 That is the kind of work I do. I'm a trading bot developer working in MQL4/MQL5, and I could implement the specification as an EA: the higher-timeframe bias, liquidity sweep and CHoCH state machine, the sizing and risk rules, and broker-specific handling for gold symbols and stop levels, followed by structured backtests against the acceptance requirements you describe.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are looking for someone to build it, would it be useful if I sent over a short example first?
 Best regards,
 Oseni Ibrahim
@@ -20486,6 +20672,7 @@
           <t>Hi Haseeb,
 I came across your XAUUSD SafeScalper EA on GitHub and saw that you take on custom EA development, strategy modifications and platform integrations.
 I'm a trading bot developer doing similar MQL4/MQL5 work: Expert Advisors, MT4 to MT5 conversion, TradingView and Telegram integrations, and fixing or maintaining existing bots. When several client requests land at once, it can help to have another developer to pass work to or to split a larger job with, for example you handle strategy logic while I cover an MT4 build or a Telegram alert module.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing a simple overflow arrangement? I can send examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -20559,6 +20746,7 @@
           <t>Hi Álvaro,
 I came across the B.E.N.D.E.R. showcase on GitHub and the Replicant copy-trading module, where each user picks a market and a broker, with IBKR and MT5 as options.
 As you expand beyond Nasdaq, the MT5 path tends to need the most care: CFD symbol names that differ per broker, contract sizes, lot steps and terminals that drop connection. I'm a trading bot developer working in MQL4/MQL5, and I could build the MT5 receiver for Replicant, an EA that takes signals from your server, maps symbols, applies per-user risk limits and reports fills back.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send a short example first.
 Best regards,
 Oseni Ibrahim
@@ -20632,6 +20820,7 @@
           <t>Hi iTrade.tools team,
 I came across QuickTrade on GitHub, the MT5 panel that combines execution, automated risk management and performance tracking, with auto partial close, breakeven offset and draggable entry, stop and target lines in v1.4.
 Since access is locked to specific account numbers and requested by email, two things often come next for tools like this: a smoother license flow, such as a key tied to the account and expiry, and an MT4 edition for traders on older brokers. I'm a trading bot developer working in MQL4/MQL5, and I could help with either, or with new panel features.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -20705,6 +20894,7 @@
           <t>Hi Vitaliy,
 I came across the Swing Zone project in your arena repo, with the KHUSA SM PRO structure engine and the two MQL5 pieces: SwingZone.mq5 for H4 levels and WebRequests to the bot, and ArenaFeed.mq5 for sending closed bars to the database.
 Those bridges tend to need care over time: retries when WebRequest fails, avoiding duplicate or missing bars after reconnects, and eventually executing trades directly from the zones. I'm a trading bot developer working in MQL4/MQL5, and I could help harden both components or add an execution module and MT4 support.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -20778,6 +20968,7 @@
           <t>Hi Haidra,
 I came across your profile and the projects listed there: the MT5 Manager REST API Copier, the Copy Trading C-Manager and the trading CRM with copy-trading rooms.
 Projects like these often pull in terminal-side work too, such as client-side EAs for MT4 and MT5 accounts, MT4 to MT5 migrations of older tools, or local risk guards. I'm a trading bot developer focused on MQL4/MQL5, and I could take on those pieces as a subcontractor while you keep the platform architecture and the client.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -20851,6 +21042,7 @@
           <t>Hi Sohaib,
 I came across your profile and the metaapi-balance-tracker project, streaming balance and equity from hundreds of MetaTrader accounts through MetaApi with rate limiting and circuit breakers.
 On projects like that, some clients eventually ask for a terminal-side option, either to cut per-account API costs or to get events without polling, for example a small MQL5 EA that pushes equity and trades to your backend, or copier and risk EAs running inside the terminal. I'm a trading bot developer focused on MQL4/MQL5, and I could handle that side as a subcontractor while you keep the platform work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -20929,6 +21121,7 @@
           <t>Hi Ans,
 I came across your profile and saw the freelance MT5 trading systems you build for a private group of Forex and Gold traders, as well as the modular FvgEA repo.
 Since your main work is Laravel and backend projects, there may be times when trader requests pile up: an MT4 version of a bot, Telegram alerts, a prop-style daily loss guard, or fixes after a broker change. I'm a trading bot developer focused on MQL4/MQL5, and I could take on those pieces as a subcontractor while you keep the client relationship.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -21002,6 +21195,7 @@
           <t>Hi TRADIVO team,
 I came across the TRADIVO V12 page in your algo2 repo and saw that you are positioning it as a professional MT5 Expert Advisor with built-in risk management and a simple setup.
 By version 12, most EA vendors are juggling buyer reports from different brokers, license handling and requests for new features or an MT4 build. I'm a trading bot developer working in MQL4/MQL5, and I could act as extra development capacity for TRADIVO, whether that means fixing broker-specific issues, adding account-based licensing, or preparing the next version.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a few examples of similar EA work?
 Best regards,
 Oseni Ibrahim
@@ -21070,6 +21264,7 @@
           <t>Hi 6amdev,
 I came across your profile and the FxBoat Quant Engine, the EA Factory that turns Python strategies into MT4, MT5 and TradingView bots with AI optimization.
 Generators like that tend to hit the same issues once real users run the output: broker-specific stop levels and filling modes, symbol suffixes, and MT4 versus MT5 order handling that the templates need to cover. I'm a trading bot developer working in MQL4/MQL5, and I could help harden the MQL templates, review generated EAs, or take on client builds that need hand-written MQL.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -21143,6 +21338,7 @@
           <t>Hi there,
 I came across your TradingView and Pine Script services repo and saw that clients bring you ideas from many sources, including MT4 and MT5 tools, and you turn them into indicators, strategies and alerts.
 Some of those clients will also want the finished strategy running on MetaTrader, either as a native MQL5 EA or with TradingView alerts executing on MT5. That is my focus: I'm a trading bot developer working in MQL4/MQL5 and TradingView to MT5 integration. We could refer work both ways, or I could handle the MetaTrader side as a subcontractor while you keep the client.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can share examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -21216,6 +21412,7 @@
           <t>Hi Yassine,
 I came across TradePilot on GitHub, the copy-trading SaaS that mirrors trades between MetaTrader accounts in real time with per-account risk sizing, and saw the MT4 and MT5 EAs that connect to your WebSocket gateway.
 As more users connect, the EA side usually needs the most attention: reconnecting cleanly after terminal restarts, resolving broker symbols, handling partial closes and stop modifications, and reporting failed copies. I'm a trading bot developer working in MQL4/MQL5, and I could help harden and test those EAs while you focus on the platform.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send a short example first.
 Best regards,
 Oseni Ibrahim
@@ -21294,6 +21491,7 @@
           <t>Hi Artan,
 I found mt5-mac-data-bridge and liked the simple approach: an MQL5 EA writing JSON files so Python on macOS can work with MT5 without Wine or Docker. Most of the reliability of a setup like that lives in the EA, such as file locking, symbol handling and how commands are confirmed back.
 I'm an MQL5 developer and could help extend or harden that EA, for example with extra data files, partial closes and modifications in the command handler, or clearer error codes for the Python side. I'm happy to follow your existing contracts and naming.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -21367,6 +21565,7 @@
           <t>Hi Ali,
 I came across meta-five and the MT5 CRM described in its README, with client onboarding, payment gateways, bonuses and a web trader built on the MetaTrader 5 Web API. Brokers who buy a CRM like that often come back asking for work inside the terminal as well.
 I'm an MQL5 developer and could act as a partner for that side: EAs or scripts for bonus and credit handling, account reports, trade copiers between client accounts, or monitoring tools that feed your CRM. You keep the client, and I deliver the MetaTrader pieces to your spec.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's useful, I can send over a few examples of MT5 work.
 Best regards,
 Oseni Ibrahim
@@ -21440,6 +21639,7 @@
           <t>Hi Dogan,
 I found your Session Rectangle indicator for MT5, which draws Sydney, Tokyo, London and New York sessions and their overlaps. I also saw MQL5 indicators and Expert Advisors listed in your profile's current focus.
 Session tools often lead to requests for session-breakout EAs, alerts when a range forms or breaks, or MT4 versions. I'm an MQL4/MQL5 developer, and I could collaborate on any of those, either building the EA layer on top of your indicator or porting it for MT4 users.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -21513,6 +21713,7 @@
           <t>Hi Bipin,
 I came across RvFx, your MQL5 grid and hedge EA with its own cycle manager and live dashboard. Cycle-based grid systems usually need the most care in basket-level protection, such as equity stops, margin checks before each level, and how a cycle recovers after a restart.
 I'm an MQL5 developer and could review CycleManager.mqh with that in mind, add equity and margin guards, or connect the dashboard state to Telegram so you can follow cycles from your phone. I'd leave the strategy itself as you designed it.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -21586,6 +21787,7 @@
           <t>Hi Daniel,
 I read your algo-trading-portfolio showcase, eight or more systems in a private monorepo, including ARIES, the event-driven framework with live execution on MetaTrader 5. With that many systems, the MT5 connection layer tends to become shared infrastructure that needs its own care.
 I'm an MQL5 developer and could help there with a terminal-side EA for fills and account events, local risk guards, or MQL versions of strategies you want to check in the Strategy Tester. I'm glad to work under an NDA on the private code.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -21659,6 +21861,7 @@
           <t>Hi Andrew,
 I came across your Meta-trader-trading-mq5 repository and the bullish continuation EA described in it. The entry rules are laid out clearly, which makes the strategy easy to build on.
 I'm an MQL5 developer and could help take it further: adding the short side, risk-based lot sizing, trailing and breakeven, running a proper Strategy Tester evaluation across symbols, and deploying it on a VPS with Telegram alerts. Given your DevOps background, I can fit into whatever deployment setup you prefer, and I'd keep your entry rules unchanged.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -21732,6 +21935,7 @@
           <t>Hi Senith,
 I came across BetterTrade and saw that it supports MetaTrader 5 history import and MT5 Auto Sync, alongside the App Store and Google Play releases. Sync with MT5 is usually the part that generates the most support questions, because brokers differ in history, commissions and symbol names.
 I'm an MQL4/MQL5 developer and could help with the terminal side, such as a sync EA that sends closed trades reliably, an MT4 version for users still on that platform, or broker edge-case fixes, so you can keep working on the app itself.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -21810,6 +22014,7 @@
           <t>Hi Mathijs,
 I came across BetterMt5 on PyPI, your friendlier wrapper around the official MetaTrader5 Python library. It's a sensible idea, since the raw API is clunky to work with day to day.
 One gap I often see with Python-only wrappers is everything that lives inside the terminal: custom indicator buffers, EA-managed positions, chart events. I'm a MetaTrader developer working in MQL4/MQL5, and I could write small MQL5 companion pieces, for example an indicator exporter or a lightweight EA, that BetterMt5 users could pair with your library, or put together a few worked examples for your README.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of what an MQL5 counterpart for BetterMt5 might look like.
 Best regards,
 Oseni Ibrahim
@@ -21878,6 +22083,7 @@
           <t>Hi Contigion team,
 I noticed the contigion-metatrader package on PyPI, the library you use to retrieve forex data across the Contigion projects. It looks like MetaTrader is already a core data source for your work.
 I'm an MQL4/MQL5 developer, and projects like this often reach a point where some logic is better placed inside the terminal: an EA that executes signals generated in Python, an indicator that plots them on the chart, or Telegram alerts fired straight from MT5. I could help with that terminal side, or take on maintenance of the MetaTrader data layer as MT5 builds change.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of that fits where Contigion is heading, I can send over a few examples of similar Python-to-MT5 setups.
 Best regards,
 Oseni Ibrahim
@@ -21946,6 +22152,7 @@
           <t>Hi there,
 I noticed you maintain both forex-mcp, an MCP server for MT5 market data over SSE, and mt5proxy, an HTTP proxy for the MetaTrader 5 Python API. Both have had releases this year, so they're clearly still active.
 I'm an MQL5 developer, and one piece I could add is a small expert advisor inside the terminal. It would push trade events, custom indicator values or chart objects to your proxy, or run execution requests with proper retcode handling and risk checks on the MT5 side. That keeps the Python layer light and covers things the Python API can't see.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send over a short example of how an EA could talk to mt5proxy.
 Best regards,
 Oseni Ibrahim
@@ -22014,6 +22221,7 @@
           <t>Hi there,
 I came across metatrader-mcp-server on PyPI, the bridge that lets Claude and ChatGPT trade MetaTrader 5 in plain language, with REST and WebSocket interfaces as well. I've also noticed it has been forked and repackaged a few times, which says a lot about the demand.
 I'm an MQL5 developer. Some features users will likely ask for are easier from inside the terminal: drawing the AI's levels on the chart, reading custom indicator buffers, or a guard EA that enforces daily loss limits no matter what the agent sends. I could build those as optional MQL5 add-ons or write worked examples for your documentation.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of these?
 Best regards,
 Oseni Ibrahim
@@ -22082,6 +22290,7 @@
           <t>Hi there,
 I noticed mcp-mt5 on PyPI, your MCP server that lets an agent compile MQL, deploy EAs, run Strategy Tester and parse the reports without opening the MetaTrader UI. The analyze_mql and deprecated-call checks are a nice touch.
 A pipeline like this works best with good reference material. I'm an MQL4/MQL5 developer and could write a small set of sample expert advisors, including an MT4 one with deprecated calls for the migration check, plus matching tester .ini presets that exercise each tool end to end. They could live in your examples folder. I'm also open to picking up MQL work from users who adopt the pipeline.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds helpful, I can send over one sample EA to start.
 Best regards,
 Oseni Ibrahim
@@ -22155,6 +22364,7 @@
           <t>Hi Leo,
 I came across mt5-mcp-by-leo and mcp-mt5-conection on PyPI, with the MQL5 backend talking to Python over TCP sockets. Covering trades, graphic objects, terminal logs and compilation through MCP is an ambitious scope.
 Keeping both the Python framework and the MQL5 socket side moving is a lot for one person. I'm an MQL4/MQL5 developer and could take on backend pieces as a subcontractor: new socket commands, JSON handling, reconnection logic, or extra tools such as indicator buffer reads and chart snapshots. You'd keep full control of the design and get clean source back.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you're open to outside help on the MQL5 side, would you like me to send a short example of socket-handling code?
 Best regards,
 Oseni Ibrahim
@@ -22228,6 +22438,7 @@
           <t>Hi Pavel,
 I came across mt4ctl, your MCP server for running headless MetaTrader 4 terminals under Wine and systemd over SSH. The headless first-login flow and per-EA AutoTrading status solve real pain for anyone running a VPS fleet.
 One piece that pairs well with it is a small heartbeat EA inside each terminal. It would write connection state, last tick, open trades and errors to a file or socket that mt4ctl reads, so the agent sees what the EAs are actually doing, not only whether the process is up. I'm an MQL4/MQL5 developer and could build it for both MT4 and MT5 if you plan to extend the tool.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -22301,6 +22512,7 @@
           <t>Hi Paulo,
 I came across mt5se, your Python framework for autonomous traders that reaches B3, NYSE and Nasdaq through MetaTrader. It's good to see it still getting releases this year, a long time after mt5b3.
 I'm an MQL5 developer and could add the terminal side of that picture. That might be an EA that runs an mt5se-trained model's decisions directly in MT5, an indicator that plots the agent's signals for review, or a few MQL5 examples for your documentation showing how the two sides interact. For students or users working with Brazilian brokers, that could make the framework easier to adopt.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of this is interesting, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -22374,6 +22586,7 @@
           <t>Hi there,
 I noticed mt5-bridge on PyPI, the FastAPI service and CLI that lets clients on any OS reach an MT5 terminal running on Windows. The recent release suggests people are actually using it.
 I'm an MQL5 developer. A bridge like this can be extended from the terminal side: a small EA that pushes trade and account events to the API instead of relying on polling, exposes custom indicator values, or blocks orders that break configured risk limits. I could build that as an optional companion, or write a couple of examples for the README showing a strategy running end to end.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example?
 Best regards,
 Oseni Ibrahim
@@ -22447,6 +22660,7 @@
           <t>Hi Soham,
 I came across MT5Forge on PyPI. The idea that a strategy only decides BUY, SELL or HOLD while the framework handles sessions, risk, notifications and monitoring is a clean way to organise MT5 bots.
 A common next request from users of Python frameworks is to check the same logic in MT5's own Strategy Tester, or to run it natively on a VPS. I'm an MQL5 developer and could write an MQL5 template that mirrors your strategy interface, so a MT5Forge strategy can be ported and compared, or provide a few examples for your readthedocs pages.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds worthwhile, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -22520,6 +22734,7 @@
           <t>Hi Slava,
 I came across mt5-grpc-server and mt5-grpc-proto on PyPI. Putting a typed gRPC API with TLS in front of MetaTrader 5 is a clean approach for remote trading and market depth access.
 Something that often comes up with Python-API servers is real-time events: trade transactions, order fills and custom indicator updates, which the Python package can only poll. I'm an MQL5 developer and could build a small EA that emits those events from OnTradeTransaction to your server, or write an example strategy client for the docs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short sketch of how that EA could plug into your proto definitions?
 Best regards,
 Oseni Ibrahim
@@ -22593,6 +22808,7 @@
           <t>Hi Brian,
 I saw mt5-lite on PyPI, your object-oriented wrapper around the official MetaTrader 5 package. Mapping MT5 error codes to Python exceptions is the kind of detail that saves people a lot of debugging.
 I'm an MQL4/MQL5 developer, and I work on the terminal side that the Python API can't reach: expert advisors, custom indicators, trade copiers and Telegram alerts sent from MT5. If users of mt5-lite ask for something that needs code inside MetaTrader, or you take on client projects that need an MQL component, I'd be glad to collaborate or take that part on.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my work.
 Best regards,
 Oseni Ibrahim
@@ -22666,6 +22882,7 @@
           <t>Hi Abdul,
 I came across mt5_mac on PyPI. Using the Wine runtime already bundled inside MetaTrader 5.app, with no Docker or Windows box, is a clever route for Mac traders.
 I noticed indicator reading currently covers Heiken Ashi computed from OHLC. I'm an MQL5 developer, and one extension would be a small MQL5 exporter indicator that writes any chart indicator's buffers, including custom or paid ones, to a file your library reads. Users would get the exact values MT5 shows rather than a recalculation. I could also write example EAs for the docs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that exporter?
 Best regards,
 Oseni Ibrahim
@@ -22739,6 +22956,7 @@
           <t>Hi Theau,
 I came across mt5-mac-bridge on PyPI. Having bridge, mock and native backends behind one identical API is a thoughtful design, and the README mentions it sits inside your own MOMQ trading project.
 If MOMQ ever needs something that runs inside the terminal, I could help. Examples are an MQL5 guard EA that enforces stops or daily loss limits even when the Python side disconnects, or an indicator that exports values the Python API can't read. I'm a MetaTrader developer working in MQL4/MQL5 and focus on that terminal side.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example of a guard EA.
 Best regards,
 Oseni Ibrahim
@@ -22812,6 +23030,7 @@
           <t>Hi Raimi,
 I saw that MT5pytrader is heading into 2.0, with structured TradeResult objects, broker preflight checks and bounded client-side trailing stops. Handling partial closes by the broker's volume step is a detail many libraries skip.
 Since the trailing stop runs client-side, it only works while the Python process is alive. I'm an MQL5 developer and could build a small companion EA that takes over break-even and trailing inside the terminal, driven by magic number or comment, so positions stay managed if the script stops. It could be an optional add-on for your docs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example?
 Best regards,
 Oseni Ibrahim
@@ -22880,6 +23099,7 @@
           <t>Hi there,
 I came across mt5-trading-lib on PyPI. An async MetaTrader 5 client with a circuit breaker, TTL caching and encrypted credentials goes well beyond the usual thin wrapper.
 One area Python can't fully cover is what happens inside the terminal: trade transaction events, custom indicator values, or protective logic that must keep working if the client disconnects. I'm an MQL5 developer and could build a small companion expert advisor that pushes events to your event-driven layer, or a guard EA that enforces stops independently. Both could be optional extras for your users.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -22953,6 +23173,7 @@
           <t>Hi Vincent,
 I came across mt5-trading-mcp and liked the consent and audit layer in front of real trades. I also noticed you already use a small MQL5 expert advisor, AgentScreenshot, for native chart captures.
 Since part of the project already lives in MQL5, there may be room for more there. One option is an EA-side risk guard that rejects or closes positions outside limits even if the agent misbehaves. Another is an exporter for custom indicator buffers, or chart annotations that show the agent's reasoning. I'm an MQL4/MQL5 developer and could help build or maintain those pieces.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one?
 Best regards,
 Oseni Ibrahim
@@ -23026,6 +23247,7 @@
           <t>Hi Krunal,
 I came across nostro_mt5_manager on PyPI, your Python wrapper for the MetaTrader 5 Manager API, along with its GitBook docs. Manager API work usually means you're close to brokers or prop setups running their own MT5 servers.
 Those clients often need terminal-side tools as well: expert advisors, trade copiers, equity and drawdown guards, or MT4-to-MT5 ports of older code. I'm an MQL4/MQL5 developer and could act as extra capacity for that side of your projects, working to your specifications while you stay focused on the Manager API layer.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could be useful, I can send over a few examples of related work.
 Best regards,
 Oseni Ibrahim
@@ -23094,6 +23316,7 @@
           <t>Hi there,
 I came across Py2MQL5 on PyPI, the wrapper that lets the official MetaTrader5 package drive several portable terminals at once. That's a real limitation of the stock package, so the workaround is useful.
 People running many terminals side by side often also need something inside each one: a local trade copier between accounts, a monitoring EA that reports equity and connection state, or per-account risk guards. I'm an MQL4/MQL5 developer and build those terminal-side tools. They could complement Py2MQL5 for multi-account users or serve as examples in your docs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working with, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23167,6 +23390,7 @@
           <t>Hi Henrique,
 I came across pymt5linux and your mt5docker image. Keeping MT5 on Linux working across terminal updates is thankless work, and moving it to Python 3.13 is appreciated by people who run it headless.
 In headless setups it helps to have something inside the terminal reporting back. I'm an MQL5 developer and could build a small heartbeat EA that writes connection state, last tick time and open positions to a file or socket, so a container health check can tell whether trading is really live. It could ship as an optional example alongside mt5docker.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -23235,6 +23459,7 @@
           <t>Hi there,
 I came across PythonMetaTrader5 on PyPI. Accepting SL and TP either as absolute prices or point offsets, with normalisation to the symbol's digits, removes a common source of rejected orders.
 I noticed pyautogui in the dependencies, which usually means some actions can't be done through the Python API alone. I'm an MQL5 developer, and a small companion EA can often take over those steps, such as chart handling, indicator reads or protective closes, by listening to commands from Python through files or sockets. That tends to be more reliable than GUI automation.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's relevant, I can send over a short example of how it would work.
 Best regards,
 Oseni Ibrahim
@@ -23308,6 +23533,7 @@
           <t>Hi Mahmudul,
 I came across shawon-mt5-automation on PyPI, your Flask webhook server that turns TradingView alerts into MT5 trades with API-key auth, USD-based SL/TP and signal gap control.
 TradingView-to-MT5 is a big part of my work as an MQL4/MQL5 developer. Some clients prefer an EA-side receiver that handles partial closes, break-even, trailing and per-symbol risk inside the terminal, next to a webhook layer like yours. If you take on client projects in this area, I'd be glad to collaborate on the MQL side or take overflow work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of an EA-side receiver.
 Best regards,
 Oseni Ibrahim
@@ -23381,6 +23607,7 @@
           <t>Hi Bahadir,
 I came across SiliconMetaTrader5, the Docker-based way to run MT5 with Python on Apple Silicon. I liked that the README is honest about using a native Windows server for live, high-capital trading.
 That handoff from Mac development to live deployment is where I usually help. I'm an MQL4/MQL5 developer and can port a strategy prototyped in Python into a native MQL5 expert advisor, set it up on a Windows VPS, and add monitoring. If your users ask about that step, or you have strategies of your own to move, I could be a useful contact.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent over a short example of a Python-to-MQL5 port?
 Best regards,
 Oseni Ibrahim
@@ -23454,6 +23681,7 @@
           <t>Hi there,
 I came across n8n-nodes-metatrader5 on npm and noticed its repository sits on BlackBull Markets' GitHub Enterprise. An n8n node is a friendly way to open MT5 automation to traders who don't write code.
 I'm an MQL4/MQL5 developer. Workflows like these often need something inside the terminal as well: an EA that receives n8n webhooks and executes with proper lot and risk checks, or one that pushes fills and equity changes back into a workflow. I could build those as companion pieces or as example templates for the node's documentation.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23527,6 +23755,7 @@
           <t>Hi there,
 I noticed n8n-nodes-ohlcv-metatrader on npm, which pulls MetaTrader candles, gold included, into n8n workflows next to crypto exchange data.
 Once the analysis runs in n8n, the next question is usually how to act on it inside MetaTrader. I'm an MQL4/MQL5 developer and could build a small EA that takes decisions from a workflow via webhook or file, places orders with lot sizing and SL/TP, and reports results back. It could work as a companion to your node or as an example workflow in the README.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -23595,6 +23824,7 @@
           <t>Hi mt5cli team,
 I came across mt5cli on npm, the Docker-first MetaTrader 5 CLI for headless Linux with EA and backtest support and no dependencies.
 A tool like this is only as convincing as its first run, so good sample material helps. I'm an MQL5 developer and could write a couple of reference expert advisors with matching tester presets that demonstrate compiling, running a backtest and reading results through the CLI. If your users bring their own EAs that fail to compile or behave differently headless, I'm also happy to take that work on.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over one sample EA to try.
 Best regards,
 Oseni Ibrahim
@@ -23668,6 +23898,7 @@
           <t>Hi Altug,
 I came across metatrader5-sdk on npm, your Node.js SDK for the MetaTrader 5 Web API. It's a useful bridge for JavaScript teams that don't want to touch Python or MQL.
 Web API integrations handle accounts and trades well, but some features only run inside the terminal: custom indicators, EA-side risk rules and chart objects. I'm an MQL4/MQL5 developer and could write companion EAs or examples for your README showing how a Node app and an MT5 expert advisor work together. I can also help if you take on client work that needs an MQL component.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's of interest, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23741,6 +23972,7 @@
           <t>Hi Halit,
 I came across biquote, the free market data API and SDKs. Offering 15,000 requests a minute with no API key is generous, and I noticed the prices come from a MetaTrader 5 feed.
 I'm an MQL4/MQL5 developer, and for a service like this the terminal-side collector matters a lot. I could help harden the feed EA with reconnection handling, stale-tick detection and heartbeat alerts, add symbols or brokers, or write an MQL5 client example so MT5 users can pull biquote's economic calendar straight into their EAs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of these?
 Best regards,
 Oseni Ibrahim
@@ -23814,6 +24046,7 @@
           <t>Hi Gil,
 I came across mt4manager on npm, your Node-API bindings for the MetaTrader 4 Manager API. Giving brokerage back-office teams a TypeScript interface instead of raw C++ is a good call.
 Brokers using tools like this often have MQL work too, such as client EAs, copier tools, risk scripts, or moving existing MT4 code to MT5 as they migrate servers. I'm an MQL4/MQL5 developer and could take on that side for your clients, or write terminal-side test EAs that generate realistic trading activity while you test the pumping and event APIs.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few relevant examples.
 Best regards,
 Oseni Ibrahim
@@ -23887,6 +24120,7 @@
           <t>Hi Mauro,
 I noticed @mautriz/mt5 on npm, the TypeScript client for your MetaTrader 5 WebSocket API. Streaming MT5 over WebSockets with a typed client is a practical setup for web dashboards and bots.
 Services like this usually rely on something inside the terminal, often an MQL5 EA or bridge, that has to keep working through MT5 build changes. I'm an MQL4/MQL5 developer and could help build or maintain that side, add events such as trade transactions or indicator values, or write example EAs for your documentation.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's relevant to what you're building, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23955,6 +24189,7 @@
           <t>Hi TradeRail team,
 I came across the traderail SDK on npm for your managed MetaTrader 5 API, including the copy-trading side. A hosted MT5 API spares developers a lot of Windows and terminal setup.
 Customers of managed APIs often come back with requests that sit inside MetaTrader: a custom EA, a copier variant with special lot rules, or equity and drawdown guards. I'm an MQL4/MQL5 developer and could be the person you refer that work to, or build example strategies that show the SDK and an MT5 EA working together.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of similar work.
 Best regards,
 Oseni Ibrahim
@@ -24023,6 +24258,7 @@
           <t>Hi there,
 I came across synapse-mt5 on npm, the native C++ MCP server that connects AI assistants to MetaTrader 5 without Python. The repo name, MCP-MQL5, suggests a good share of the work happens on the MQL5 side.
 I'm an MQL4/MQL5 developer and could help extend that part: new tools for indicator buffers or chart objects, EA-side risk limits the AI can't bypass, or MT4 support if users ask for it. I'm happy to work within your architecture and hand back clean source.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of those tools?
 Best regards,
 Oseni Ibrahim
@@ -24091,6 +24327,7 @@
           <t>Hi there,
 I came across StrategyLab on npm, your AI-powered EA development framework for MetaTrader 5 built around Claude Code. Having a structured workflow instead of prompting from scratch makes a lot of sense.
 AI-written EAs tend to fail in similar places: order filling modes, broker stop levels, netting versus hedging accounts, and new-bar detection. I'm an MQL4/MQL5 developer and could act as a human review and fix step for EAs produced with StrategyLab, or write hand-checked template EAs the framework could start from.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, I can send over a short checklist and an example.
 Best regards,
 Oseni Ibrahim
@@ -24159,6 +24396,7 @@
           <t>Hi there,
 I came across mt5-quant-forex-panel on npm, your MetaTrader 5 quant panel with ten backtested strategies, a multi-signal core and a live dashboard.
 Some users will want to run those strategies natively in MT5, to confirm them in the Strategy Tester with real tick data or to keep them running on a VPS without the panel. I'm an MQL4/MQL5 developer and could port selected strategies into MQL5 expert advisors that follow your logic and parameters, with risk limits enforced inside the terminal.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's interesting, I can send over a short example of a ported strategy.
 Best regards,
 Oseni Ibrahim
@@ -24232,6 +24470,7 @@
           <t>Hi Clawtrade team,
 I came across Clawtrade, the self-hosted AI trading agent platform that brings crypto venues, Interactive Brokers and MetaTrader 5 together in one dashboard.
 The MT5 connector runs through the Python API, which works but brings forex-specific surprises: broker symbol suffixes, filling modes, stop levels and netting versus hedging accounts. I'm an MQL4/MQL5 developer and could help make that module sturdier, or add an optional MQL5 EA that executes agent decisions inside the terminal with its own risk checks. It would stay independent of the agent loop, so stops still apply if the server restarts.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -24305,6 +24544,7 @@
           <t>Hi Peter,
 I came across your metatrader4 package for trading MT4 from Node.js. I noticed the setup depends on dingmaotu's mql4-lib and mql-zmq, copied by hand into the MQL4 folders.
 Those libraries are not very active anymore, and many brokers are moving clients to MT5. I'm an MQL4/MQL5 developer and could build an MT5 version of the bridge EA using the same message format, or simplify the MT4 install so it needs fewer external pieces. That would let your Node.js API cover both platforms.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -24373,6 +24613,7 @@
           <t>Hi there,
 I came across @0xrelogic/mt5-analysis-mcp on npm, with analysis tools, trading operations and a 15-condition alert system for MT5. I also noticed the recent pip value calculation fix.
 Pip and tick values are easy to get wrong outside the terminal, especially for metals, indices and non-USD accounts. I'm an MQL5 developer and could build a small helper EA that returns the terminal's own tick value, contract size and margin figures, and can also run your alert conditions inside MT5 so they fire even when the MCP server is idle.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -24441,6 +24682,7 @@
           <t>Hi there,
 I came across @herjarsa/mt5-mcp-super on npm, the one-command installer that sets up your MT5 MCP server in Claude Code, OpenCode, Codex and Gemini CLI. Making setup that easy should bring in a lot of MT5 traders.
 Many of them will soon ask for things that only work inside the terminal: custom indicator values, chart drawings from the agent, or an EA that enforces risk limits whatever the agent sends. I'm an MQL4/MQL5 developer and could build those as companion pieces for the server.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -24509,6 +24751,7 @@
           <t>Hi there,
 I came across mql5-mcp on npm, which lets an agent compile and test expert advisors and indicators. Closing the loop between writing MQL5 and seeing compiler and tester output is what makes AI-assisted EA work usable.
 I'm an MQL4/MQL5 developer and could help in two ways: a set of small reference EAs and indicators with known expected results that serve as tests and docs examples, and a human review step for tricky cases the agent keeps getting wrong, such as filling modes, stop levels and multi-symbol handling.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds helpful, I can send over one reference EA to start.
 Best regards,
 Oseni Ibrahim
@@ -24577,6 +24820,7 @@
           <t>Hi there,
 I came across mql5-ea-mcp, your MCP server that indexes the MQL5 help, the Algo Book and the Neural Networks Book, with an error database for diagnosing EA problems.
 The most useful error entries usually come from live accounts rather than the docs: invalid stops from broker freeze levels, unsupported filling modes, netting account surprises, and 4756 or 10030 codes. I'm an MQL4/MQL5 developer and could contribute a set of these real cases with fixes, and I'm also open to working together on EA client projects.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a few sample entries?
 Best regards,
 Oseni Ibrahim
@@ -24650,6 +24894,7 @@
           <t>Hi IndexNano team,
 I came across @indexnano/mt5-ws on npm, the WebSocket SDK for your MT5 API with real-time orders and quotes.
 Services like this usually depend on something inside MetaTrader that has to stay reliable through terminal updates, and customers soon ask for extras such as custom EAs, trade copiers or risk guards next to their API integration. I'm an MQL4/MQL5 developer and could help with that terminal side, or take the MQL requests your customers bring in, working under your brand and to your specifications.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's relevant, I can send over a few examples of similar work.
 Best regards,
 Oseni Ibrahim
@@ -24723,6 +24968,7 @@
           <t>Hi Charles-Antoine,
 I came across tree-sitter-mql5 on npm. A proper Tree-sitter grammar for MQL5 is something the community has long lacked for editors and code tools.
 Grammars tend to break on the odd parts of the language: D'...' and C'...' literals, input groups, #property lines, templates, #import blocks and MT4-style code that still compiles in MT5. I'm an MQL4/MQL5 developer with a lot of real EA and indicator code, and I could put together a varied test corpus of these cases. I'm also open to working together on MQL-related projects.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a first batch of test files?
 Best regards,
 Oseni Ibrahim
@@ -24791,6 +25037,7 @@
           <t>Hi there,
 I came across your mql5-json, mql5-promise and mql5-timer packages. Shipping MQL5 libraries through npm, and bringing a Promise-style interface into MQL5, is an unusual approach that I liked.
 I'm also an MQL4/MQL5 developer, working on expert advisors, trade copiers, Telegram and webhook integrations. If you or the HommaTech mql-simplify project ever need extra hands, whether on client EAs or on new modules like an HTTP/WebRequest wrapper built on your promise library, I'd be glad to collaborate or take on subcontracted work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds interesting, I can send over a few examples of my code.
 Best regards,
 Oseni Ibrahim
@@ -24864,6 +25111,7 @@
           <t>Hi Hristiyan,
 I came across mql5-lib on npm, the MQL5 language definitions for C++ IDEs. Being able to write MQL5 in a proper IDE with completion, instead of MetaEditor, is something many of us want.
 I'm an MQL4/MQL5 developer and could help test the definitions against real EA and indicator code, trade classes, chart objects and event handlers, and report or fix the gaps. I'm also open to collaborating or taking on overflow if you do client MQL5 work.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's useful, I can send over a sample set of files to test against.
 Best regards,
 Oseni Ibrahim
@@ -24932,6 +25180,7 @@
           <t>Hi there,
 I came across mql-interpreter on npm, a TypeScript lexer, parser, semantic checker and runtime for running MQL4/5 in Node.js. That's a big undertaking.
 As the built-in stubs grow, a reliable reference helps: real EAs and scripts with known outputs from MetaTrader itself, covering OrderSend and CTrade behaviour, series indexing, ArraySetAsSeries and similar quirks. I'm an MQL4/MQL5 developer and could build a corpus like that, and help check how built-ins behave in the real terminal, including differences between MT4 and MT5 builds.
+Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a first set of reference scripts?
 Best regards,
 Oseni Ibrahim

</xml_diff>

<commit_message>
Revert pricing line from cold emails; add inbox monitor runbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -6527,7 +6527,6 @@
           <t>Hi Breno,
 I read the MT5 Web Replicator README, with the Rails dashboard receiving and replicating MT5/MQL order data across accounts alongside the python-signal client, and saw that you are open to co-maintainers or partners.
 I am an MQL4/MQL5 developer who works on trade copiers and MetaTrader integrations, so the terminal side is where I could help most: the EA that reports and receives orders, symbol mapping and lot scaling between accounts, reconnect handling, and MT4 support if you ever want it. I am comfortable working inside an existing codebase and keeping changes small and documented.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still looking for someone to share the load, I would be glad to talk it through. Would it be useful if I sent over a few examples of my copier work first?
 Best regards,
 Oseni Ibrahim
@@ -6606,7 +6605,6 @@
           <t>Hi Felix,
 I came across your TradeMate showcase, the risk-first MT5 Expert Advisor with its Python monitor, six filter layers and daily loss halt. Presenting it with private source and a clear engineering write-up is a smart way to show clients what you build.
 I am an MQL4/MQL5 developer as well, focused on EAs, risk management, trade copiers and MT4 to MT5 conversion. Since you take on client projects, I thought collaboration could help both of us: I could cover MT4 versions of your EAs, take on smaller modules when your schedule is full, or handle Strategy Tester runs and VPS setup.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my work. Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -6690,7 +6688,6 @@
           <t>Hi Hưng,
 I came across ICT System EA v2.0, your MT5 Expert Advisor built on Inner Circle Trader concepts for The5%ers, with the backtest results laid out in the README.
 For prop-firm use, the pieces around the strategy often decide whether an account survives: a daily loss limit calculated exactly as the firm defines it, a pause around high-impact news, and equity checks that stop trading before the max loss is touched. I am an MQL5 developer and build these as modules that plug into an existing EA without changing entries.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are planning further versions or running the EA on more funded accounts, I would be glad to help. Would it be useful if I sent over a short example of such a module?
 Best regards,
 Oseni Ibrahim
@@ -6774,7 +6771,6 @@
           <t>Hi Jayadev,
 I came across your profile and the TradingView to MT5 webhook bridge with its queued, deduplicated order intake. I also saw that Pine-to-MQL5 ports, trade copiers and prop-firm rule logic are all part of what you deliver.
 I am an MQL4/MQL5 developer doing the same kind of work, and I wondered whether extra capacity on the MetaTrader side would ever help, for example taking a Pine-to-MQL5 port or an MT4 version of a client EA when your queue is full, delivered to your standards and under your name.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is something you would consider, I can send over a few examples of my MQL code so you can judge quality first. Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -6858,7 +6854,6 @@
           <t>Hi Noel,
 I came across TelegramSignalTrader, your EA for trading and managing accounts through Telegram, and noticed the setup guide centres on the MT4 file, TelegramSignalTrader.mq4.
 As more brokers and prop firms move clients to MT5, a maintained MQL5 version with the same Telegram commands can save you a lot of support questions. I am an MQL4/MQL5 developer and do MT4 to MT5 conversions regularly, including the parts that change the most: order handling moving to positions and deals, and WebRequest-based Telegram calls.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If an MT5 build or general maintenance of the EA would be useful to TradeAdviser, I would be glad to help. Would it be useful if I sent over a short example of a converted module?
 Best regards,
 Oseni Ibrahim
@@ -6937,7 +6932,6 @@
           <t>Hi Morteza,
 I came across tv-connector, your TradingView to MT5 bridge with HMAC-verified webhooks, a Redis queue and an MT5 EA that polls for orders. Clean design, and a good fit for traders who want something self-hosted.
 I am an MQL4/MQL5 developer and work on similar bridges, copiers and risk modules. Since you build trading systems for others, I thought there might be room to cooperate: I could write the MT4 version of your EA, add trade management features on the MQL side, or take on EA work when you have more projects than time.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my MQL code first. Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -7016,7 +7010,6 @@
           <t>Hi Pranay,
 I came across forex-mt5-strategies, your set of seven MQL5 Expert Advisors with Strategy Tester reports and design documents, including the custom oscillators built from parametric curves.
 Since you work across many venues, I thought an MQL-focused collaborator might be useful. I am an MQL4/MQL5 developer and handle the MetaTrader-specific parts that eat time: broker filling modes, stops-level checks, tester automation for multi-symbol runs, VPS deployment and MT4 versions when clients need them.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you take on client work involving MT5 EAs, I would be glad to support it. Would it be useful if I sent over a short example of my tester automation setup?
 Best regards,
 Oseni Ibrahim
@@ -7090,7 +7083,6 @@
           <t>Hi ArkoRisk team,
 I came across ArkoRisk, the open-source MT5 manager for position sizing, pending orders and prop-firm risk, with lot calculation by balance or equity percent and draggable Entry, SL and TP lines.
 Tools like this get a lot of requests once traders start using them: an MT4 edition, daily loss locks for prop accounts, partial close presets, or sizing across several positions at once. I am an MQL4/MQL5 developer who builds risk management panels and EAs, and I could help implement some of these or port the tool to MT4.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would welcome help with the backlog, I would be happy to contribute. Would it be useful if I sent over a short example of a daily loss lock module?
 Best regards,
 Oseni Ibrahim
@@ -7169,7 +7161,6 @@
           <t>Hi Sergio,
 I came across SignalReplicator and noticed that the Desktop plan only works with MT5 because the desktop expert advisor is written in MQL5, so MT4 users have to move to the Cloud plan.
 An MQL4 version of the desktop EA would let MT4 traders use the cheaper desktop option and reduce how much of your volume depends on MetaApi. I am an MQL4/MQL5 developer who works on Telegram copiers, and I could port the EA while keeping the same behaviour: multi-TP handling, break-even, trailing, partial closes and per-channel risk.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, I would be glad to help. Would it be useful if I sent over a short example of an MT4 receiver matching an MQL5 one?
 Best regards,
 Oseni Ibrahim
@@ -7248,7 +7239,6 @@
           <t>Hi FlowMetrix team,
 I came across FlowMetrix, your Windows app for managing several MT5 accounts and terminals from one dashboard with copy trading between them.
 A common request for multi-account tools is MT4 support, since many traders still hold MT4 accounts with prop firms and brokers. I am an MQL4/MQL5 developer who builds copier components, and I could write the MT4 side so those accounts appear in the same dashboard, along with symbol mapping, lot scaling rules and safeguards for partial closes and reconnects.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If widening platform support is on your list, I would be happy to help. Would it be useful if I sent over a short example of an MT4 to MT5 copy module?
 Best regards,
 Oseni Ibrahim
@@ -7322,7 +7312,6 @@
           <t>Hi ICT Library team,
 I came across ICT_Library_MQ5 and liked how it exposes SMC and ICT patterns as typed snapshots on closed candles, with the detection rules documented. Reaching over 200 stars for an MQL5 library is impressive.
 Popular libraries tend to get the same questions again and again: how to use it inside a full EA, and whether it runs on MT4. I am an MQL4/MQL5 developer and could help with both, for example a few reference EAs showing risk-managed entries built on the library, or an MQL4 port of the core detection.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would welcome a contributor or paid help for your own projects, I would be happy to talk. Would it be useful if I sent over a short example EA first?
 Best regards,
 Oseni Ibrahim
@@ -7406,7 +7395,6 @@
           <t>Hi Jason,
 I came across GGTH Predictor, where the Python side runs a five-model ensemble plus news sentiment and the MQL5 EA reads the results from shared JSON files to manage EURUSD trades.
 In setups like this, the EA usually needs the most defensive code: detecting stale or half-written prediction files, handling restarts without duplicate orders, and keeping risk limits independent of the model output. I am an MQL4/MQL5 developer and could help harden that side, extend it to more symbols, or set the whole system up on a VPS so both processes restart cleanly.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are continuing to develop GGTH, I would be glad to help. Would it be useful if I sent over a short example of a file-based signal reader?
 Best regards,
 Oseni Ibrahim
@@ -7480,7 +7468,6 @@
           <t>Hi DojiMonitorEA team,
 I came across DojiMonitorEA, the MT5 Expert Advisor that scans every Market Watch symbol for Doji candles and sends terminal or push notifications, and saw you invite people to get in touch about collaboration.
 A scanner like this is easy to grow into something traders will pay for: Telegram alerts with a chart snapshot, extra patterns such as engulfing or pin bars, multi-timeframe filters, or an MT4 edition. I am an MQL4/MQL5 developer and build scanners, alert systems and Telegram integrations for MetaTrader.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are open to developing it further, I would be glad to help. Would it be useful if I sent over a short example of a Telegram alert module in MQL5?
 Best regards,
 Oseni Ibrahim
@@ -7559,7 +7546,6 @@
           <t>Hi Chacha,
 I came across your AI Telegram Signal Copier backend, which filters Telegram messages, turns signals like 'BUY GOLD NOW SL 2330 TP 2360' into JSON with OpenAI, and hands them to an MT5 EA on Algo Forge.
 As signal channels get more varied, most of the work shifts to the EA: multiple take-profits, later edits to SL and TP, 'close half' messages, and avoiding duplicate orders after a restart. I am an MQL4/MQL5 developer who builds this kind of trade management, and I could also produce an MT4 version for users on that platform.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are taking the project further or using it for clients, I would be glad to help. Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -7643,7 +7629,6 @@
           <t>Hi Fortune,
 I came across your Triple-EA Prop-Firm Portfolio, with three MT5 EAs on US500 and USDJPY coordinated by a central PortfolioRiskManager. Sharing one risk budget across separate EAs is something most prop traders never get right.
 I am an MQL4/MQL5 developer who works on prop-firm risk management, multi-EA coordination and MT4 to MT5 ports. If you are extending the portfolio, adding firms with different daily loss definitions, or taking on clients who want something similar, I could help with the MQL side, testing across brokers, or VPS deployment.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If collaboration sounds useful, I would be glad to talk. Would it be useful if I sent over a short example of a shared-risk module?
 Best regards,
 Oseni Ibrahim
@@ -7722,7 +7707,6 @@
           <t>Hi QuantumEdgeProPlus team,
 I came across QuantumEdgeProPlus v11.0, your MT5 Expert Advisor with reinforcement learning and risk management, and saw that a professional edition is sold through Gumroad.
 Once an EA has paying users, a good share of the work becomes support: broker-specific errors, symbol suffixes, different contract sizes on gold and indices, and requests for an MT4 build. I am an MQL4/MQL5 developer and could take on part of that load, from fixing reported issues to preparing an MT4 edition and testing new versions before release.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If extra help would let you focus on the strategy itself, I would be glad to assist. Would it be useful if I sent over a few examples of my EA work?
 Best regards,
 Oseni Ibrahim
@@ -7801,7 +7785,6 @@
           <t>Hi Toki,
 I came across AI Trader for MT4, your framework that connects large language models to MetaTrader 4 with risk rules, a signal lifecycle and traceable execution.
 Since many brokers and prop firms now only offer MT5, an MQL5 bridge that speaks the same protocol as your MT4 side could widen the audience without changing the Python layer. I am an MQL4/MQL5 developer and have worked on this kind of bridge, including the MT4 to MT5 differences in order and position handling.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If adding MT5 support or hardening the MQL4 bridge is on your list, I would be glad to help. Would it be useful if I sent over a short example of an MQL5 bridge receiver?
 Best regards,
 Oseni Ibrahim
@@ -7881,7 +7864,6 @@
 I came across your Forex-Gold-Auto-Trader repository, the gold EA for MT4 and MT5 with configurable risk rules and a one-time license.
 Looking at your profile, you also take on a wide range of automation work outside trading, so keeping two MQL builds in sync, handling buyer customization requests and dealing with broker-specific issues can take a lot of time. I'm an MQL4/MQL5 developer who focuses only on MetaTrader work: EA fixes, MT4/MT5 parity, extra risk controls and Telegram notifications.
 If you ever want to pass on MQL tasks or client requests around the gold EA, I'd be happy to help as a subcontractor.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful? I can send over a few examples of my EA work.
 Best regards,
 Oseni Ibrahim
@@ -7961,7 +7943,6 @@
 I came across your GitHub profile and liked the line "Coding or Trading! Depending on the hour." I noticed you work in MQL4 and MQL5 next to your Next.js and TypeScript work at 1MF Ventures.
 When one person covers both the web stack and the trading side, MetaTrader projects often sit half-finished. I'm an MQL4/MQL5 developer who focuses only on MetaTrader: building Expert Advisors and indicators, fixing or porting MT4 code to MT5, and connecting EAs to web backends or Telegram.
 If you have a trading tool you'd like built or finished while you focus on the rest of 1MF Ventures, I'd be happy to help.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -8041,7 +8022,6 @@
 I came across your Gartal-Inc repository and the Decision Alpha Lab work, and the scale of the testing stood out: more than 9,700 documented tests with explicit quality gates.
 With that much research, the step from a validated idea to a reliable MetaTrader EA can become a bottleneck. I'm an MQL4/MQL5 developer and could help turn strategies that pass your gates into production Expert Advisors, with the same position sizing and risk rules, clean logging, and exports that match your Python analysis so live and backtest results can be compared.
 I'm also happy to build MT4 and MT5 versions of the same logic if you want both.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how I'd structure one of these EAs?
 Best regards,
 Oseni Ibrahim
@@ -8121,7 +8101,6 @@
 I came across TV2MT5 and liked the idea of charting on TradingView while the trades land in MetaTrader 5 from a local Windows machine.
 I noticed it targets MT5 only. A fair number of traders are still on MT4 accounts with their broker or prop firm, and they often ask for the same kind of copier. I'm an MQL4/MQL5 developer and could help build an MT4 receiver EA that plugs into your existing flow, or tidy up the MetaTrader side of the project, such as symbol mapping, partial closes and error handling for rejected orders.
 Happy to contribute through pull requests or as paid work, whichever suits you.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how the MT4 side could look?
 Best regards,
 Oseni Ibrahim
@@ -8201,7 +8180,6 @@
 I came across your MT5-SMC-trading-bot repository, with the Order Block, FVG and BOS modes, adaptive ATR filters and regime detection, and saw that you offer consulting to institutions.
 When an open-source EA gets attention, requests tend to follow: an MT4 version, broker-specific tweaks, extra risk rules or Telegram alerts for a particular desk. I'm an MQL4/MQL5 developer and could take on that kind of work as a subcontractor, so your consulting clients get what they need while you stay on the strategy and research side.
 An MT4 port of the SMC logic would be a natural first piece.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples of my MQL work.
 Best regards,
 Oseni Ibrahim
@@ -8286,7 +8264,6 @@
 I came across your mt5-trade-gateway repository, the order validation layer that blocks over-trading, invalid entries and trades around news events, with custom setups available on request.
 Custom setups usually mean new rule types, broker quirks and news-filter changes for each client. I'm an MQL4/MQL5 developer and could help with that side as a subcontractor, for example adding client-specific rules, building an MT4 version for traders still on MT4 accounts, or wiring alerts to Telegram when a trade is blocked.
 I'm happy to work under NDA since the code is proprietary.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples of similar risk tools.
 Best regards,
 Oseni Ibrahim
@@ -8365,7 +8342,6 @@
           <t>Hi Rafał,
 I came across your blessing-ea-optimizer repository. Optimizing all 134 Blessing EA parameters with Bayesian and genetic search on M1 tick data, then exporting .set files for MT4 and MT5, is a serious piece of work.
 You mention you're a domain expert rather than a traditional programmer, so I thought the MetaTrader side might be where some help is useful. I'm an MQL4/MQL5 developer and could, for example, automate Strategy Tester runs to validate your .set files, add logging to the EA so live results can be compared with your optimizer, or trim Blessing's logic into a cleaner EA based on what your tests show matters.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -8444,7 +8420,6 @@
           <t>Hi Simon,
 I came across the Botara 3.0 repository, with the Fisher Transform, RSI, volume oscillator and ATR logic, and saw that you mention MT4 and MT5 availability and offer custom bot development.
 Since most of the project is Python, I thought the MetaTrader builds might be where extra help is useful. I'm an MQL4/MQL5 developer and could implement or maintain the Botara logic as native Expert Advisors, keep the MT4 and MT5 versions matching your Python signals, and take on MetaTrader-specific requests from your clients as a subcontractor.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how I'd structure the EA?
 Best regards,
 Oseni Ibrahim
@@ -8519,7 +8494,6 @@
 I came across the AKG ALGO website repository and saw the range of MT4/MT5 robots you sell, from the entry license to the higher tiers, along with MQL source code access and a marketplace of EAs and indicators.
 Selling on both platforms means every robot needs two builds that behave the same way, and each MetaTrader update or broker quirk can create support work. I'm an MQL4/MQL5 developer and could help keep the MT4 and MT5 versions in sync, fix issues buyers report, add Telegram alerts or risk controls, or build new products for the marketplace.
 I'd be glad to start with one robot so you can judge the quality.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -8603,7 +8577,6 @@
           <t>Hi Mizhar,
 I came across your GitHub profile and the Forex Trading EA Scripts project, the MetaTrader 4 Expert Advisors with strategy logic, risk controls and backtesting.
 With your CTO role at Finovation Technologies and a long list of fintech and enterprise projects, I imagine the trading work gets less time than it deserves. I'm an MQL4/MQL5 developer and could help as a subcontractor: maintaining the MT4 EAs, porting them to MT5 so they run on newer broker and prop firm accounts, or handling MetaTrader requests from Finovation clients.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples of my MQL work.
 Best regards,
 Oseni Ibrahim
@@ -8687,7 +8660,6 @@
           <t>Hi Sage,
 I came across your GitHub profile and saw that you offer MetaTrader 4/5 Expert Advisor development that is spec-driven, backtested and walk-forward tested.
 That is the same kind of work I do. I'm an MQL4/MQL5 developer focused on building and fixing EAs, MT4-to-MT5 conversions, TradingView-to-MT5 ports and Telegram integrations. When client projects stack up or a job needs a second pair of hands, it can help to have someone reliable to share the load, and I'd be happy to work that way with you, either under your name or as a referral partner for jobs you can't take.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -8772,7 +8744,6 @@
 I came across your UT-Bot-Trading-System repository, with the UT Bot Alerts indicator and the UT Bot Phase EA, and noticed that most of your products, like the Multi-Symbol Trend Pullback EA and the RSI scanner, are built for MT4.
 A growing share of buyers now trade on MT5-only brokers and prop firms, so MT5 versions could open the products to more people. I'm an MQL4/MQL5 developer and could port the UT Bot tools to MQL5 while keeping the same inputs and signals, then check that both versions match in the Strategy Tester.
 I could also help when custom development requests come in faster than you can handle them.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of an MT4-to-MT5 port?
 Best regards,
 Oseni Ibrahim
@@ -8856,7 +8827,6 @@
           <t>Hi Abdiwahab,
 I came across your GitHub profile and saw that you build custom trading infrastructure for brokers, prop firms and serious traders, covering Expert Advisors, copy trading, APIs and Web3 integrations.
 Work like that often has an MQL-heavy part, such as EAs, copier endpoints inside MT4/MT5 or bridges to external APIs, that can hold up the rest of a project. I'm an MQL4/MQL5 developer focused on exactly those pieces, and I'd be glad to take them on as a subcontractor under NDA so you can stay on architecture and client work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples of my EA and bridge work.
 Best regards,
 Oseni Ibrahim
@@ -8935,7 +8905,6 @@
           <t>Hi Josias,
 I came across your profile and the Trade Pulse Technologies project, the automated forex EA platform with MT4/MT5 bots and Paystack and PayPal payments.
 A platform like this needs the MetaTrader side to be dependable: EAs that behave the same on MT4 and MT5, handle broker differences and report cleanly back to your cloud backend. Since you're also building AI, fleet and e-commerce projects, I thought extra MQL help might be useful. I'm an MQL4/MQL5 developer and could build or maintain the bots, add risk controls or Telegram notifications, and test them across brokers.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -9020,7 +8989,6 @@
 I came across your Custom-Indicators-MQL4 repository, with the RSI tools, trend validation, position sizing and correlation indicators that thousands of traders have downloaded on MQL5.com.
 They are written for MetaTrader 4, and many traders now use MT5 only, which limits who can use them on the Market. I'm an MQL4/MQL5 developer and could port your indicators to MQL5 with the same inputs, buffers and alerts, so you can publish MT5 versions alongside the originals.
 I could also take overflow work from your Fiverr or MQL5 freelance clients when you're busy.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of your indicators ported to MT5?
 Best regards,
 Oseni Ibrahim
@@ -9099,7 +9067,6 @@
           <t>Hi Vadim,
 I came across the TradingForge Terminal releases repository. Transpiling MQL4 Expert Advisors to C# so they can run on Binance Futures and other venues is an interesting approach, and I saw that MQL5 support is on the roadmap.
 MQL5 brings a different order model, handles for indicators and many small behaviour differences, so a solid set of reference EAs and test cases makes that step much easier. I'm an MQL4/MQL5 developer and could write MQL5 test EAs that cover those edge cases, compare their results in MetaTrader against your transpiled output, and help users port MQL4 strategies that don't transpile cleanly.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful? I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -9174,7 +9141,6 @@
 I came across your trading-bot-demo repository with demo versions of your Expert Advisors and indicators for MT4, MT5 and cTrader, and the full versions available for purchase.
 Selling the same tools on three platforms means every update has to be repeated and tested several times. I'm an MQL4/MQL5 developer and could take the MetaTrader side off your plate: keeping MT4 and MT5 builds in sync, fixing issues that buyers report, adding features such as Telegram alerts or extra risk settings, or building new products from your ideas.
 I'd be happy to begin with a single EA so you can see how I work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a few examples?
 Best regards,
 Oseni Ibrahim
@@ -9248,7 +9214,6 @@
           <t>Hi Helmsman Trade Manager team,
 I came across the helmsman-guide repository for Helmsman Trade Manager. A free trade panel for both MT4 and MT5, with no activation, no account limit and a 64-page user guide, is a generous piece of work.
 Keeping a panel like that working on two platforms, and answering feature requests from users, takes a lot of time. I'm an MQL4/MQL5 developer and could help maintain the MT4 and MT5 builds, fix bugs that users report, or build add-ons such as Telegram alerts or prop firm drawdown limits if you ever plan a paid edition.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples of panels and EAs I've worked on.
 Best regards,
 Oseni Ibrahim
@@ -9327,7 +9292,6 @@
           <t>Hi Viktor,
 I came across your GitHub profile and your background founding Forex Trader s.r.o. and RV-FX s.r.o., along with the custom bot architecture and MQL4/MQL5 Expert Advisor work you offer.
 When the architecture is yours, the MQL implementation, testing across brokers and MT4-to-MT5 ports can become the slow part of a project. I'm an MQL4/MQL5 developer who focuses on exactly that, and I'd be glad to act as a subcontractor under NDA, following your specifications and code standards.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short code sample first.
 Best regards,
 Oseni Ibrahim
@@ -9402,7 +9366,6 @@
 I came across your portfolio repository and the Swing Breakout V2.0 indicator you sell for TradingView through lynk.id.
 Many forex traders do their charting and execution in MetaTrader, so an MT4 or MT5 version of the indicator could reach buyers who don't use TradingView. I'm an MQL4/MQL5 developer and regularly convert Pine Script tools into MetaTrader indicators, keeping the same signals and alerts, and can also turn them into an EA if you want automated entries.
 I'd verify the MetaTrader output against your TradingView version bar by bar before handing it over.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of a Pine-to-MT5 conversion?
 Best regards,
 Oseni Ibrahim
@@ -9481,7 +9444,6 @@
           <t>Hi AlphaTRADER team,
 I noticed you publish both FuturePivots4 and FuturePivots5, along with FutureTargetsLite and AlphaRSI for MT5, plus an mt5linux setup behind your platform.
 Keeping MT4 and MT5 versions of the same indicator in step usually means every fix is done twice, and users of each platform tend to ask for alerts or an EA that trades the levels. I'm a trading bot developer who works in MQL4 and MQL5, and I could take on part of that maintenance: syncing both versions, adding alert and push notification options, or building a small EA wrapper around the pivot and target levels.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds helpful, I can send over a short example of how I would structure it.
 Best regards,
 Oseni Ibrahim
@@ -9560,7 +9522,6 @@
           <t>Hi Rodrigo,
 I came across LadinoBot, your open-source MQL5 robot, and saw it has passed 200 stars. The README's stop options (fixed, by candle and others) show how much thought went into the trade management.
 Projects like this tend to collect issues as MT5 builds and broker settings change, and forks often ask for features such as Telegram alerts or daily loss limits. I'm a trading bot developer working in MQL5, and I could help keep LadinoBot compiling cleanly on current builds, review open issues, or add a risk module if you want to extend it.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be helpful, I can send over a short example of similar maintenance work.
 Best regards,
 Oseni Ibrahim
@@ -9639,7 +9600,6 @@
           <t>Hi Moein,
 I noticed MetatraderMCP, which indexes 4,853 MQL4/MQL5 documentation entries, sitting next to PineMCP on your profile. Tooling that bridges TradingView and MetaTrader like that usually means you get requests to move strategies from one platform to the other.
 I'm a trading bot developer focused on MQL4/MQL5. Most of my work is Pine Script to MT5 conversions, MT4 to MT5 ports and EA fixes. If Fractalyst takes on client projects where the MetaTrader side is the bottleneck, I'd be happy to act as subcontract capacity, working to your specs and under your name if you prefer.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent a short sample, for example a small Pine strategy rebuilt as an MQL5 EA, so you can check the code quality first?
 Best regards,
 Oseni Ibrahim
@@ -9709,7 +9669,6 @@
 I saw your MT4 Python machine-learning trading bot deployment repo on GitHub. It's clear you're packaging MetaTrader automation for clients.
 In projects like that the Python and ML side usually goes smoothly, and the time goes into the MQL part: the bridge EA, order handling edge cases per broker, and clients who then ask for the same bot on MT5. That's where I work. I'm a trading bot developer handling MQL4/MQL5 EAs, MT4 to MT5 conversions and broker or Telegram integrations.
 If you ever need overflow capacity on the MetaTrader side, I'm happy to work white-label under your delivery process, with clear scopes and handover notes.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can also send over a few short code examples first.
 Best regards,
 Oseni Ibrahim
@@ -9789,7 +9748,6 @@
 I came across tradepostpro. It's a clever way to turn daily MT4/MT5 results into posts across X, Threads, Instagram and the other platforms. I saw that MT4 data comes in through an MQL4 EA writing CSV files, while MT5 goes through the Python API.
 Keeping those two paths consistent is usually where the small problems show up: different history fields, time zones or closed-trade detection. I'm a trading bot developer working in MQL4/MQL5, and I can write a matching MQL5 exporter EA, or tighten up the MQL4 one, so both terminals produce the same CSV format for your pipeline.
 If this is something you're working on, I can send over a short example exporter so you can check whether the output fits tradepostpro.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -9863,7 +9821,6 @@
           <t>Hi Bertin,
 I read the bbstrader README, especially the part on overcoming the MQL5 bottleneck with the C++/Python bridge to MetaTrader 5.
 Even with that approach, some users still want native pieces inside the terminal: an EA that mirrors a bbstrader strategy for the MT5 tester, custom indicators ported to MQL5, or a bridge EA for brokers where the Python API is not an option. That is the kind of MQL5 work I do as a trading bot developer.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you get requests like that from bbstrader users or clients, I could take them on as a subcontractor. Would it be useful if I sent a short example first?
 Best regards,
 Oseni Ibrahim
@@ -9937,7 +9894,6 @@
           <t>Hi Deco,
 I came across MT5 Strategy Analyzer and the feature that detects grid, scalping and other styles from a trader's history, then translates strategies between frameworks.
 When the target is MetaTrader 5, the translated strategy has to become a working MQL5 Expert Advisor, and that is where edge cases pile up: order filling modes, grid recovery logic, spread filters. I build MQL5 EAs and could help review generated code, or build the EA for your fintech clients once the analyzer has identified the strategy.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -10011,7 +9967,6 @@
           <t>Hi Umek,
 I came across QuantumBotX, the Windows-first MT5 bot and backtesting platform, and noticed the note that it is actively maintained but built in spare time.
 If the list of MetaTrader-side work is growing faster than your free hours, I could help. I build MQL5 Expert Advisors, and could write native EA versions of QuantumBotX strategies so users can run them on a VPS or in the MT5 Strategy Tester, or help with execution and deployment issues users report.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would take some load off, I can send a short example first. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -10090,7 +10045,6 @@
           <t>Hi Raphael,
 I came across your GitHub profile and Trady.chat, the trading assistant with a psychological focus, and saw that MQL5 Expert Advisors sit in your stack next to n8n, WebSockets and the OpenAI API.
 An assistant like that becomes much more useful when it can see what the trader actually did. I'm a MetaTrader developer and could build a small MT5 EA that streams positions, closed trades and account equity to Trady.chat over WebSockets or HTTP, so the assistant can comment on real behaviour such as revenge trading or oversizing, without asking users to log trades by hand.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, would it be useful if I sent over a short example of the MT5 side?
 Best regards,
 Oseni Ibrahim
@@ -10164,7 +10118,6 @@
           <t>Hi ByTamerFX team,
 I came across the ByTamerFX Pro showcase and read through the changelog. The pace of EA releases is impressive, and I noticed one entry where the server EA had stopped writing to the bytamer.com MT5 state endpoint until the URL was forced at init.
 I'm an MQL4/MQL5 developer, and links like that between an EA, a web API, a desktop terminal and a mobile app are the kind of plumbing I work on regularly: heartbeat checks, retry and queueing when the endpoint is unreachable, and alerts when data goes stale. If extra MQL5 capacity would help, whether for that layer, regression testing between releases or new EA modules, I would be glad to support your work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of a heartbeat and retry pattern?
 Best regards,
 Oseni Ibrahim
@@ -10238,7 +10191,6 @@
           <t>Hi Lachlan,
 I came across MicroQuant and liked the 'Micro Quant' idea behind it: a repeatable logic stack that pulls MT5 OHLC into PostgreSQL and adds AI, technical and news context before any decision is made.
 I'm an MQL4/MQL5 developer. If you're planning to let MicroQuant act on its trade plans, a small MQL5 EA is a reliable way to do it: it can read approved decisions from your WebSocket or database, apply position sizing and hard stops inside the terminal, and report fills back. I could build that and help with a stable VPS setup for the MT5 side, keeping to your existing stack.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that decision-to-EA handoff?
 Best regards,
 Oseni Ibrahim
@@ -10307,7 +10259,6 @@
           <t>Hi Nodalytics team,
 I came across nodalytics/metatrader-terminal and liked how clearly the README explains the reverse SSH tunnel and the WebSocket stream that pushes only the differences, since MT5 has no push API of its own.
 I'm an MQL4/MQL5 developer working on the MetaTrader side of setups like this: EAs and services that feed an external API, execution and risk modules, and keeping terminal bridges stable across builds and broker changes. If your team ever needs extra hands on the MT5 layer, such as an EA-side event publisher to complement the polling loop or help maintaining the container as you add accounts, I could take that on as a contractor.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is useful, I can send over a short example of an MQL5 event publisher.
 Best regards,
 Oseni Ibrahim
@@ -10376,7 +10327,6 @@
           <t>Hi Trade Vectors team,
 I came across your trading-strategy-templates-python repo and noticed that alongside the NSE/BSE and IBKR work, Trade Vectors lists MetaTrader broker integration and an MQL5 + Python bridge for MT5 forex and CFD clients.
 I'm a trading bot developer specialising in MQL4/MQL5. Agencies covering many markets sometimes prefer to hand the MetaTrader-specific parts to someone who works in MQL every day, so I wanted to offer myself as white-label capacity: Expert Advisors built from client specs, MQL5 sides of Python bridges, MT4 to MT5 conversions and fixes to existing EAs. You would keep the client relationship and I would deliver documented source code.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you'd consider, I can send over a few examples of recent MQL5 work.
 Best regards,
 Oseni Ibrahim
@@ -10450,7 +10400,6 @@
           <t>Hi Kipli team,
 I came across ProChart XAUUSD on GitHub, the FastAPI and MT5 chart app that alerts when gold nears Fibonacci entry areas, and saw that you offer custom versions, broker integrations and dashboards.
 Custom client requests like that often need work inside MetaTrader: an EA that places the trade when a Fibonacci zone triggers, a lighter MQL5 data feed instead of the Python MT5 package, or MT4 support for clients on older brokers. I'm a trading bot developer working in MQL4/MQL5, and I could take on that MetaTrader side for your custom projects.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can share examples first.
 Best regards,
 Oseni Ibrahim
@@ -10519,7 +10468,6 @@
           <t>Hi Copiix team,
 I came across the Copiix GitHub organization and saw that the copier handles MT4, MT5 and cTrader in any combination, free and without registration. Keeping MT4 and MT5 EAs in step across terminal updates and broker symbol differences is steady work, especially when every user is on a different setup.
 I'm an MQL4/MQL5 developer and could take on part of that load: fixing edge cases reported by users, adding features such as symbol mapping or lot rules, or reviewing the copier EAs for stability on both platforms. I work async and can start on a single small ticket so you can judge the fit.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of similar copier work?
 Best regards,
 Oseni Ibrahim
@@ -10593,7 +10541,6 @@
           <t>Hi Fintechee team,
 I noticed in the FiSDK README that Fintechee.io lets vendors sell C/C++/MQL-based EAs and indicators, and that Expert-Advisor-Studio runs EAs directly in the browser. That mix usually means someone has to translate MetaTrader logic into your runtime, or the other way around, for customers and white-label partners.
 I build and convert MT4/MT5 Expert Advisors and indicators, and I could help with ports from MQL4/MQL5 into your EA format, or with MetaTrader versions of strategies built in your studio. I can also handle smaller jobs such as indicator rewrites for your marketplace sellers.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -10662,7 +10609,6 @@
           <t>Hi Fivitech team,
 I came across fivitech-mt5-connector on PyPI, with its MT5Pool for connecting to and managing several MetaTrader 5 servers through manager and API credentials. That suggests you work close to brokers running their own MT5 infrastructure.
 Those clients often need terminal-side pieces too: expert advisors, custom indicators, equity-protection or risk tools for traders, or MT4-to-MT5 conversions of legacy code. I'm an MQL4/MQL5 developer and could act as extra capacity for that part of your projects, working to your specs and handing over clean, documented source.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you ever have MQL work queued up behind the server-side tasks, would you be open to me sending a few relevant examples?
 Best regards,
 Oseni Ibrahim
@@ -10731,7 +10677,6 @@
           <t>Hi MetaRPC team,
 I saw that you publish MetaRpcMT4 and MetaRpcMT5, gRPC Python clients for MetaTrader, and that both got fresh releases this week. Supporting two terminal generations in parallel is no small job.
 I'm an MQL4/MQL5 developer. For a gateway like yours, I could help with reference strategies built on your SDK for the documentation, test EAs that check order and position behaviour against the gRPC results, or porting client-side tools between MT4 and MT5. I'm happy to work as outside capacity under your specs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a couple of examples of related MetaTrader integration work.
 Best regards,
 Oseni Ibrahim
@@ -10800,7 +10745,6 @@
           <t>Hi LuxAlgo team,
 I came across @luxalgo/journal-importers on npm and saw that the new trade journal can import MetaTrader HTML statements. That tells me a good part of your users trade on MT4 and MT5.
 Statement imports are manual by nature. I'm an MQL4/MQL5 developer and could build a small MetaTrader EA that sends closed trades to the journal automatically, including screenshots, magic numbers and comments, so MT users get the same experience as API-connected brokers. I also port TradingView-style tools to MQL5 if that ever comes up.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the sync EA?
 Best regards,
 Oseni Ibrahim
@@ -10879,7 +10823,6 @@
           <t>Hi Simon,
 I came across the mt5-mcp-server package on npm, published under the afx-markets GitHub organisation, which gives AI assistants access to MetaTrader 5 symbol and trading data.
 If it's heading toward client-facing use, some features are easier from inside the terminal. Examples are an EA that enforces account-level risk rules whatever the assistant requests, streaming of trade events, or exporting custom indicator values. I'm an MQL4/MQL5 developer and could build those pieces or support the MetaTrader side generally, working to your specs and handing over documented source.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example?
 Best regards,
 Oseni Ibrahim
@@ -10953,7 +10896,6 @@
           <t>Hi FxSocket team,
 I came across the @fxsocket/sdk package, your typed Node.js client for MT4 and MT5 account management, trading and streaming, with automatic reconnect and subscription replay.
 API customers often come back with needs the API doesn't cover: a custom EA running beside their integration, indicator values the platform doesn't expose, or MT4 code that has to move to MT5. I'm an MQL4/MQL5 developer and could be the partner you point those requests to, or write example EAs that show FxSocket and in-terminal code working together.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's useful, I can send over a few examples of my work.
 Best regards,
 Oseni Ibrahim
@@ -11022,7 +10964,6 @@
           <t>Hi XBTFX team,
 I came across @xbtfx/mcp-trading, the MCP server that lets Claude, Codex and Cursor trade XBTFX MetaTrader 5 accounts through your Trading API.
 Traders coming in through AI agents often still want something running in the terminal itself. That could be an EA that enforces their own risk limits, trade management that runs while the agent is offline, or indicators that show what the agent did on the chart. I'm an MQL4/MQL5 developer and could build such tools for your clients or example EAs for the API documentation.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds relevant, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -11091,7 +11032,6 @@
           <t>Hi Yuants team,
 I came across @yuants/vendor-mt4 on npm, the MetaTrader 4 connector for the Yuants trading system.
 MT4 connectors usually depend on an MQL4 bridge running in the terminal, and many brokers now only open new accounts on MT5. I'm an MQL4/MQL5 developer and could help maintain the MT4 bridge side or build an MT5 equivalent with the same message format, so a vendor-mt5 package would need few changes in your TypeScript code. The EA would handle reconnection and report account state regularly.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's on your list, I can send over a short example of an MT5 bridge EA.
 Best regards,
 Oseni Ibrahim
@@ -11160,7 +11100,6 @@
           <t>Hi OrvaLabs team,
 I noticed orva-mt5-bridge, the MQL5 bridge that pushes MetaTrader 5 market data over HTTP and TCP into the Orva platform.
 Bridges like this usually work well in testing and then meet dropped connections, terminal restarts and brokers with odd symbol names once they run all day. I'm a trading bot developer working in MQL5, and I could help with reconnect and buffering logic, symbol mapping, or adding order execution endpoints so the AI side can act on its signals through the same bridge.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how I would handle reconnects in MQL5?
 Best regards,
 Oseni Ibrahim
@@ -11234,7 +11173,6 @@
           <t>Hi Cesar,
 I came across mql5-execution-components and your Castle Trade LLC profile, including the asynchronous execution framework work.
 Since you take contract work through Upwork, I thought it worth reaching out. I'm a trading bot developer working in MQL4/MQL5, mainly on EA fixes, MT4 to MT5 conversion, Telegram integration and trade copiers. When client work on the MetaTrader side piles up, I could take on defined pieces such as ports, broker compatibility fixes or testing harnesses so you can stay focused on the architecture.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of my MQL5 code?
 Best regards,
 Oseni Ibrahim
@@ -11313,7 +11251,6 @@
           <t>Hi Hossein,
 I came across WealthPole-Architecture-Demo, the modular MQL5 EA starter from Fintor AI, and the trend and risk engines you describe on your profile.
 Modular EA designs pay off, but every new engine still needs its inputs, tests and broker edge cases handled. I'm a trading bot developer working in MQL4/MQL5, and I could help build or test specific modules, for example the daily drawdown guard, exposure control, or a Telegram reporting layer, following the structure and naming you've already set up in the demo.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -11387,7 +11324,6 @@
           <t>Hi Sergei,
 I came across FinCore and XTradeServer, and noticed the README invites people to write about improvements, installation and support for a secured version.
 Both projects lean on MetaTrader 5 connectivity, and that part tends to need attention as MT5 builds and brokers change. I'm a trading bot developer working in MQL4/MQL5, and I could help on the MetaTrader side: the EA or script that reports deals and positions into FinCore, terminal management for XTradeServer, or updating older MQL code so it compiles cleanly on current builds.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example of similar work.
 Best regards,
 Oseni Ibrahim
@@ -11461,7 +11397,6 @@
           <t>Hi Pedro,
 I came across horizon5-mt, your MetaTrader framework with portfolio optimization, and it looks like a serious piece of engineering rather than a one-off EA.
 Frameworks like this usually reach a point where the core is solid but there's a backlog of strategy modules, reporting and small integrations to add. I'm a trading bot developer working in MQL4/MQL5, and I could help with that backlog, for example writing new strategy components against your interfaces, adding Telegram notifications for fills and drawdown, or building backtest export scripts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of similar work?
 Best regards,
 Oseni Ibrahim
@@ -11540,7 +11475,6 @@
           <t>Hi Nawfal,
 I came across mq5_skills, your AI skill for producing production-ready MT5 Expert Advisors, and the MT_MANAGER account tool alongside it.
 The quality of generated EAs depends heavily on the examples and rules the skill draws on, especially around order filling modes, stop levels and error handling that trip up new EAs. I'm a trading bot developer who writes MQL4/MQL5 daily, and I could contribute reviewed reference EAs and checklists, or help extend MT_MANAGER with risk limits and alerts. Everything would be written to match your conventions.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -11619,7 +11553,6 @@
           <t>Hi Ali,
 I came across metatrader-mcp and the Phoenix platform on your profile, the 21-service automated trading setup that includes MQL5 components.
 In platforms like that, the MetaTrader piece is often the one that needs the most care: terminals that disconnect, symbols that differ by broker, and EAs that must report state back cleanly. I'm a trading bot developer working in MQL4/MQL5, and I could help with the MT5 side, for example extending metatrader-mcp with order and position endpoints or hardening the EA that feeds Phoenix so it recovers cleanly after terminal restarts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -11698,7 +11631,6 @@
           <t>Hi Hemang,
 I came across Algotrading_Multi_account_Modern_UI, the web control panel for running trades across multiple accounts, and noticed it's tagged for MQL5.
 Multi-account tools get much more useful when MetaTrader 5 accounts can be driven the same way as the others, which usually means a small EA or bridge on each terminal that accepts commands and reports positions back. I'm a trading bot developer working in MQL4/MQL5, and I could build that connector, including reconnect handling, per-account risk limits and a simple status report your UI can display.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short outline of how I'd approach it?
 Best regards,
 Oseni Ibrahim
@@ -11777,7 +11709,6 @@
           <t>Hi Max,
 I came across mt5-device-fingerprint-tool and the MT-Indicator-Locker projects, which generate SHA-256 license codes to protect MT5 indicators.
 Vendors who try tools like these usually need help on the MQL5 side: wiring the license check into an existing EA or indicator without breaking it, handling offline cases and giving clear messages when a key fails. I'm a trading bot developer working in MQL4/MQL5, and I could write ready-to-use MQL5 include files and example integrations to sit alongside your tools, so vendors can adopt them in an afternoon rather than a week.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -11851,7 +11782,6 @@
           <t>Hi Tibor,
 I came across TradeForge, your Python framework for MetaTrader 5 with the live engine, Optuna optimisation and Telegram control.
 Python-driven MT5 setups often benefit from a small MQL5 companion running in the terminal, one that draws signals and levels on the chart and acts as a last safety check on order size and daily loss if the Python side misbehaves. I'm a trading bot developer working in MQL4/MQL5, and I could build that companion to fit TradeForge's config format and read the same parameters your optimiser produces.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -11920,7 +11850,6 @@
           <t>Hi Daedalus team,
 I came across your MetaTrader tools, advance-trade-management, GriffinATM and Lynxguard, the checker that compares tick data across brokers.
 Trade managers get a steady stream of requests once people use them: partial closes, basket breakeven, prop-firm daily limits, and fixes when a broker uses unusual stop levels. I'm a trading bot developer working in MQL4/MQL5, and I could help with those additions or with an MT4 version if your users ask for one. I'm used to working inside someone else's code without changing its style.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples of trade management code I've written.
 Best regards,
 Oseni Ibrahim
@@ -11994,7 +11923,6 @@
           <t>Hi Joao Pedro,
 I came across Connexus, your MQL5 HTTP library, and Logify for logging. Both solve problems I run into on almost every EA project.
 The most common things people build on top of an HTTP library in MQL5 are Telegram notifications, TradingView webhook receivers and small REST dashboards. I'm a trading bot developer working in MQL4/MQL5, and I'd be glad to contribute worked examples of those using Connexus, or help with client projects that need this kind of integration if you take on freelance work and want a hand with the MetaTrader side.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12073,7 +12001,6 @@
           <t>Hi Artem,
 I came across mt5-cloud-level-alerts, the service that syncs MT5 chart levels to the cloud and sends Telegram alerts.
 The MetaTrader client is usually the tricky part of a tool like this: catching every object change, surviving terminal restarts and WebRequest limits, and supporting MT4 users who ask for the same thing. I'm a trading bot developer working in MQL4/MQL5, and I could help with that client side, including an MT4 port, so you can keep your focus on the service and front end. I'd document the client so it is easy to maintain later.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -12147,7 +12074,6 @@
           <t>Hi LoanXfer team,
 I came across mt5-risk-reward-tool and mt5-economic-calendar, and saw on your profile that you take freelance work on trading bots and exchange backends.
 Clients who start on exchange bots often come back asking for the same logic in MetaTrader, and MQL has enough quirks that it can eat time. I'm a trading bot developer focused on MQL4/MQL5, and I could take on the MetaTrader pieces of your projects, such as EAs, trade copiers or TradingView to MT5 bridges, while you handle the backend work. I can work under your name and hand over documented source.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -12221,7 +12147,6 @@
           <t>Hi Sebastian,
 I came across your MT5 tools, especially mt5-panel-maestro with the kill switch and mt5-telegram-assistant for drawdown alerts.
 We seem to work on very similar things. I'm a trading bot developer working in MQL4/MQL5, mostly on EA fixes, Telegram integration, trade copiers and risk management. Freelance demand is rarely even, so I'm reaching out to suggest sharing overflow work: if you have a client project that needs an extra pair of hands, or an MT4 version of one of your tools, I could help, and I'd be glad to send work your way too.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -12295,7 +12220,6 @@
           <t>Hi Dewyndl team,
 I came across metatrader-automation-scripts-toolkit, with the trailing stop and grid EAs, and saw from your profile that you offer backend and integration services to clients in Europe and the CIS.
 When clients ask for MetaTrader work it is often more than a script: a full EA, a copier between accounts, or a bridge from TradingView. I'm a trading bot developer focused on MQL4/MQL5, and I could handle that side of your projects as a subcontractor while you keep the backend and API work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of my MQL5 code?
 Best regards,
 Oseni Ibrahim
@@ -12369,7 +12293,6 @@
           <t>Hi Khaleq,
 I came across your ICT_indicator repository and liked the closed-bar-only rule, where signals are only finalised after right-side confirmation. That is the part many SMC tools get wrong.
 Indicators with that much logic usually lead users to ask for two things: alerts they can trust and an EA that trades the signals with proper risk controls. I'm a trading bot developer working in MQL4/MQL5, and I could build an EA wrapper that reads the indicator buffers, adds position sizing and daily loss limits, and sends Telegram alerts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12443,7 +12366,6 @@
           <t>Hi Ali,
 I came across your MQL5 Programming for Traders course repository, the introduction to building trading robots and Expert Advisors in MQL5.
 Students of courses like this usually get stuck at the step after the basics: adding real risk management, sending alerts to Telegram, or converting an old MT4 indicator they already use. I'm a trading bot developer working in MQL4/MQL5, and I could prepare a few worked example EAs on those topics, or review student code if you run cohorts, to sit alongside your lessons.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful? I can send over a sample first.
 Best regards,
 Oseni Ibrahim
@@ -12517,7 +12439,6 @@
           <t>Hi Handiko,
 I came across Trading-Strategy-Development-Example and Improvement-to-an-existing-strategy, and liked how you walk through improving a strategy step by step instead of just posting final code.
 I'm a trading bot developer working in MQL4/MQL5, and your approach is close to how I handle client work. If you take on strategy projects or want help turning research into production EAs with proper risk handling, Telegram alerts and VPS deployment, I could help as a collaborator or subcontractor on the MetaTrader side.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of my code first.
 Best regards,
 Oseni Ibrahim
@@ -12596,7 +12517,6 @@
           <t>Hi Saymon,
 I came across mcp-metaeditor, your MCP server that runs MetaTrader 5's MetaEditor under Linux and Wine. Compiling MQL5 from outside Windows is something a lot of developers want.
 Tools like this get tested hardest on messy real projects: many include files, resources, DLL imports and strategy tester runs. I'm a trading bot developer working in MQL4/MQL5, and I could put mcp-metaeditor through its paces on real multi-file EAs, report where it breaks, and contribute test fixtures, or help your users with EA work if they ask.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example project to start with.
 Best regards,
 Oseni Ibrahim
@@ -12665,7 +12585,6 @@
           <t>Hi AtingMQL5 team,
 I came across AtingMQL5 and liked the automatic filling mode selection, since the wrong filling mode is one of the most common reasons an EA fails on a new broker.
 Libraries like this spread faster when there are complete example EAs showing the classes working together. I'm a trading bot developer working in MQL4/MQL5, and I could contribute a couple of example EAs built on AtingMQL5, for instance a session breakout using LimitsByTimeRange with CSV-filtered backtests, or help on bot projects if you take client work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -12739,7 +12658,6 @@
           <t>Hi Desmond,
 I came across MT5-EA-Project and saw in the README that you welcome collaboration on the collection, including the Power-Pivot strategy.
 Collections of EAs tend to grow uneven over time, with each one handling lot sizing, trailing and alerts a little differently. I'm a trading bot developer working in MQL4/MQL5, and I could help bring them onto a shared risk and notification module, add Telegram alerts, or write MT4 versions of the ones people ask for. I'd keep each strategy's logic untouched and only standardise the shared parts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -12813,7 +12731,6 @@
           <t>Hi Sajid,
 I came across grid-master-pro-mt5-ea and noticed it has picked up well over a hundred stars, which usually means plenty of people running it on different brokers.
 Grid EAs draw the most requests for protective features: equity stop, maximum open levels, news pauses and prop-firm daily loss rules. I'm a trading bot developer working in MQL4/MQL5, and I could help add those safeguards or handle broker compatibility issues users report, so the project keeps moving while you work on AlHarih's other products and client work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -12887,7 +12804,6 @@
           <t>Hi Duc Duy,
 I came across Algo-Trading-Lab, with the reinforcement learning agents (PPO, SAC, TD3 and others) alongside the indicator-based strategies.
 The step from a trained agent to live trading in MetaTrader is often where projects stall, because it needs a dependable bridge, order validation and account-level limits. I'm a trading bot developer working in MQL4/MQL5, and I could build the MT5 side: an EA that receives the model's actions, checks them against risk rules and reports fills back to Python, so live results can be compared fairly with your backtests.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -12961,7 +12877,6 @@
           <t>Hi Joe,
 I came across MQL5-Bots, with the MACD and RSI strategies, and noticed your TrendBot work on Deriv's Volatility Index.
 Deriv's synthetic indices on MT5 have their own quirks, including large minimum lots, 24/7 sessions and fast spikes, so EAs written for forex often need changes to behave there. I'm a trading bot developer working in MQL4/MQL5, and I could help adapt the bots for synthetics with suitable sizing and a Telegram alert layer, or collaborate on client bots if you take that kind of work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -13035,7 +12950,6 @@
           <t>Hi BigHeroAI team,
 I came across bigheroai-showcase and the BigHeroAI decision system for MetaTrader 5, along with your ICT/SMC Pine indicators.
 Two things usually follow a setup like this: the MQL5 bridge needs to survive disconnects and report state reliably, and users of the Pine indicators ask for MT5 versions. I'm a trading bot developer working in MQL4/MQL5, and I could help with either, hardening the bridge EA or converting the confirmed-bar ICT/SMC indicators to MQL5 with signals that match the TradingView versions bar for bar.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13104,7 +13018,6 @@
           <t>Hi Ishaan,
 I came across mt5-mac-python-bridge. Getting Python to drive MetaTrader 5 on a Mac is something I see traders struggle with often.
 Once the data side works, people usually want to place and manage orders through the same bridge and to know when the terminal has gone quiet. I'm a trading bot developer working in MQL4/MQL5, and I could build an MQL5 EA counterpart that executes orders with proper error codes, enforces basic risk limits and sends a regular heartbeat back to Python.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13183,7 +13096,6 @@
           <t>Hi Leeank,
 I came across Algorithmic-Trading-Bot, the Python bot you run on MetaTrader 5, and saw you're working on Inversiones Bloom.
 Python bots on MT5 usually hit the same practical issues in live use: the terminal disconnects, orders are rejected for broker-specific reasons, and nobody notices until the next morning. I'm a trading bot developer working in MQL4/MQL5, and I could add an MQL5 safety and monitoring layer with Telegram alerts, or help set up a stable VPS deployment for the bot.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -13257,7 +13169,6 @@
           <t>Hi Gilbran,
 I came across mt5-signal-copier-architecture, your Telegram to MT5 copier, and saw on your profile that it runs unattended with your other production services.
 Copiers like this tend to break on the execution side rather than the parsing side: signal edits that should move a stop, multiple take profits, duplicate messages and symbol suffixes that differ by broker. I'm a trading bot developer working in MQL4/MQL5, and I could help harden the MT5 EA for those cases and add a heartbeat so you know it is still trading.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13331,7 +13242,6 @@
           <t>Hi Ahmed,
 I came across forex-news-killer, your MT4 EA that protects accounts around news events.
 Since most brokers and prop firms have moved to MT5, I'd expect people in your Discord and YouTube audience to ask for an MT5 version. MQL5 also has a built-in economic calendar, which removes the need for outside news feeds. I'm a trading bot developer working in MQL4/MQL5, and I could convert the EA to MT5 using that calendar while keeping your existing inputs and behaviour, so current users can switch without relearning the settings.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -13406,7 +13316,6 @@
 I came across pixiu, a Python backtesting tool built around MetaTrader 4 and 5. It's useful for people who don't want to live inside the Strategy Tester.
 A common question from MetaTrader users is whether a strategy backtested outside MT4/MT5 matches what their EA does in the terminal. I'm a trading bot developer working in MQL4/MQL5, and I could write reference EAs that mirror a few pixiu strategies. You could then compare fills, spreads and results against the MT4/MT5 tester and document any differences.
 If this is something you're working on, I can send over a short example, one simple strategy as both a pixiu script and an MQL5 EA, so you can judge whether it's worth doing more.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13481,7 +13390,6 @@
 I came across ubot-mt4, your MetaTrader 4 Expert Advisor. It stood out because of your backend and ML background, which shows in how the bot is laid out.
 Many traders now only get MT5 accounts from brokers and prop firms, so MT4-only EAs are harder to use. I'm a trading bot developer who does MT4 to MT5 conversions: rewriting order logic for MT5 positions and deals, checking indicator handles and validating both versions side by side in the Strategy Tester. I can also add Telegram trade notifications or a drawdown guard if that's useful.
 If you'd like, I can port a small part of ubot-mt4 to MQL5 and send it over as an example.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -13561,7 +13469,6 @@
 I came across your MT4 Manager REST API in ASP.NET Core. Exposing Manager functions over REST is exactly what broker back offices and CRMs ask for.
 Clients who start on MT4 usually ask for the same thing on MT5 soon after, along with terminal-side pieces such as EAs for reporting, risk checks or trade copying that the API alone can't cover. I'm a trading bot developer working in MQL4/MQL5 and MetaTrader integrations. If your .NET work brings in broker projects, I'd be glad to cover the MQL and MT5 parts as a collaborator.
 If this sounds relevant, I can send over a couple of short examples of EA-side components that would sit next to your API.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -13641,7 +13548,6 @@
 I came across your Automatic Setter Expert Advisor for MT4, which deploys up to 150 strategy instances per session. That saves a lot of time for anyone running strategy portfolios, for example from StrategyQuant-style generators.
 The same need exists on MT5, but charts, templates and EA inputs are handled differently there, so the MT4 tool can't just be recompiled. I'm a trading bot developer who works on MT4 to MT5 conversions and deployment tooling. I could build an MQL5 version with the same batch workflow.
 If that sounds interesting, I can send over a short example showing how the attach-and-configure step works on MT5.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -13721,7 +13627,6 @@
 I came across MetatraderSharp and the cookbook. A cleaner C# wrapper around MTsocketAPI for both MT4 and MT5 is useful for .NET developers who don't want to write MQL.
 Sooner or later, library users hit the terminal side: behaviour that differs between MT4 and MT5 accounts, custom indicators they want to read, or small EAs to run alongside the socket connection. I'm a trading bot developer working in MQL4/MQL5 and MetaTrader integrations, and I'd be happy to contribute cookbook examples or help with MQL work around the library.
 If this fits where you're taking the project, I can send over a short example of an MQL5 helper that exposes custom indicator values to a C# client.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13801,7 +13706,6 @@
 I came across AlgoExpertHub and saw that forex execution for MT4/MT5 goes through MetaApi and mtapi.io. That works well for getting started, but per-account cloud fees and an extra dependency tend to add up as subscribers grow.
 One option is a native MQL4/MQL5 receiver EA that polls or listens to your Laravel API and places trades directly in the subscriber's terminal, with lot sizing, symbol mapping and a daily loss limit. I'm a trading bot developer who builds signal executors, trade copiers and Telegram integrations for MetaTrader.
 If this is something you're working on, I can send over a short example of a receiver EA that reads signals from a JSON endpoint.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13876,7 +13780,6 @@
 I came across MT4ForexParser, which turns MetaTrader 4 .hst history into CSV and pandas. It fits nicely with PriceGenerator for strategy testing.
 Most brokers are moving users to MT5, where history is stored differently and is best exported from inside the terminal. I'm a trading bot developer working in MQL4/MQL5. I could write an MQL5 script or EA that exports bars and ticks in the same CSV layout your parser produces, so MT5 data drops straight into your existing pipeline.
 If that would help, I can send over a short example exporter so you can compare its output with an MT4ForexParser file.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -13951,7 +13854,6 @@
 I came across MT4 Position Helper (MT4持仓助手). It looks like you support a real user group through QQ and keep the EA updated.
 As more brokers move clients to MT5, position-management tools like yours are often among the first things traders ask for on the new platform. The MT5 position and order model is different, so a direct recompile doesn't work. I'm a trading bot developer who does MT4 to MT5 conversions, and I could port the helper to MQL5 while keeping the same panel and behaviour your users already know.
 If you're interested, I can send over a short example of one feature, such as batch close or breakeven, running in MQL5.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -14025,7 +13927,6 @@
           <t>Hi Gifari,
 I came across XAUBot AI and liked how the XGBoost model, SMC features and HMM regime detection are combined for XAUUSD on MetaTrader 5. I also saw SURGE-WSI following a similar path.
 Since the logic lives in Python, the terminal only acts on what the bridge sends. I build MQL5 Expert Advisors, and a small companion EA could keep the daily loss limit, session filter and trailing or breakeven rules running inside MT5 even if the Python side disconnects or restarts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits where the project is heading, I can send over a short example of how I usually structure that kind of guard EA. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -14104,7 +14005,6 @@
           <t>Hi Omega,
 I saw StrategyTester5 and the strategytester5.com docs. Bringing a proper backtesting layer to the MetaTrader 5 Python API is something a lot of Python traders have been missing.
 One thing that usually comes up with a tool like this is people wanting ST5 results to line up with the native MT5 Strategy Tester. I work on MQL5 Expert Advisors, and I could write mirror EAs for your example strategies so users can compare fills, order handling and report numbers side by side. I also take on overflow MQL5 work if clients ask you for EA versions of their Python strategies.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent over a small example of such a comparison EA?
 Best regards,
 Oseni Ibrahim
@@ -14183,7 +14083,6 @@
           <t>Hi José,
 I came across mt5-docker-api and your public trade journal at jose.ar. Running MT5 in Docker with VNC and a REST layer, then publishing 5,600+ trades openly, is a solid engineering setup.
 I build MQL5 Expert Advisors, and I thought there might be room for an in-terminal piece next to the container: an EA that handles execution checks, writes trade events in a format your journal can ingest, or enforces risk limits locally when the API is not reachable.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of that overlaps with what you are building next, I can send a short example of how I would structure it. Would you be open to that?
 Best regards,
 Oseni Ibrahim
@@ -14262,7 +14161,6 @@
           <t>Hi Bechara,
 I saw Claude Trader, with its 14 agents covering strategy, entries, capital management and position watching on MetaTrader 5, and TradeAI Gold on your profile.
 With agents deciding trades, it often helps to have a deterministic layer inside the terminal that does not depend on the API session. I develop MQL5 Expert Advisors and could build a compact guard EA that enforces max exposure, daily drawdown and hard stops, and reports state back to your system.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is on your list for the gold bot or client projects, I can send over a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -14341,7 +14239,6 @@
           <t>Hi Fredy,
 I came across mt5-arch-integration and the note that mt5linux/RPyC often hits IPC timeouts under Wine 11, which is why you went with the Mt5ArchBridge.mq5 file bridge.
 That EA ends up carrying the whole integration, so small things like command acknowledgements, retry handling and file locking make a big difference. I write MQL5 Expert Advisors and bridges, and could help extend the bridge with more order types and status reporting, or try a socket-based variant that still behaves under Wine.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are planning more work on it, I can send a short example of how I handle the file protocol side. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -14420,7 +14317,6 @@
           <t>Hi Elkhan,
 I saw ForexAiTrader and liked the principle that Claude proposes and the deterministic risk engine disposes. Routing execution through MetaApi keeps the Node side clean.
 One gap in cloud setups is that the terminal itself does not know the risk rules. I build MQL5 Expert Advisors and could write a small EA that enforces the same hard limits (max lots, daily loss, max open trades) inside MT5, so they hold even if the API link drops. A direct EA bridge is another option if you want to reduce dependence on the cloud service.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent a short example?
 Best regards,
 Oseni Ibrahim
@@ -14499,7 +14395,6 @@
           <t>Hi Amir,
 I came across TradingAgents, with the AI analyst team, the 25-strategy engine and MT5 streaming in one desktop app, and I saw you are also building Traders Royal.
 For a product like this, the MetaTrader side often decides how it feels: tick delivery, order confirmation and how the app recovers after a terminal restart. I build MQL5 Expert Advisors and bridges, and could write an EA that pushes ticks and account events to the app and handles execution requests with proper checks.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -14573,7 +14468,6 @@
           <t>Hi Prabal,
 I saw TradeLens and liked the idea of a calm, read-only companion that shows the risk story of an MT5 trade before the click.
 A natural extension could be an MQL5 panel or indicator that draws the same numbers on the chart itself: risk in money, margin after entry, stop distance compared with ATR. That way traders see it right where they place the order. I build MQL5 indicators and Expert Advisors and could put together that chart-side piece so it reads from the same assumptions.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is interesting, I can send over a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -14652,7 +14546,6 @@
           <t>Hi Kelvin,
 I saw your Deriv MT5 synthetic indices bot. The rules are clearly defined: 4H trend from fractal swings, the 4H order block, a 15M fair value gap entry and a structural target that must clear 1:3.
 Because the rules are so precise, they translate well into a native MQL5 Expert Advisor. That would let the strategy run on a VPS inside MT5, and you could test it in the MT5 Strategy Tester on Deriv's synthetic symbols. I build MQL5 EAs and have worked with this kind of swing and gap logic.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example of how I would structure it?
 Best regards,
 Oseni Ibrahim
@@ -14731,7 +14624,6 @@
           <t>Hi Zorion,
 I read the oas-execute-mcp README. Putting six independent checks and an audit log between a model and a broker order is a careful design, and running it against a live MetaTrader 5 terminal makes the stakes real.
 One layer you might find useful is a guard inside the terminal itself: an MQL5 Expert Advisor that checks every new position against hard limits and closes anything that slipped past, independent of the Python side. I build MQL5 EAs and could write that as a small, auditable component.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your approach, I can send over a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -14810,7 +14702,6 @@
           <t>Hi Thai,
 I came across mt5-python-bridge and the list of silent failure modes in the MetaTrader5 package that you wrote tests for. It is clear it came from running a real XAUUSD and FX system.
 Some of those problems are easier to close from inside the terminal: an MQL5 service or EA can confirm executions through OnTradeTransaction, keep protective stops on the broker side and export deal history with server time. I build MQL5 Expert Advisors and could write a small component that works alongside your bridge.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is useful for the production system, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -14884,7 +14775,6 @@
           <t>Hi Tej,
 I saw smc-ob-scanner, the Python port of the Volumetric Order Block script with a dashboard, CLI and an MQL5 expert advisor on top.
 Keeping Pine, Python and MQL5 versions in agreement is usually the tricky part, especially around how zones are invalidated and how bar indexing differs. I work on TradingView to MT5 conversions and MQL5 Expert Advisors, and could help with parity checks, an MQL5 indicator version that draws the zones on MT5 charts, or forex clients who want the MetaTrader side handled.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -14958,7 +14848,6 @@
           <t>Hi marketprolab team,
 I came across marketprolab and its starting premise: describe the instrument exactly as it appears in the MT5 Specification window and let the simulator behave accordingly.
 Two MQL5 pieces could support that. One is a script that exports symbol specifications (contract size, swap, margin, stops level) straight from the terminal into your format. The other is a set of reference Expert Advisors that run the example strategies in the MT5 Strategy Tester, so users can compare results side by side. I build MQL5 EAs and scripts like these.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -15032,7 +14921,6 @@
           <t>Hi Ezekiel,
 I came across your MT5 momentum trading platform, with the split between control plane and execution plane, the deterministic risk engine and the operator dashboard.
 When a platform like this goes from paper to several live accounts, running a Python terminal link per account gets heavy. An alternative is a lightweight MQL5 Expert Advisor in each terminal that receives instructions from the control plane, applies local checks and reports fills back idempotently. I build MQL5 EAs and bridges of that kind.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are heading toward live multi-account runs, I can send a short example. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -15111,7 +14999,6 @@
           <t>Hi Deepak,
 I came across TradePulse and the master-slave copier built on Redis Streams, including the note that MetaTrader5 only allows one terminal per Python process.
 That constraint is a common reason copier products move the capture and execution parts into MQL5. A master EA can publish trade events the moment they happen, and a slave EA can apply them with lot scaling and symbol mapping, while your Flask and Redis layer keeps the routing. I build MQL5 trade copiers and bridges like this.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are looking at scaling the copier, I can send a short example. Would that help?
 Best regards,
 Oseni Ibrahim
@@ -15190,7 +15077,6 @@
           <t>Hi Hans,
 I came across your XAUUSD scalper that combines CNN, LSTM and self-attention in PyTorch and trades through MetaTrader 5.
 For scalping, the round trip between Python and the terminal can matter. MQL5 can load ONNX models directly, so one option is exporting the network and running inference inside an Expert Advisor, with the EA handling entries, stops and spread filters locally. Another is keeping Python for inference and adding an MQL5 risk layer. I build MQL5 EAs and can help with either.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the ONNX route?
 Best regards,
 Oseni Ibrahim
@@ -15269,7 +15155,6 @@
           <t>Hi Daniel,
 I saw Unit8 and its goal of one strategy codebase across MetaTrader 5 and CCXT exchanges without rewrites.
 The MT5 side usually needs more care than exchanges: filling modes that differ per broker, netting versus hedging accounts, stop level limits and symbol suffixes. I build MQL5 Expert Advisors and bridges, and could help with a small in-terminal EA that handles these details and exposes a clean interface to your adapter, or review the adapter against a few real broker setups.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is useful for the project, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15343,7 +15228,6 @@
           <t>Hi Rahman,
 I came across your Telegram VIP signal auto-trader. Handling Arabic RTL text and invisible characters before parsing is a detail most copiers get wrong.
 On the execution side, an MQL5 Expert Advisor that receives the parsed signal can place orders and manage them natively: multiple take profits with partial closes, moving the stop to breakeven, and processing edits like 'close half' or 'move SL' reliably. I build Telegram-to-MT5 copiers and trade management EAs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want to extend the bot in that direction, I can send a short example. Would that be helpful?
 Best regards,
 Oseni Ibrahim
@@ -15422,7 +15306,6 @@
           <t>Hi Leonardo,
 I saw MT5-Claude, the tool that reads candles and indicators from MetaTrader 5 and asks Claude for signals with key levels and risk management.
 A useful next step could be showing the answer where traders look: an MQL5 indicator that draws the entry, stop, target and key levels on the chart, or an Expert Advisor that places the trade after a confirmation click with lot size calculated from risk. I build MQL5 indicators and EAs and could write that piece so it reads the output your tool already produces.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent a short example?
 Best regards,
 Oseni Ibrahim
@@ -15501,7 +15384,6 @@
           <t>Hi Ishan,
 I came across TradeBridge, the MT5 to MCP bridge with regime detection, ATR sizing, bracket orders and trailing stops, small enough to fit on a 512 MB VPS.
 Trailing stops and brackets are one area where an in-terminal Expert Advisor helps: it reacts on every tick even if the Python services or the agent are busy or restarting. I build MQL5 EAs and could write a compact manager EA that your bridge configures through MCP, while the EA does the tick-level work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits the design, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15580,7 +15462,6 @@
           <t>Hi Alif,
 I came across nautilus_mt5, the MetaTrader 5 adapter for NautilusTrader with both data and execution clients.
 For an execution client, NautilusTrader expects accurate order and fill events, and polling the MT5 Python API can miss partial fills or modifications. An MQL5 Expert Advisor listening to OnTradeTransaction can push those events as they happen, which makes the adapter's state much easier to keep in sync. I build MQL5 EAs and bridges and could write that event feed.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would like to try it, I can send over a short example. Would that be useful?
 Best regards,
 Oseni Ibrahim
@@ -15654,7 +15535,6 @@
           <t>Hi Kevin,
 I came across Tradetropy and its idea that engine differences are just a transport detail behind one Strategy API, with footprint analysis built in.
 For footprint work on MetaTrader 5, the Python package can be limiting on tick flags and market depth. An MQL5 Expert Advisor can subscribe to book events and every tick, then stream them to Tradetropy with low overhead and accept orders back. I build MQL5 EAs and data bridges and could write that transport component.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans for the MT5 side, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15728,7 +15608,6 @@
           <t>Hi Warren,
 I came across your MT5 MCP server that gives Claude access to prices, account state, positions and trade execution in MetaTrader 5.
 Two MQL5 additions could make it more useful. One is an EA that exposes values from custom indicators, which the Python package cannot read directly, so Claude can reason on the same signals a trader sees. The other is an in-terminal guard that caps risk on anything the assistant opens. I build MQL5 Expert Advisors and indicators.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either sounds interesting, I can send a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15807,7 +15686,6 @@
           <t>Hi Ruei-Ci,
 I came across Chip Whisperer, which computes volume profile levels such as POC and value area from MT5 data and answers questions through Claude and Telegram.
 It would be natural for traders to see those same levels on the MetaTrader chart. I build MQL5 indicators and Expert Advisors and could write a volume profile indicator that matches your calculation, draws the levels, and raises alerts when price reaches them, so the Telegram answers and the chart stay consistent.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that is interesting, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -15886,7 +15764,6 @@
           <t>Hi Agustin,
 I came across mt5-backtesting-toolkit and the way it separates experiment definitions from terminal details, with a fake runner for deterministic tests.
 The step from the fake runner to real terminals usually needs a couple of MQL5 pieces: an example EA whose inputs match your experiment schema, and OnTester or frame export code that writes results in a format your parser expects instead of scraping HTML reports. I build MQL5 Expert Advisors and testing hooks and could put together that reference pair.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -15965,7 +15842,6 @@
           <t>Hi Paul,
 I came across Forex Signal Bot, with its SMC market structure analysis, liquidity mapping, fair value gaps and Streamlit dashboard on top of MetaTrader 5.
 SMC logic is much easier to trust when you can see it on the chart. I build MQL5 indicators and Expert Advisors and could turn the structure, liquidity and FVG detection into an MT5 indicator that draws the zones, and optionally an EA that trades them on a VPS with the same risk rules as your Python version.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, I can send over a short example. Would you be open to it?
 Best regards,
 Oseni Ibrahim
@@ -16039,7 +15915,6 @@
           <t>Hi LogicCrafterDZ team,
 I noticed your numbered MT5 strategy series on GitHub: SmartOrderBlocks, Liquidity Sweep Reversal, Gap Reversion Pro and Smart Scalp PA, alongside the Null Hypothesis research engine. It is a well organised way to test one idea per EA.
 When a series grows like this, the same risk sizing, session filters, trade management and logging code tends to get copied into each EA. I'm a MetaTrader developer and could help pull that into a shared MQL5 include library, so new strategies only contain their entry logic, and add optional Telegram reports for fills and daily results.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of how such a shared core is usually structured.
 Best regards,
 Oseni Ibrahim
@@ -16118,7 +15993,6 @@
           <t>Hi Harrison,
 I came across the Neuro Trading overview on GitHub and saw that MetaTrader 5 connectivity and structured risk management sit at the centre of the platform, with you as founder and lead developer.
 Integration layers like that tend to take a lot of maintenance: symbol naming differences between brokers, fill and requote handling, and keeping risk limits enforced even when the platform side is unavailable. I'm a MetaTrader developer and build MQL5 bridge EAs and broker-side risk modules that sit between a platform and the MT5 terminal.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want extra hands on the MT5 side while you focus on the AI and product work, would you be open to discussing it? I can also send over a short example of a bridge EA.
 Best regards,
 Oseni Ibrahim
@@ -16187,7 +16061,6 @@
           <t>Hi IU Technical team,
 I came across the Multi-Pair Grid Trading Manager on GitHub, a desktop app that runs grid strategies across several pairs through the MetaTrader 5 API with MySQL logging and a config panel for credentials.
 Grid systems carry most of their risk in the basket, so I wanted to suggest one addition: a small MQL5 companion EA that runs inside MT5 and enforces basket stop, equity drawdown and max-level limits even if the desktop app or its connection stops. It can also push grid status to Telegram. I'm a MetaTrader developer and build this kind of guard layer for Python-driven systems.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of how the companion EA and the desktop app could share state?
 Best regards,
 Oseni Ibrahim
@@ -16256,7 +16129,6 @@
           <t>Hi ALSHAHEEN team,
 I came across the ALSHAHEEN documents on GitHub and saw that the app, distributed through the Microsoft Store, works on top of the user's own signed-in MetaTrader 5 terminal with Algo Trading enabled.
 Products built this way usually spend a lot of support time on the MT5 side: broker symbol suffixes, different filling modes, disabled algo trading and terminal builds that behave slightly differently. I'm a MetaTrader developer and can help with helper EAs or scripts that run diagnostics inside the terminal, normalise symbols and filling types, and report problems back to your app.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would take some load off your support queue, I can send over a short example of a diagnostics EA.
 Best regards,
 Oseni Ibrahim
@@ -16330,7 +16202,6 @@
           <t>Hi Chibuike,
 I came across your AI automation portfolio and the trading bot that connects MetaTrader 5, OpenAI and Telegram with daily loss limits and a live dashboard. I also saw you offer Telegram bots and API integrations on Fiverr.
 Clients who ask for a trading bot often end up needing native MetaTrader code as well: an MT4 or MT5 Expert Advisor, a custom indicator, or a TradingView alert converted into MQL5. I'm a MetaTrader developer and would be glad to work as a subcontract partner on those parts, while you keep the Python, AI and Telegram side.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could help you take on more trading jobs, I can send over a few examples of recent MQL5 work.
 Best regards,
 Oseni Ibrahim
@@ -16409,7 +16280,6 @@
           <t>Hi Samuel,
 I came across QUARSHFX Intelligence and your note on why v1 uses OANDA rather than MetaTrader: the MetaTrader5 Python package only runs on Windows with the terminal open, which does not fit a free Linux cloud host.
 There is another route for the MetaTrader bridge you mention for later. The signal engine stays on your Linux server, and a small MQL5 Expert Advisor inside the trader's own MT4 or MT5 terminal polls your API with WebRequest, then places and manages the trades locally. No Python on Windows is needed, and it works with any MetaTrader broker. I'm a MetaTrader developer and build this kind of signal-to-EA bridge.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send over a short example of the EA side.
 Best regards,
 Oseni Ibrahim
@@ -16488,7 +16358,6 @@
           <t>Hi André,
 I came across FXNews and was impressed by the discipline around it: composite scoring with MT5 calendar context, historical validation reports, and a build that fails on any MQL5 warning, not just errors.
 Since FXNews is deliberately chart-only, I wondered whether you have considered an optional layer on top. That could be a Telegram or push alert when a pair crosses a score threshold, or a separate EA that reads the scores and handles entries under fixed risk rules while the indicator stays untouched. I'm a MetaTrader developer and would follow the same zero-warning standard.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either idea interests you, I can send over a short example of how an EA can read an indicator's scores cleanly.
 Best regards,
 Oseni Ibrahim
@@ -16562,7 +16431,6 @@
           <t>Hi Maziar,
 I came across your GitHub profile and saw that AIOTA Trading Journal Pro syncs with MetaTrader 5 and is published on the MQL5 Market, alongside the Market Structure Suite and the other AIOTA products you are building.
 Selling on the Market brings its own MQL5 workload: passing automatic validation after each update, keeping MT4 and MT5 editions in step, and fixing edge cases buyers report on different brokers. I'm a MetaTrader developer and could take some of that off your plate, from new features in the sync component to Market-ready builds of new tools.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If extra MQL5 capacity would help, would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -16641,7 +16509,6 @@
           <t>Hi Daniel,
 I came across Helios and its self-learning setup that pairs a Python ML system with a MetaTrader 5 Expert Advisor. I noticed the troubleshooting section includes a case for the MT5 EA not receiving signals.
 That link between Python and the EA is where most hybrid systems get fragile. I'm a MetaTrader developer, and I usually handle it with a heartbeat between both sides, automatic reconnects, acknowledgements for every order and a safe mode in the EA that keeps stops managed if the signals stop. I can also add equity-based limits directly in MQL5.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still developing Helios, would it be useful if I sent over a short example of that bridge pattern?
 Best regards,
 Oseni Ibrahim
@@ -16715,7 +16582,6 @@
           <t>Hi Kukuh,
 I came across AI Forex Trading Assistant and its design where each user connects their own MT5 account through an isolated terminal and a private Python bridge, with Telegram as the interface. I noticed per-account worker provisioning, bridge verification and restart recovery on Windows VPS are still on the list.
 That is the part I work on most. I'm a MetaTrader developer and set up multi-terminal MT5 hosting on Windows VPS, with watchdogs that restart crashed terminals, health checks for each account, and a small MQL5 guard EA that keeps stops and daily limits enforced inside the terminal if the bridge drops.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want help getting that layer production-ready, would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -16789,7 +16655,6 @@
           <t>Hi BotTrade team,
 I came across your BotTrade workspace with the Lorentzian Classification and ML Kernel Regression EAs for MT5. I noticed the README points out two risks: stealth SL/TP orders are lost if the VPS or terminal goes down, and WebRequest calls to alert services can slow the EA.
 Both have practical fixes. A wide emergency stop can sit on the broker server while the stealth levels stay hidden, and alerts can move to a separate queue so the trading logic never waits for the network. I'm a MetaTrader developer and add this kind of protection and Telegram alerting to existing MQL5 EAs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you would like, I can send over a short example of the emergency-stop pattern.
 Best regards,
 Oseni Ibrahim
@@ -16868,7 +16733,6 @@
           <t>Hi Osama,
 I came across your profile and the white-label MT5 copy-trading SaaS: multi-tenant control plane, Stripe billing, Discord and Telegram bots, and MetaTrader 5 master and follower Expert Advisors.
 In copy trading the EAs usually generate most of the support tickets: broker symbol suffixes, lot scaling between account sizes, partial closes, slippage limits and followers reconnecting after a restart. I'm a MetaTrader developer and could help on that layer, whether that means hardening the current EAs, adding MT4 followers or building per-tenant risk rules.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 With your full-stack and Web3 work also running, would extra MQL5 capacity be useful? I can send over a short example of a follower EA's sync logic.
 Best regards,
 Oseni Ibrahim
@@ -16947,7 +16811,6 @@
           <t>Hi Umair,
 I came across your case study on the live-vs-backtest divergence, where break-even and trailing were evaluated at bar close and the profit factor fell from 1.38 to 0.55. It is one of the clearest explanations of that problem I have read.
 I'm a MetaTrader developer focused on building and repairing MT4/MT5 EAs. Your diagnosis service and my work seem to fit together: once you find the cause, clients often need the trade management rewritten to tick level, an MT4 EA ported to MT5, or monitoring added so the issue does not come back. I would be glad to take on that implementation work as a partner, or refer clients who need a diagnosis to you.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -17021,7 +16884,6 @@
           <t>Hi Kenny,
 I came across your DRL XAUUSD bot and the walk-forward setup around the Soft Actor-Critic agent. I also read your honest note that the live mt5bridge.py does not mirror the backtest yet: it thresholds the action to long, short or flat, uses a fixed lot size, and places no per-trade stop loss or take profit.
 That live execution layer is my area. I'm a MetaTrader developer and could help map the agent's continuous action to position size, attach broker-side stops so trades stay protected if the script stops, and move the macro circuit breaker into a small MQL5 guard EA.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you plan to keep developing the project, I can send over a short example of how that bridge could look.
 Best regards,
 Oseni Ibrahim
@@ -17095,7 +16957,6 @@
           <t>Hi Sri Ram,
 I came across HydraPrime and the write-up behind it. Two years of solo iteration on a gold EA shows, especially in details like state recovery through terminal global variables after a VPS restart and the move to CPositionInfo and COrderInfo wrappers.
 I'm a MetaTrader developer, and the work that usually comes next for an EA at this stage is operational: Telegram reports for fills and drawdown, a watchdog on the VPS, and checks across brokers whose gold symbols, contract sizes and stop levels differ. I'd be glad to help with any of that, or be a second reviewer on the MQL5 code.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of the monitoring side first.
 Best regards,
 Oseni Ibrahim
@@ -17169,7 +17030,6 @@
           <t>Hi Mehdi,
 I came across GoldTraderEA and saw how much interest it has drawn, with around 145 stars for a gold EA that combines 14 weighted strategies with multi-layer confirmation.
 Open-source EAs that get popular usually collect the same kinds of requests: it does not trade on a certain broker because of symbol suffixes or stop levels, can it send Telegram alerts, is there an MT4 version. I'm a MetaTrader developer and would be glad to help with that maintenance, whether that means fixing broker compatibility, adding notifications or building a clean MT4 port, so you can keep working on the strategy side.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a short example of the kind of changes I mean.
 Best regards,
 Oseni Ibrahim
@@ -17243,7 +17103,6 @@
           <t>Hi Carlos,
 I came across your MQL5 Trading Bot and liked the engineering around it: an LSTM filter in front of four SMC setups, order retries with backoff, and daily drawdown protection. I noticed the model talks to the EA through a CSV file in MQL5/Files.
 File bridges work, but they tend to be where stale signals and silent stalls creep in. I'm a MetaTrader developer and could help move that link to a socket or HTTP channel with heartbeats and timestamps, so the EA knows when a prediction is fresh and falls back safely when it is not. I can add Telegram alerts for fills and errors at the same time.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that bridge?
 Best regards,
 Oseni Ibrahim
@@ -17312,7 +17171,6 @@
           <t>Hi gold-mouse team,
 I came across your MQL5 Copy Trading Bot, where the master writes trades to a binary file and several slave accounts read it to mirror positions. It is a clean, simple design, and I noticed the README already has a section on file operation errors.
 The file approach limits copying to terminals on the same machine. I'm a MetaTrader developer and have extended copiers like this with a small relay so masters and followers can run on different VPS servers, along with broker symbol mapping, lot scaling by balance and an MT4 follower for mixed setups.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still developing the bot, would it be useful if I sent over a short example of the relay approach?
 Best regards,
 Oseni Ibrahim
@@ -17386,7 +17244,6 @@
           <t>Hi Amon,
 I came across your MQL5 Projects repository with its collection of Expert Advisors, indicators and scripts, and saw that you work across MQL4, MQL5 and Python for traders who want automated solutions.
 I'm a MetaTrader developer doing similar work: MT4 and MT5 EAs, MT4-to-MT5 conversions, TradingView-to-MT5 integrations and Telegram alerts. Solo developers often get client requests in waves, so I wanted to suggest a simple partnership where we pass overflow or specialised jobs to each other, for example you keep the Python and analysis side while I take an MQL port or a copier module.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds reasonable, I can send over a few examples of my MQL5 code first.
 Best regards,
 Oseni Ibrahim
@@ -17460,7 +17317,6 @@
           <t>Hi Joel,
 I came across your Signal Service Platform, where a master Sender EA posts trades to the Express API and the dashboard handles subscriptions and flags disconnected MT5 accounts every hour.
 In setups like this the EAs decide what subscribers experience. A missed POST during a broker hiccup or a symbol with a different suffix on a follower account shows up as a missing trade. I'm a MetaTrader developer and could help harden that layer: a local retry queue and heartbeat in the Sender EA, symbol mapping and lot scaling in the receiving EA, and an MT4 receiver if some subscribers are still on MT4.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example first.
 Best regards,
 Oseni Ibrahim
@@ -17534,7 +17390,6 @@
           <t>Hi Faris,
 I came across your GitHub profile and saw that MT5 strategy development and automated trading infrastructure sit alongside your simulation engines and software platform work, including a trading signal management platform.
 I'm a MetaTrader developer focused on MQL4 and MQL5: Expert Advisors, indicators, risk modules, Telegram alerts and bridges between MT5 and Python or web backends. When the MQL side of a client project is the bottleneck, I can take that part as a subcontractor while you keep the architecture and the rest of the stack.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful for your pipeline, I can send over a few examples of recent MQL5 work.
 Best regards,
 Oseni Ibrahim
@@ -17603,7 +17458,6 @@
           <t>Hi Punokawan team,
 I came across EA Punokawan V.8_MA on GitHub, with its Dynamic Recovery Cycle, break-even projection, semi-manual buttons and hidden SL/TP.
 For averaging EAs, hidden stops are good against stop hunting, but they only exist while the terminal is running. If the VPS or connection drops, the account has no protection. I'm a MetaTrader developer and often add a wide broker-side safety stop behind the hidden levels, plus an equity guard. I can also build account-bound, time-limited trial licences, so the trial copies you send out stay under control.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either would help the next version, I can send over a short example of how the safety stop works alongside hidden SL/TP.
 Best regards,
 Oseni Ibrahim
@@ -17682,7 +17536,6 @@
           <t>Hi James,
 I came across JamesmariaEA, the MT5 Expert Advisor that trades EURUSD, EURGBP and gold with dynamic lot sizing and an equity-based stop, and saw you run it headless on Linux through Wine and Xvfb.
 With no screen to glance at, the weak points are usually visibility and combined risk: nobody notices when the terminal disconnects, and correlated EUR pairs can stack exposure. I'm a MetaTrader developer and can add Telegram reports for fills, errors and daily results, a heartbeat that warns you if the terminal goes quiet, and a cap on total exposure across the three symbols.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the monitoring module?
 Best regards,
 Oseni Ibrahim
@@ -17751,7 +17604,6 @@
           <t>Hi EA Perfect FX team,
 I came across your USDJPY M15 Expert Advisor for MT5 on GitHub, with its published Strategy Tester report and the 7-day free trial offered to anyone who sends their account number, one EA per account.
 Managing that by hand gets heavy as more traders ask for trials. I'm a MetaTrader developer and can build the account binding and trial expiry into the EA itself, with a small licence server so you can switch a trial to a paid licence or extend it without sending a new file. If you plan more pairs or an MT4 edition, I can help there too.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would save you time, I can send over a short example of the licence flow.
 Best regards,
 Oseni Ibrahim
@@ -17830,7 +17682,6 @@
           <t>Hi Sivaraman,
 I came across MT5-Dev and the ChartDrawBridge EA that fills a real gap: the official MetaTrader5 Python package cannot draw on charts, so your file-based command protocol lets Python place lines, labels and arrows.
 I'm a MetaTrader developer and have built similar bridges. If you want to take it further, a socket channel with acknowledgements removes the polling delay of files, and the same EA can also accept trade or alert commands, so one bridge covers drawing and execution. I could help with the MQL5 side of that, or with making it robust enough to share with other traders.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of the socket version first.
 Best regards,
 Oseni Ibrahim
@@ -17899,7 +17750,6 @@
           <t>Hi TradeDash team,
 I came across TradeDash MT5 EA, the on-chart dashboard for fast order entry, direct-price stop loss and take profit, trailing control and exit-all.
 Panels like this sell well to prop firm traders, and they usually ask for two things: lot size calculated from a risk percentage and stop distance, and a daily loss lock that closes everything and blocks new orders once a limit is hit. Many retail brokers also still run MT4. I'm a MetaTrader developer and could add those risk features and build a matching MT4 edition, so the dashboard reaches both groups.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of the daily loss lock.
 Best regards,
 Oseni Ibrahim
@@ -17973,7 +17823,6 @@
           <t>Hi Mykhailo,
 I came across your profile and TradeHub, with eight years of MQL4 and MQL5 work across Expert Advisors, trade copiers and risk management systems, and the BbRsi EA you published.
 I'm a MetaTrader developer doing similar work, mainly MT4 and MT5 EAs, MT4-to-MT5 conversions, TradingView-to-MT5 integrations and Telegram alerts. Busy freelance periods usually bring more good projects than one person can take, so I wanted to offer myself as a subcontractor for overflow work, delivered to your standards and under your name with the client.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could be useful, I can send over a few samples of my MQL5 code so you can judge the quality first.
 Best regards,
 Oseni Ibrahim
@@ -18047,7 +17896,6 @@
           <t>Hi MX Forex Trader team,
 I came across your Admin Panel v11 and saw that clients are managed in the cloud with PostgreSQL and JWT auth, but the MT5 EA still gets its licence list through MX_Clients.csv, downloaded and copied into MQL5/Files every time a client is added.
 Since the API is already online, the EA could check the licence itself. I'm a MetaTrader developer and can add a WebRequest call to your API at start-up and at intervals, with a cached result and a grace period so a short outage does not stop trading. New clients would work the moment you add them, and expired ones stop automatically.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that licence check?
 Best regards,
 Oseni Ibrahim
@@ -18121,7 +17969,6 @@
           <t>Hi Pranav,
 I came across your Trading Journal MT5 to Google Sheets EA, which posts each trade to a Google Apps Script URL through WebRequest. It is a simple, practical way to keep a journal without paid software.
 The weak point with Apps Script is that a timeout or quota limit can drop a trade without anyone noticing. I'm a MetaTrader developer and could add a small local queue in the EA that retries failed posts, marks trades as sent to avoid duplicates, and backfills history after the terminal restarts. An MT4 version would also let traders on MT4 brokers use it.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still improving the tool, would it be useful if I sent over a short example of the retry queue?
 Best regards,
 Oseni Ibrahim
@@ -18200,7 +18047,6 @@
           <t>Hi Badal,
 I came across the Lite version of your Trend-Following EA v2 and saw that the full version is licensed by email, with prop-firm-style risk management and a five-year NAS100 test on MT5 tick data.
 Once licences start selling, two requests tend to follow: locking each copy to the buyer's account with an expiry date, and ready-made presets for each prop firm's daily loss and maximum drawdown rules. I'm a MetaTrader developer and can build both into the EA, along with a simple way for you to extend or revoke licences without sending new files.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of the licence and preset logic first.
 Best regards,
 Oseni Ibrahim
@@ -18274,7 +18120,6 @@
           <t>Hi Andrés,
 I came across Atoms para MQL5 on your profile and liked the approach: new-bar detection, indicators, risk management and order execution as small decoupled units instead of one large EA file.
 I'm a MetaTrader developer, and libraries like this are exactly what I use when building EAs for clients. If you would like to grow Atoms, I could contribute modules that most EAs end up needing, such as session and news filters, trailing and break-even managers or a Telegram notifier, following your naming and coupling rules. I would also be open to passing along EA projects that could be built on it.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds interesting, would it be useful if I sent over a short example module first?
 Best regards,
 Oseni Ibrahim
@@ -18348,7 +18193,6 @@
           <t>Hi Monarch Trades team,
 I came across your MT4/MT5 indicators collection on GitHub, with tick movement, last-digit and candle pattern tools, and saw that you offer premium indicators and one-to-one mentorship.
 When indicators are sold, two requests usually follow. Students ask for an EA that trades the signals automatically with fixed risk rules, and paid files need protecting so they do not spread through Telegram groups. I'm a MetaTrader developer and can turn indicator logic into MT4 and MT5 Expert Advisors and add account-number licensing with expiry dates to premium tools.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If either would help your offer, would you be open to discussing it? I can send over a short example first.
 Best regards,
 Oseni Ibrahim
@@ -18427,7 +18271,6 @@
           <t>Hi Dr. Khodakarami,
 I came across MT-Core-Lib and the way each YouTube session on YourTradeMaster has its own example Experts and Indicators in the TMCoreTest folders. It is a practical way to teach MQL5.
 Preparing and testing those examples for every video takes a lot of time. I'm a MetaTrader developer, and I could help build and test example projects on top of your library, including more advanced ones students often ask for, such as a trade manager panel, Telegram alerts or a TradingView-to-MT5 bridge. You would keep full control of the teaching and the code style.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you plan more sessions, would it be useful if I sent over a short example built on MT-Core-Lib?
 Best regards,
 Oseni Ibrahim
@@ -18501,7 +18344,6 @@
           <t>Hi Brent,
 I came across Pythology on GitHub and saw that you develop and optimise strategies for clients, whether they start in Python or as MT5 Expert Advisors, and that your USD Strength Index and regime dashboard update live from MT5.
 Once a strategy is optimised, clients often want it delivered as a clean MT5 EA they can run on a VPS or prop account. I'm a MetaTrader developer and could work as your MQL5 implementation partner, turning the final parameters into a robust EA with proper order handling and risk limits, and building MT5 data exports for your dashboards when needed.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a short example of my MQL5 work first.
 Best regards,
 Oseni Ibrahim
@@ -18580,7 +18422,6 @@
           <t>Hi Andreas,
 I came across your GitHub profile and saw that, next to your web work for clients, you build algorithmic trading bots in C# for MetaTrader and cTrader.
 I'm a MetaTrader developer focused on MQL4 and MQL5. Clients who start on cTrader often later ask for the same bot on MT4 or MT5 because their broker or prop firm only offers MetaTrader, and the port to native MQL5 can take more time than expected. I would be glad to act as a subcontractor on those parts, or on any MetaTrader-specific work such as risk modules, trade copiers or Telegram alerts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could be useful, I can send over a few examples of my MQL5 code.
 Best regards,
 Oseni Ibrahim
@@ -18659,7 +18500,6 @@
           <t>Hi Naphat,
 I came across Vortex Prime and the two-year GBPUSD H1 dataset you published with it. I also liked that the README asks users to start in dry-run mode before risking real money.
 With grid and martingale logic, most of the risk sits in the basket rather than any single trade. I'm a MetaTrader developer and often add three things to EAs like this: an equity-based basket stop, a hard cap on grid levels and lot size, and Telegram alerts when the basket passes set drawdown levels. Together they give users a clear safety net when they move from dry-run to live.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are still developing the EA, would it be useful if I sent over a short example of the basket guard?
 Best regards,
 Oseni Ibrahim
@@ -18733,7 +18573,6 @@
           <t>Hi Uğur,
 I came across MT4 Monitor v2 and its setup that syncs MT4 account data into SQLite and Google Sheets for the mt4pool project. It is a practical way to keep an eye on several accounts in one sheet.
 Most brokers and prop firms now push new accounts to MT5, so at some point the pool will likely mix both platforms. I'm a MetaTrader developer and could build an MT5 export EA that writes the same fields your pipeline already expects, so MT5 accounts appear next to the MT4 ones without changes to the Node side. I can also add Telegram alerts for drawdown limits or accounts that stop reporting.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the MT5 export EA?
 Best regards,
 Oseni Ibrahim
@@ -18807,7 +18646,6 @@
           <t>Hi Ratna,
 I came across your MT5 to MatchTrader Trade Copier, which mirrors MT5 trades onto MatchTrader prop firm accounts from a Python app.
 Copiers built on the MetaTrader5 Python package usually poll the terminal, so fast modifications or partial closes can arrive late, and nothing is sent if the script pauses. I'm a MetaTrader developer and could add a small MQL5 master EA that pushes every trade event to your copier the moment it happens through OnTradeTransaction, with a sequence number so nothing is missed after a restart. Symbol mapping and lot scaling per prop account can live in the same layer.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would strengthen the copier, would it be useful if I sent over a short example of the event-push EA?
 Best regards,
 Oseni Ibrahim
@@ -18881,7 +18719,6 @@
           <t>Hi Saif,
 I came across your GitHub profile and saw that you build custom indicators, Expert Advisors and forex bots on MetaTrader 4 and 5 for clients worldwide through Upwork.
 I'm a MetaTrader developer doing the same kind of work, with a focus on MT4-to-MT5 conversions, TradingView-to-MT5 bridges, trade copiers and Telegram integrations. Freelance work tends to come in waves, so I wanted to suggest a simple arrangement: when you have more jobs than time, or a client needs a module outside your usual scope, I can build it as a subcontractor and you stay the client's point of contact.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my MQL5 work first.
 Best regards,
 Oseni Ibrahim
@@ -18960,7 +18797,6 @@
           <t>Hi Massimo,
 I came across PipLock AI and liked the idea of a killswitch that makes traders stick to their own rules, with EA_PipLock sending heartbeats and account data to your Supabase webhook.
 One thing that would make it stronger is letting the EA enforce the core rules itself: closing positions and blocking new orders inside MT5 when the daily loss or trade count is reached, even if the phone or webhook is offline. I'm a MetaTrader developer and could add that, along with a queue for failed webhook posts and an MT4 version for traders on MT4 brokers.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of in-terminal rule enforcement?
 Best regards,
 Oseni Ibrahim
@@ -19039,7 +18875,6 @@
           <t>Hi Muhammad,
 I came across your profile and the 15+ funded-trader applications you have shipped, with challenge flows, leaderboards and live MT5, MatchTrader and TradeLocker account sync.
 On prop-firm projects, the MetaTrader side often needs pieces a full-stack team does not usually build: an EA that checks daily loss and drawdown on every tick, tools that export trade history in the exact format the dashboard expects, or checks for EA and copy-trading rules. I'm a MetaTrader developer and could be your MQL5 partner for those parts, so you can quote and deliver complete platforms.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of MT5 rule-monitoring code.
 Best regards,
 Oseni Ibrahim
@@ -19118,7 +18953,6 @@
           <t>Hi Jeh,
 I came across your JehKTech profile and the MetaTrader 5 copier architecture you run across funded accounts at firms like GoatFunded, AlphaCapital and FundedNext.
 Copying across prop firms gets tricky because every firm has its own daily loss rule, drawdown type and symbol names. I'm a MetaTrader developer and often build MQL5 receivers for copiers like this, where each follower account has its own rule guard that blocks or scales a trade before it breaks that firm's limits, with symbol and lot mapping per account. Native receivers also cut the delay compared with Python polling.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits where your copier is heading, would it be useful if I sent over a short example of the rule guard?
 Best regards,
 Oseni Ibrahim
@@ -19197,7 +19031,6 @@
           <t>Hi Nancy,
 I came across your profile and the multi-broker platform you built at Naxfront, with an async engine routing signals over ZeroMQ to NinjaTrader, MT5/FTMO, Interactive Brokers and Tradovate.
 Of those four, the MT5 leg usually needs the most care: the EA on the terminal side has to reconnect cleanly, confirm every fill back to the engine and respect FTMO's daily loss and max drawdown rules even when the engine sends something it should not. I'm a MetaTrader developer and build ZeroMQ and socket endpoint EAs for exactly this kind of setup.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you want a second pair of hands on the MT5 side, would you be open to discussing it? I can send over a short example first.
 Best regards,
 Oseni Ibrahim
@@ -19276,7 +19109,6 @@
           <t>Hi Svenn,
 I came across your profile and the stonedesk-harness work: a per-book risk state machine, firm-aware drawdown, a watchdog and an execution-quality ledger, with nautilus-mt5-bridge connecting it all to MetaTrader 5. The focus on systems that fail safely is refreshing.
 One layer that fits your philosophy is a small MQL5 companion EA on the terminal side of the bridge. It would enforce the firm's hard drawdown limit inside MT5 even if the engine or bridge stops, and report fill prices, slippage and server timestamps straight from OnTradeTransaction for your ledger and reconciliation. I'm a MetaTrader developer and build this kind of in-terminal guard.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -19350,7 +19182,6 @@
           <t>Hi Sergio,
 I came across your NewsFilter library for MT5 and liked how small it keeps things: one WebRequest per day to the Forex Factory feed, cached and parsed with JAson.mqh, ready to drop into prop-firm EAs.
 Two additions come up often with news filters like this. The first is a fallback to MT5's built-in economic calendar when the feed is unreachable or the URL is not whitelisted. The second is Strategy Tester support, where WebRequest is not available, by loading a stored history of past events, so traders can backtest with the filter switched on. I'm a MetaTrader developer and could help with either, or with an MT4 port.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of the calendar fallback?
 Best regards,
 Oseni Ibrahim
@@ -19424,7 +19255,6 @@
           <t>Hi Francisco,
 I came across your profile and the trading-ea-mql5 workspace template, with its risk-first, feature-driven structure, and saw you use it for an S&amp;P 500 highs and lows EA on prop firm accounts in MetaTrader 5.
 Combining that with a medical career cannot leave much spare time. I'm a MetaTrader developer and could take on parts of the EA work that are easy to get wrong on prop accounts: guards for each firm's daily loss and drawdown rules, a news filter around US data releases, and Telegram reports so you can check the account between shifts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, would it be useful if I sent over a short example built on your template's structure?
 Best regards,
 Oseni Ibrahim
@@ -19503,7 +19333,6 @@
           <t>Hi Javad,
 I came across JR MQL5 Market and RiskCockpit in particular: a prop-firm risk manager covering FundedNext, FTMO, E8 and The5ers rules is useful, and I noticed the .ex5 files are bound to each user's account number and sent out by hand within 24-48 hours.
 I'm an MQL4/MQL5 developer. Two things I could help with if they are on your list: MT4 versions of RiskCockpit and ProSessionBox, since many prop traders are still on MT4, and a simple automated way to issue account-bound builds so requests don't depend on your inbox. I'm also happy to take on new tools under your brand while you keep the design decisions.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of how I would handle the account binding.
 Best regards,
 Oseni Ibrahim
@@ -19572,7 +19401,6 @@
           <t>Hi Madarik Trader Pro team,
 I came across Madarik Trader Pro on GitHub and saw that it connects Deriv, Binance, MetaTrader 5 and TradingView webhooks in one bot, with a licence key per device.
 I'm an MQL4/MQL5 developer. For MT5 users, a small native Expert Advisor can make execution sturdier than driving the terminal only from Python: it can receive your bot's signals, apply lot sizing and stop rules inside MT5, and keep managing open trades if the phone or PC running the bot disconnects. I could build that companion EA to match your licence system, or add an MT4 version for users on older brokers.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're considering, I can send over a short example of how the EA would receive signals.
 Best regards,
 Oseni Ibrahim
@@ -19646,7 +19474,6 @@
           <t>Hi Neo,
 I came across your CRT Turtle Soup EAs and noticed the README says they are alert-only by default, with no auto-trading yet. The wick validation and the multi-symbol scanning across 60+ instruments from one chart are a solid base for that next step.
 I'm an MQL4/MQL5 developer, and adding execution to detection logic like this is work I do often: optional auto-entry with the existing Entry/SL/TP1/TP2 levels, partial closes at TP1, per-symbol risk limits and Telegram notifications, all switchable by inputs so the alert-only mode stays the default. The same approach could apply to the Ichimoku and gold scalper EAs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're planning, I can send over a short example of how I'd structure it.
 Best regards,
 Oseni Ibrahim
@@ -19725,7 +19552,6 @@
           <t>Hi Abdurrahman,
 I came across Traxovia AI and the 7-gate ICT engine: order blocks, fair value gaps and CHoCH confirmation, then an XGBoost confidence layer before live MT5 execution on five pairs.
 I'm an MQL4/MQL5 developer focused on the MetaTrader side of platforms like this. Once signals leave the FastAPI stack, a small MQL5 execution EA can take care of broker-specific lot and stop rounding, spread checks at entry, partial closes and trailing, and keep managing trades if the API container restarts. I could also help set up the terminal on a Windows VPS with basic health alerts so the live side runs unattended.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send over a short example of the signal-to-EA handoff.
 Best regards,
 Oseni Ibrahim
@@ -19804,7 +19630,6 @@
           <t>Hi Brayan,
 I came across your Order Blocks EA repo, the Pine Script v6 to MQL5 conversion with indicator parity checked over 12 years of EURUSD M30 data, and saw that you take freelance MQL5 and conversion projects.
 I'm a trading bot developer doing similar work: MT4/MT5 Expert Advisors, MT4 to MT5 conversion, TradingView integration and EA maintenance. When projects stack up, it can help to have another developer to pass overflow to, or to split a larger job, for example you handle the Pine logic and I cover MT4 builds, risk modules or Telegram alerts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing a simple overflow arrangement? I can send a few examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -19878,7 +19703,6 @@
           <t>Hi there,
 I came across MT5-Bridge-TradingView, the open-source bridge that picks up trades from the TradingView Strategy Tester and executes them on MetaTrader 5, and saw that you offer commercial support for custom features and installs.
 Requests on bridges like this tend to cluster around the MT5 side: partial closes, pending order types, broker symbol suffixes, lot rounding and an MT4 receiver for clients still on MT4. I'm a trading bot developer working in MQL4/MQL5 and TradingView integrations, and I could take on some of those custom jobs as a subcontractor when your queue fills up.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing that? I can send over a few examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -19952,7 +19776,6 @@
           <t>Hi Freedom,
 I came across MT5 Reverse Trader on GitHub, the PyQt5 copier that watches MT5 investor accounts and mirrors their positions to a master account, with the option to reverse direction.
 One limit of copiers built only on the Python MetaTrader5 package is that each process talks to one terminal and has to poll for changes. A small MQL5 EA on each source terminal can push trade events as they happen and handle modifications and partial closes more cleanly. I'm a trading bot developer working in MQL4/MQL5, and I could build that EA layer, or an MT4 version, to sit alongside your app.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -20021,7 +19844,6 @@
           <t>Hi Simple AlgoTrading Solutions team,
 I came across the Gold Daily Breakout EA documentation hub on GitHub and saw that you sell MINI and PRO versions on Gumroad, with prop firm settings for FTMO, BlueGuardian and others.
 Keeping two builds and several prop presets in step each time the breakout logic changes takes time, and buyers tend to ask for MT4 versions or extra protections like daily loss locks. I'm a trading bot developer working in MQL4/MQL5, and I could help maintain both builds from one codebase, add firm-specific guards, or produce an MT4 edition of the EA.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of that would help, I can send over a few examples of similar EA work.
 Best regards,
 Oseni Ibrahim
@@ -20095,7 +19917,6 @@
           <t>Hi Sadegh,
 I came across your profile and the NeuronAlgo portfolio, where research from Qlib and ML pipelines ends up deployed as MQL5 Expert Advisors on MT5, with live EAs running for over a year on prop-firm accounts.
 For small quant teams, turning a validated idea into a clean production EA with drawdown limits and allocation logic is often where time disappears. I'm a trading bot developer working in MQL4/MQL5, and I could take on that implementation step, or maintain existing EAs as brokers and prop rules change, so your time stays on research.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -20169,7 +19990,6 @@
           <t>Hi Rana,
 I came across the gold-trade-advanced-bot repo and IntradayAurumPulsePro, and saw that you offer a premium version with multi-pair support and commercial licensing for clients and prop firms.
 Once a premium EA is sold to different clients, requests pile up: account-locked licenses, custom risk settings, prop-firm daily loss guards, or an MT4 build. I'm a trading bot developer working in MQL4/MQL5, and I could help as extra capacity on those client-specific builds so you can keep focus on the core strategy.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a few examples of similar work.
 Best regards,
 Oseni Ibrahim
@@ -20243,7 +20063,6 @@
           <t>Hi Vipin,
 I came across your GitHub profile and saw that you build live algorithmic trading systems for clients, including MT5/MQL5 strategies and broker API integrations, alongside your Python work.
 When a client project needs deep MQL work, such as a full Expert Advisor, an MT4 to MT5 conversion, or an MQL5 bridge to a Python backend, it can pull time away from the rest of the build. I'm a trading bot developer focused on MQL4/MQL5, and I'd be happy to take on those parts as a subcontractor while you keep the client relationship and the Python side.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing a simple arrangement? I can share examples first.
 Best regards,
 Oseni Ibrahim
@@ -20317,7 +20136,6 @@
           <t>Hi there,
 I came across AI Backtester on GitHub, the web platform for testing and optimizing Python trading bots against real MetaTrader 5 market data.
 A natural next step for users is taking a strategy that passed your tests and running it natively inside MT5, or pulling cleaner tick and bar history straight from the terminal. I'm a trading bot developer working in MQL4/MQL5, and I could help with an MQL5 exporter EA for data, or a template that turns tested Python logic into an Expert Advisor with the same risk settings.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -20386,7 +20204,6 @@
           <t>Hi JIG BOT team,
 I came across the JIG BOT v1 page on GitHub, the XAUUSD M1 engine for MT5 with VWAP take-profit, a 10-level recovery multiplier, cent account support and SHA-256 machine verification behind a 7-day trial.
 EAs sold this way usually need steady upkeep: license checks that survive terminal reinstalls, fixes for brokers with unusual gold symbols or stop levels, and extra safeguards buyers ask for. I'm a trading bot developer working in MQL4/MQL5, and I could help maintain those parts, or build an MT4 edition if your users request one.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would be useful, I can send over a few examples of similar EA work.
 Best regards,
 Oseni Ibrahim
@@ -20455,7 +20272,6 @@
           <t>Hi there,
 I came across your Telegram Signal to MT5 Auto Trader on GitHub and noticed the Future Updates list: more signal formats, custom lot sizing, advanced position management and additional platforms.
 Several of those are easier and more reliable inside the terminal. A small MQL5 companion EA can handle partial take-profits, breakeven and trailing stops even if the Python side is briefly offline, and an MT4 version covers users on older brokers. I'm a trading bot developer working in MQL4/MQL5, and I could build those pieces to plug into your existing signal reader.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -20524,7 +20340,6 @@
           <t>Hi Kawacoline,
 I came across OrderFlow Core, the Auction Market Theory system that pairs a native MQL5 Expert Advisor with a Python state machine and Telegram control, and also saw Airstrike-BTC-Engine running on MetaTrader 5.
 Two MT5 engines at once means a lot of MQL5 work: execution handling, volume profile calculations inside the terminal, and the testing that keeps the EA and Python side in agreement. I'm a trading bot developer working in MQL4/MQL5, and I could act as extra capacity on the EA side of either project.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -20593,7 +20408,6 @@
           <t>Hi Ophireum team,
 I came across the SYMMETRIX GOLD SMC document on GitHub and noticed it is marked as a production-candidate specification, with validation and broker-specific integration still required, and written for MQL5 developers among others.
 That is the kind of work I do. I'm a trading bot developer working in MQL4/MQL5, and I could implement the specification as an EA: the higher-timeframe bias, liquidity sweep and CHoCH state machine, the sizing and risk rules, and broker-specific handling for gold symbols and stop levels, followed by structured backtests against the acceptance requirements you describe.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you are looking for someone to build it, would it be useful if I sent over a short example first?
 Best regards,
 Oseni Ibrahim
@@ -20672,7 +20486,6 @@
           <t>Hi Haseeb,
 I came across your XAUUSD SafeScalper EA on GitHub and saw that you take on custom EA development, strategy modifications and platform integrations.
 I'm a trading bot developer doing similar MQL4/MQL5 work: Expert Advisors, MT4 to MT5 conversion, TradingView and Telegram integrations, and fixing or maintaining existing bots. When several client requests land at once, it can help to have another developer to pass work to or to split a larger job with, for example you handle strategy logic while I cover an MT4 build or a Telegram alert module.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing a simple overflow arrangement? I can send examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -20746,7 +20559,6 @@
           <t>Hi Álvaro,
 I came across the B.E.N.D.E.R. showcase on GitHub and the Replicant copy-trading module, where each user picks a market and a broker, with IBKR and MT5 as options.
 As you expand beyond Nasdaq, the MT5 path tends to need the most care: CFD symbol names that differ per broker, contract sizes, lot steps and terminals that drop connection. I'm a trading bot developer working in MQL4/MQL5, and I could build the MT5 receiver for Replicant, an EA that takes signals from your server, maps symbols, applies per-user risk limits and reports fills back.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send a short example first.
 Best regards,
 Oseni Ibrahim
@@ -20820,7 +20632,6 @@
           <t>Hi iTrade.tools team,
 I came across QuickTrade on GitHub, the MT5 panel that combines execution, automated risk management and performance tracking, with auto partial close, breakeven offset and draggable entry, stop and target lines in v1.4.
 Since access is locked to specific account numbers and requested by email, two things often come next for tools like this: a smoother license flow, such as a key tied to the account and expiry, and an MT4 edition for traders on older brokers. I'm a trading bot developer working in MQL4/MQL5, and I could help with either, or with new panel features.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -20894,7 +20705,6 @@
           <t>Hi Vitaliy,
 I came across the Swing Zone project in your arena repo, with the KHUSA SM PRO structure engine and the two MQL5 pieces: SwingZone.mq5 for H4 levels and WebRequests to the bot, and ArenaFeed.mq5 for sending closed bars to the database.
 Those bridges tend to need care over time: retries when WebRequest fails, avoiding duplicate or missing bars after reconnects, and eventually executing trades directly from the zones. I'm a trading bot developer working in MQL4/MQL5, and I could help harden both components or add an execution module and MT4 support.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -20968,7 +20778,6 @@
           <t>Hi Haidra,
 I came across your profile and the projects listed there: the MT5 Manager REST API Copier, the Copy Trading C-Manager and the trading CRM with copy-trading rooms.
 Projects like these often pull in terminal-side work too, such as client-side EAs for MT4 and MT5 accounts, MT4 to MT5 migrations of older tools, or local risk guards. I'm a trading bot developer focused on MQL4/MQL5, and I could take on those pieces as a subcontractor while you keep the platform architecture and the client.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -21042,7 +20851,6 @@
           <t>Hi Sohaib,
 I came across your profile and the metaapi-balance-tracker project, streaming balance and equity from hundreds of MetaTrader accounts through MetaApi with rate limiting and circuit breakers.
 On projects like that, some clients eventually ask for a terminal-side option, either to cut per-account API costs or to get events without polling, for example a small MQL5 EA that pushes equity and trades to your backend, or copier and risk EAs running inside the terminal. I'm a trading bot developer focused on MQL4/MQL5, and I could handle that side as a subcontractor while you keep the platform work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -21121,7 +20929,6 @@
           <t>Hi Ans,
 I came across your profile and saw the freelance MT5 trading systems you build for a private group of Forex and Gold traders, as well as the modular FvgEA repo.
 Since your main work is Laravel and backend projects, there may be times when trader requests pile up: an MT4 version of a bot, Telegram alerts, a prop-style daily loss guard, or fixes after a broker change. I'm a trading bot developer focused on MQL4/MQL5, and I could take on those pieces as a subcontractor while you keep the client relationship.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -21195,7 +21002,6 @@
           <t>Hi TRADIVO team,
 I came across the TRADIVO V12 page in your algo2 repo and saw that you are positioning it as a professional MT5 Expert Advisor with built-in risk management and a simple setup.
 By version 12, most EA vendors are juggling buyer reports from different brokers, license handling and requests for new features or an MT4 build. I'm a trading bot developer working in MQL4/MQL5, and I could act as extra development capacity for TRADIVO, whether that means fixing broker-specific issues, adding account-based licensing, or preparing the next version.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a few examples of similar EA work?
 Best regards,
 Oseni Ibrahim
@@ -21264,7 +21070,6 @@
           <t>Hi 6amdev,
 I came across your profile and the FxBoat Quant Engine, the EA Factory that turns Python strategies into MT4, MT5 and TradingView bots with AI optimization.
 Generators like that tend to hit the same issues once real users run the output: broker-specific stop levels and filling modes, symbol suffixes, and MT4 versus MT5 order handling that the templates need to cover. I'm a trading bot developer working in MQL4/MQL5, and I could help harden the MQL templates, review generated EAs, or take on client builds that need hand-written MQL.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send over a few examples first.
 Best regards,
 Oseni Ibrahim
@@ -21338,7 +21143,6 @@
           <t>Hi there,
 I came across your TradingView and Pine Script services repo and saw that clients bring you ideas from many sources, including MT4 and MT5 tools, and you turn them into indicators, strategies and alerts.
 Some of those clients will also want the finished strategy running on MetaTrader, either as a native MQL5 EA or with TradingView alerts executing on MT5. That is my focus: I'm a trading bot developer working in MQL4/MQL5 and TradingView to MT5 integration. We could refer work both ways, or I could handle the MetaTrader side as a subcontractor while you keep the client.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can share examples of my work first.
 Best regards,
 Oseni Ibrahim
@@ -21412,7 +21216,6 @@
           <t>Hi Yassine,
 I came across TradePilot on GitHub, the copy-trading SaaS that mirrors trades between MetaTrader accounts in real time with per-account risk sizing, and saw the MT4 and MT5 EAs that connect to your WebSocket gateway.
 As more users connect, the EA side usually needs the most attention: reconnecting cleanly after terminal restarts, resolving broker symbols, handling partial closes and stop modifications, and reporting failed copies. I'm a trading bot developer working in MQL4/MQL5, and I could help harden and test those EAs while you focus on the platform.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it? I can send a short example first.
 Best regards,
 Oseni Ibrahim
@@ -21491,7 +21294,6 @@
           <t>Hi Artan,
 I found mt5-mac-data-bridge and liked the simple approach: an MQL5 EA writing JSON files so Python on macOS can work with MT5 without Wine or Docker. Most of the reliability of a setup like that lives in the EA, such as file locking, symbol handling and how commands are confirmed back.
 I'm an MQL5 developer and could help extend or harden that EA, for example with extra data files, partial closes and modifications in the command handler, or clearer error codes for the Python side. I'm happy to follow your existing contracts and naming.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -21565,7 +21367,6 @@
           <t>Hi Ali,
 I came across meta-five and the MT5 CRM described in its README, with client onboarding, payment gateways, bonuses and a web trader built on the MetaTrader 5 Web API. Brokers who buy a CRM like that often come back asking for work inside the terminal as well.
 I'm an MQL5 developer and could act as a partner for that side: EAs or scripts for bonus and credit handling, account reports, trade copiers between client accounts, or monitoring tools that feed your CRM. You keep the client, and I deliver the MetaTrader pieces to your spec.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's useful, I can send over a few examples of MT5 work.
 Best regards,
 Oseni Ibrahim
@@ -21639,7 +21440,6 @@
           <t>Hi Dogan,
 I found your Session Rectangle indicator for MT5, which draws Sydney, Tokyo, London and New York sessions and their overlaps. I also saw MQL5 indicators and Expert Advisors listed in your profile's current focus.
 Session tools often lead to requests for session-breakout EAs, alerts when a range forms or breaks, or MT4 versions. I'm an MQL4/MQL5 developer, and I could collaborate on any of those, either building the EA layer on top of your indicator or porting it for MT4 users.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -21713,7 +21513,6 @@
           <t>Hi Bipin,
 I came across RvFx, your MQL5 grid and hedge EA with its own cycle manager and live dashboard. Cycle-based grid systems usually need the most care in basket-level protection, such as equity stops, margin checks before each level, and how a cycle recovers after a restart.
 I'm an MQL5 developer and could review CycleManager.mqh with that in mind, add equity and margin guards, or connect the dashboard state to Telegram so you can follow cycles from your phone. I'd leave the strategy itself as you designed it.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -21787,7 +21586,6 @@
           <t>Hi Daniel,
 I read your algo-trading-portfolio showcase, eight or more systems in a private monorepo, including ARIES, the event-driven framework with live execution on MetaTrader 5. With that many systems, the MT5 connection layer tends to become shared infrastructure that needs its own care.
 I'm an MQL5 developer and could help there with a terminal-side EA for fills and account events, local risk guards, or MQL versions of strategies you want to check in the Strategy Tester. I'm glad to work under an NDA on the private code.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to discussing it?
 Best regards,
 Oseni Ibrahim
@@ -21861,7 +21659,6 @@
           <t>Hi Andrew,
 I came across your Meta-trader-trading-mq5 repository and the bullish continuation EA described in it. The entry rules are laid out clearly, which makes the strategy easy to build on.
 I'm an MQL5 developer and could help take it further: adding the short side, risk-based lot sizing, trailing and breakeven, running a proper Strategy Tester evaluation across symbols, and deploying it on a VPS with Telegram alerts. Given your DevOps background, I can fit into whatever deployment setup you prefer, and I'd keep your entry rules unchanged.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -21935,7 +21732,6 @@
           <t>Hi Senith,
 I came across BetterTrade and saw that it supports MetaTrader 5 history import and MT5 Auto Sync, alongside the App Store and Google Play releases. Sync with MT5 is usually the part that generates the most support questions, because brokers differ in history, commissions and symbol names.
 I'm an MQL4/MQL5 developer and could help with the terminal side, such as a sync EA that sends closed trades reliably, an MT4 version for users still on that platform, or broker edge-case fixes, so you can keep working on the app itself.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working on, I can send over a few examples.
 Best regards,
 Oseni Ibrahim
@@ -22014,7 +21810,6 @@
           <t>Hi Mathijs,
 I came across BetterMt5 on PyPI, your friendlier wrapper around the official MetaTrader5 Python library. It's a sensible idea, since the raw API is clunky to work with day to day.
 One gap I often see with Python-only wrappers is everything that lives inside the terminal: custom indicator buffers, EA-managed positions, chart events. I'm a MetaTrader developer working in MQL4/MQL5, and I could write small MQL5 companion pieces, for example an indicator exporter or a lightweight EA, that BetterMt5 users could pair with your library, or put together a few worked examples for your README.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of what an MQL5 counterpart for BetterMt5 might look like.
 Best regards,
 Oseni Ibrahim
@@ -22083,7 +21878,6 @@
           <t>Hi Contigion team,
 I noticed the contigion-metatrader package on PyPI, the library you use to retrieve forex data across the Contigion projects. It looks like MetaTrader is already a core data source for your work.
 I'm an MQL4/MQL5 developer, and projects like this often reach a point where some logic is better placed inside the terminal: an EA that executes signals generated in Python, an indicator that plots them on the chart, or Telegram alerts fired straight from MT5. I could help with that terminal side, or take on maintenance of the MetaTrader data layer as MT5 builds change.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of that fits where Contigion is heading, I can send over a few examples of similar Python-to-MT5 setups.
 Best regards,
 Oseni Ibrahim
@@ -22152,7 +21946,6 @@
           <t>Hi there,
 I noticed you maintain both forex-mcp, an MCP server for MT5 market data over SSE, and mt5proxy, an HTTP proxy for the MetaTrader 5 Python API. Both have had releases this year, so they're clearly still active.
 I'm an MQL5 developer, and one piece I could add is a small expert advisor inside the terminal. It would push trade events, custom indicator values or chart objects to your proxy, or run execution requests with proper retcode handling and risk checks on the MT5 side. That keeps the Python layer light and covers things the Python API can't see.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your roadmap, I can send over a short example of how an EA could talk to mt5proxy.
 Best regards,
 Oseni Ibrahim
@@ -22221,7 +22014,6 @@
           <t>Hi there,
 I came across metatrader-mcp-server on PyPI, the bridge that lets Claude and ChatGPT trade MetaTrader 5 in plain language, with REST and WebSocket interfaces as well. I've also noticed it has been forked and repackaged a few times, which says a lot about the demand.
 I'm an MQL5 developer. Some features users will likely ask for are easier from inside the terminal: drawing the AI's levels on the chart, reading custom indicator buffers, or a guard EA that enforces daily loss limits no matter what the agent sends. I could build those as optional MQL5 add-ons or write worked examples for your documentation.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of these?
 Best regards,
 Oseni Ibrahim
@@ -22290,7 +22082,6 @@
           <t>Hi there,
 I noticed mcp-mt5 on PyPI, your MCP server that lets an agent compile MQL, deploy EAs, run Strategy Tester and parse the reports without opening the MetaTrader UI. The analyze_mql and deprecated-call checks are a nice touch.
 A pipeline like this works best with good reference material. I'm an MQL4/MQL5 developer and could write a small set of sample expert advisors, including an MT4 one with deprecated calls for the migration check, plus matching tester .ini presets that exercise each tool end to end. They could live in your examples folder. I'm also open to picking up MQL work from users who adopt the pipeline.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds helpful, I can send over one sample EA to start.
 Best regards,
 Oseni Ibrahim
@@ -22364,7 +22155,6 @@
           <t>Hi Leo,
 I came across mt5-mcp-by-leo and mcp-mt5-conection on PyPI, with the MQL5 backend talking to Python over TCP sockets. Covering trades, graphic objects, terminal logs and compilation through MCP is an ambitious scope.
 Keeping both the Python framework and the MQL5 socket side moving is a lot for one person. I'm an MQL4/MQL5 developer and could take on backend pieces as a subcontractor: new socket commands, JSON handling, reconnection logic, or extra tools such as indicator buffer reads and chart snapshots. You'd keep full control of the design and get clean source back.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If you're open to outside help on the MQL5 side, would you like me to send a short example of socket-handling code?
 Best regards,
 Oseni Ibrahim
@@ -22438,7 +22228,6 @@
           <t>Hi Pavel,
 I came across mt4ctl, your MCP server for running headless MetaTrader 4 terminals under Wine and systemd over SSH. The headless first-login flow and per-EA AutoTrading status solve real pain for anyone running a VPS fleet.
 One piece that pairs well with it is a small heartbeat EA inside each terminal. It would write connection state, last tick, open trades and errors to a file or socket that mt4ctl reads, so the agent sees what the EAs are actually doing, not only whether the process is up. I'm an MQL4/MQL5 developer and could build it for both MT4 and MT5 if you plan to extend the tool.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -22512,7 +22301,6 @@
           <t>Hi Paulo,
 I came across mt5se, your Python framework for autonomous traders that reaches B3, NYSE and Nasdaq through MetaTrader. It's good to see it still getting releases this year, a long time after mt5b3.
 I'm an MQL5 developer and could add the terminal side of that picture. That might be an EA that runs an mt5se-trained model's decisions directly in MT5, an indicator that plots the agent's signals for review, or a few MQL5 examples for your documentation showing how the two sides interact. For students or users working with Brazilian brokers, that could make the framework easier to adopt.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If any of this is interesting, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -22586,7 +22374,6 @@
           <t>Hi there,
 I noticed mt5-bridge on PyPI, the FastAPI service and CLI that lets clients on any OS reach an MT5 terminal running on Windows. The recent release suggests people are actually using it.
 I'm an MQL5 developer. A bridge like this can be extended from the terminal side: a small EA that pushes trade and account events to the API instead of relying on polling, exposes custom indicator values, or blocks orders that break configured risk limits. I could build that as an optional companion, or write a couple of examples for the README showing a strategy running end to end.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example?
 Best regards,
 Oseni Ibrahim
@@ -22660,7 +22447,6 @@
           <t>Hi Soham,
 I came across MT5Forge on PyPI. The idea that a strategy only decides BUY, SELL or HOLD while the framework handles sessions, risk, notifications and monitoring is a clean way to organise MT5 bots.
 A common next request from users of Python frameworks is to check the same logic in MT5's own Strategy Tester, or to run it natively on a VPS. I'm an MQL5 developer and could write an MQL5 template that mirrors your strategy interface, so a MT5Forge strategy can be ported and compared, or provide a few examples for your readthedocs pages.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds worthwhile, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -22734,7 +22520,6 @@
           <t>Hi Slava,
 I came across mt5-grpc-server and mt5-grpc-proto on PyPI. Putting a typed gRPC API with TLS in front of MetaTrader 5 is a clean approach for remote trading and market depth access.
 Something that often comes up with Python-API servers is real-time events: trade transactions, order fills and custom indicator updates, which the Python package can only poll. I'm an MQL5 developer and could build a small EA that emits those events from OnTradeTransaction to your server, or write an example strategy client for the docs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short sketch of how that EA could plug into your proto definitions?
 Best regards,
 Oseni Ibrahim
@@ -22808,7 +22593,6 @@
           <t>Hi Brian,
 I saw mt5-lite on PyPI, your object-oriented wrapper around the official MetaTrader 5 package. Mapping MT5 error codes to Python exceptions is the kind of detail that saves people a lot of debugging.
 I'm an MQL4/MQL5 developer, and I work on the terminal side that the Python API can't reach: expert advisors, custom indicators, trade copiers and Telegram alerts sent from MT5. If users of mt5-lite ask for something that needs code inside MetaTrader, or you take on client projects that need an MQL component, I'd be glad to collaborate or take that part on.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of my work.
 Best regards,
 Oseni Ibrahim
@@ -22882,7 +22666,6 @@
           <t>Hi Abdul,
 I came across mt5_mac on PyPI. Using the Wine runtime already bundled inside MetaTrader 5.app, with no Docker or Windows box, is a clever route for Mac traders.
 I noticed indicator reading currently covers Heiken Ashi computed from OHLC. I'm an MQL5 developer, and one extension would be a small MQL5 exporter indicator that writes any chart indicator's buffers, including custom or paid ones, to a file your library reads. Users would get the exact values MT5 shows rather than a recalculation. I could also write example EAs for the docs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of that exporter?
 Best regards,
 Oseni Ibrahim
@@ -22956,7 +22739,6 @@
           <t>Hi Theau,
 I came across mt5-mac-bridge on PyPI. Having bridge, mock and native backends behind one identical API is a thoughtful design, and the README mentions it sits inside your own MOMQ trading project.
 If MOMQ ever needs something that runs inside the terminal, I could help. Examples are an MQL5 guard EA that enforces stops or daily loss limits even when the Python side disconnects, or an indicator that exports values the Python API can't read. I'm a MetaTrader developer working in MQL4/MQL5 and focus on that terminal side.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that would help, I can send over a short example of a guard EA.
 Best regards,
 Oseni Ibrahim
@@ -23030,7 +22812,6 @@
           <t>Hi Raimi,
 I saw that MT5pytrader is heading into 2.0, with structured TradeResult objects, broker preflight checks and bounded client-side trailing stops. Handling partial closes by the broker's volume step is a detail many libraries skip.
 Since the trailing stop runs client-side, it only works while the Python process is alive. I'm an MQL5 developer and could build a small companion EA that takes over break-even and trailing inside the terminal, driven by magic number or comment, so positions stay managed if the script stops. It could be an optional add-on for your docs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would you be open to me sending over a short example?
 Best regards,
 Oseni Ibrahim
@@ -23099,7 +22880,6 @@
           <t>Hi there,
 I came across mt5-trading-lib on PyPI. An async MetaTrader 5 client with a circuit breaker, TTL caching and encrypted credentials goes well beyond the usual thin wrapper.
 One area Python can't fully cover is what happens inside the terminal: trade transaction events, custom indicator values, or protective logic that must keep working if the client disconnects. I'm an MQL5 developer and could build a small companion expert advisor that pushes events to your event-driven layer, or a guard EA that enforces stops independently. Both could be optional extras for your users.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23173,7 +22953,6 @@
           <t>Hi Vincent,
 I came across mt5-trading-mcp and liked the consent and audit layer in front of real trades. I also noticed you already use a small MQL5 expert advisor, AgentScreenshot, for native chart captures.
 Since part of the project already lives in MQL5, there may be room for more there. One option is an EA-side risk guard that rejects or closes positions outside limits even if the agent misbehaves. Another is an exporter for custom indicator buffers, or chart annotations that show the agent's reasoning. I'm an MQL4/MQL5 developer and could help build or maintain those pieces.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one?
 Best regards,
 Oseni Ibrahim
@@ -23247,7 +23026,6 @@
           <t>Hi Krunal,
 I came across nostro_mt5_manager on PyPI, your Python wrapper for the MetaTrader 5 Manager API, along with its GitBook docs. Manager API work usually means you're close to brokers or prop setups running their own MT5 servers.
 Those clients often need terminal-side tools as well: expert advisors, trade copiers, equity and drawdown guards, or MT4-to-MT5 ports of older code. I'm an MQL4/MQL5 developer and could act as extra capacity for that side of your projects, working to your specifications while you stay focused on the Manager API layer.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that could be useful, I can send over a few examples of related work.
 Best regards,
 Oseni Ibrahim
@@ -23316,7 +23094,6 @@
           <t>Hi there,
 I came across Py2MQL5 on PyPI, the wrapper that lets the official MetaTrader5 package drive several portable terminals at once. That's a real limitation of the stock package, so the workaround is useful.
 People running many terminals side by side often also need something inside each one: a local trade copier between accounts, a monitoring EA that reports equity and connection state, or per-account risk guards. I'm an MQL4/MQL5 developer and build those terminal-side tools. They could complement Py2MQL5 for multi-account users or serve as examples in your docs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If this is something you're working with, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23390,7 +23167,6 @@
           <t>Hi Henrique,
 I came across pymt5linux and your mt5docker image. Keeping MT5 on Linux working across terminal updates is thankless work, and moving it to Python 3.13 is appreciated by people who run it headless.
 In headless setups it helps to have something inside the terminal reporting back. I'm an MQL5 developer and could build a small heartbeat EA that writes connection state, last tick time and open positions to a file or socket, so a container health check can tell whether trading is really live. It could ship as an optional example alongside mt5docker.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -23459,7 +23235,6 @@
           <t>Hi there,
 I came across PythonMetaTrader5 on PyPI. Accepting SL and TP either as absolute prices or point offsets, with normalisation to the symbol's digits, removes a common source of rejected orders.
 I noticed pyautogui in the dependencies, which usually means some actions can't be done through the Python API alone. I'm an MQL5 developer, and a small companion EA can often take over those steps, such as chart handling, indicator reads or protective closes, by listening to commands from Python through files or sockets. That tends to be more reliable than GUI automation.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's relevant, I can send over a short example of how it would work.
 Best regards,
 Oseni Ibrahim
@@ -23533,7 +23308,6 @@
           <t>Hi Mahmudul,
 I came across shawon-mt5-automation on PyPI, your Flask webhook server that turns TradingView alerts into MT5 trades with API-key auth, USD-based SL/TP and signal gap control.
 TradingView-to-MT5 is a big part of my work as an MQL4/MQL5 developer. Some clients prefer an EA-side receiver that handles partial closes, break-even, trailing and per-symbol risk inside the terminal, next to a webhook layer like yours. If you take on client projects in this area, I'd be glad to collaborate on the MQL side or take overflow work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example of an EA-side receiver.
 Best regards,
 Oseni Ibrahim
@@ -23607,7 +23381,6 @@
           <t>Hi Bahadir,
 I came across SiliconMetaTrader5, the Docker-based way to run MT5 with Python on Apple Silicon. I liked that the README is honest about using a native Windows server for live, high-capital trading.
 That handoff from Mac development to live deployment is where I usually help. I'm an MQL4/MQL5 developer and can port a strategy prototyped in Python into a native MQL5 expert advisor, set it up on a Windows VPS, and add monitoring. If your users ask about that step, or you have strategies of your own to move, I could be a useful contact.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it help if I sent over a short example of a Python-to-MQL5 port?
 Best regards,
 Oseni Ibrahim
@@ -23681,7 +23454,6 @@
           <t>Hi there,
 I came across n8n-nodes-metatrader5 on npm and noticed its repository sits on BlackBull Markets' GitHub Enterprise. An n8n node is a friendly way to open MT5 automation to traders who don't write code.
 I'm an MQL4/MQL5 developer. Workflows like these often need something inside the terminal as well: an EA that receives n8n webhooks and executes with proper lot and risk checks, or one that pushes fills and equity changes back into a workflow. I could build those as companion pieces or as example templates for the node's documentation.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23755,7 +23527,6 @@
           <t>Hi there,
 I noticed n8n-nodes-ohlcv-metatrader on npm, which pulls MetaTrader candles, gold included, into n8n workflows next to crypto exchange data.
 Once the analysis runs in n8n, the next question is usually how to act on it inside MetaTrader. I'm an MQL4/MQL5 developer and could build a small EA that takes decisions from a workflow via webhook or file, places orders with lot sizing and SL/TP, and reports results back. It could work as a companion to your node or as an example workflow in the README.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -23824,7 +23595,6 @@
           <t>Hi mt5cli team,
 I came across mt5cli on npm, the Docker-first MetaTrader 5 CLI for headless Linux with EA and backtest support and no dependencies.
 A tool like this is only as convincing as its first run, so good sample material helps. I'm an MQL5 developer and could write a couple of reference expert advisors with matching tester presets that demonstrate compiling, running a backtest and reading results through the CLI. If your users bring their own EAs that fail to compile or behave differently headless, I'm also happy to take that work on.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over one sample EA to try.
 Best regards,
 Oseni Ibrahim
@@ -23898,7 +23668,6 @@
           <t>Hi Altug,
 I came across metatrader5-sdk on npm, your Node.js SDK for the MetaTrader 5 Web API. It's a useful bridge for JavaScript teams that don't want to touch Python or MQL.
 Web API integrations handle accounts and trades well, but some features only run inside the terminal: custom indicators, EA-side risk rules and chart objects. I'm an MQL4/MQL5 developer and could write companion EAs or examples for your README showing how a Node app and an MT5 expert advisor work together. I can also help if you take on client work that needs an MQL component.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's of interest, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -23972,7 +23741,6 @@
           <t>Hi Halit,
 I came across biquote, the free market data API and SDKs. Offering 15,000 requests a minute with no API key is generous, and I noticed the prices come from a MetaTrader 5 feed.
 I'm an MQL4/MQL5 developer, and for a service like this the terminal-side collector matters a lot. I could help harden the feed EA with reconnection handling, stale-tick detection and heartbeat alerts, add symbols or brokers, or write an MQL5 client example so MT5 users can pull biquote's economic calendar straight into their EAs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of these?
 Best regards,
 Oseni Ibrahim
@@ -24046,7 +23814,6 @@
           <t>Hi Gil,
 I came across mt4manager on npm, your Node-API bindings for the MetaTrader 4 Manager API. Giving brokerage back-office teams a TypeScript interface instead of raw C++ is a good call.
 Brokers using tools like this often have MQL work too, such as client EAs, copier tools, risk scripts, or moving existing MT4 code to MT5 as they migrate servers. I'm an MQL4/MQL5 developer and could take on that side for your clients, or write terminal-side test EAs that generate realistic trading activity while you test the pumping and event APIs.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few relevant examples.
 Best regards,
 Oseni Ibrahim
@@ -24120,7 +23887,6 @@
           <t>Hi Mauro,
 I noticed @mautriz/mt5 on npm, the TypeScript client for your MetaTrader 5 WebSocket API. Streaming MT5 over WebSockets with a typed client is a practical setup for web dashboards and bots.
 Services like this usually rely on something inside the terminal, often an MQL5 EA or bridge, that has to keep working through MT5 build changes. I'm an MQL4/MQL5 developer and could help build or maintain that side, add events such as trade transactions or indicator values, or write example EAs for your documentation.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's relevant to what you're building, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -24189,7 +23955,6 @@
           <t>Hi TradeRail team,
 I came across the traderail SDK on npm for your managed MetaTrader 5 API, including the copy-trading side. A hosted MT5 API spares developers a lot of Windows and terminal setup.
 Customers of managed APIs often come back with requests that sit inside MetaTrader: a custom EA, a copier variant with special lot rules, or equity and drawdown guards. I'm an MQL4/MQL5 developer and could be the person you refer that work to, or build example strategies that show the SDK and an MT5 EA working together.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a few examples of similar work.
 Best regards,
 Oseni Ibrahim
@@ -24258,7 +24023,6 @@
           <t>Hi there,
 I came across synapse-mt5 on npm, the native C++ MCP server that connects AI assistants to MetaTrader 5 without Python. The repo name, MCP-MQL5, suggests a good share of the work happens on the MQL5 side.
 I'm an MQL4/MQL5 developer and could help extend that part: new tools for indicator buffers or chart objects, EA-side risk limits the AI can't bypass, or MT4 support if users ask for it. I'm happy to work within your architecture and hand back clean source.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example of one of those tools?
 Best regards,
 Oseni Ibrahim
@@ -24327,7 +24091,6 @@
           <t>Hi there,
 I came across StrategyLab on npm, your AI-powered EA development framework for MetaTrader 5 built around Claude Code. Having a structured workflow instead of prompting from scratch makes a lot of sense.
 AI-written EAs tend to fail in similar places: order filling modes, broker stop levels, netting versus hedging accounts, and new-bar detection. I'm an MQL4/MQL5 developer and could act as a human review and fix step for EAs produced with StrategyLab, or write hand-checked template EAs the framework could start from.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that fits your plans, I can send over a short checklist and an example.
 Best regards,
 Oseni Ibrahim
@@ -24396,7 +24159,6 @@
           <t>Hi there,
 I came across mt5-quant-forex-panel on npm, your MetaTrader 5 quant panel with ten backtested strategies, a multi-signal core and a live dashboard.
 Some users will want to run those strategies natively in MT5, to confirm them in the Strategy Tester with real tick data or to keep them running on a VPS without the panel. I'm an MQL4/MQL5 developer and could port selected strategies into MQL5 expert advisors that follow your logic and parameters, with risk limits enforced inside the terminal.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's interesting, I can send over a short example of a ported strategy.
 Best regards,
 Oseni Ibrahim
@@ -24470,7 +24232,6 @@
           <t>Hi Clawtrade team,
 I came across Clawtrade, the self-hosted AI trading agent platform that brings crypto venues, Interactive Brokers and MetaTrader 5 together in one dashboard.
 The MT5 connector runs through the Python API, which works but brings forex-specific surprises: broker symbol suffixes, filling modes, stop levels and netting versus hedging accounts. I'm an MQL4/MQL5 developer and could help make that module sturdier, or add an optional MQL5 EA that executes agent decisions inside the terminal with its own risk checks. It would stay independent of the agent loop, so stops still apply if the server restarts.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -24544,7 +24305,6 @@
           <t>Hi Peter,
 I came across your metatrader4 package for trading MT4 from Node.js. I noticed the setup depends on dingmaotu's mql4-lib and mql-zmq, copied by hand into the MQL4 folders.
 Those libraries are not very active anymore, and many brokers are moving clients to MT5. I'm an MQL4/MQL5 developer and could build an MT5 version of the bridge EA using the same message format, or simplify the MT4 install so it needs fewer external pieces. That would let your Node.js API cover both platforms.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds useful, I can send over a short example.
 Best regards,
 Oseni Ibrahim
@@ -24613,7 +24373,6 @@
           <t>Hi there,
 I came across @0xrelogic/mt5-analysis-mcp on npm, with analysis tools, trading operations and a 15-condition alert system for MT5. I also noticed the recent pip value calculation fix.
 Pip and tick values are easy to get wrong outside the terminal, especially for metals, indices and non-USD accounts. I'm an MQL5 developer and could build a small helper EA that returns the terminal's own tick value, contract size and margin figures, and can also run your alert conditions inside MT5 so they fire even when the MCP server is idle.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -24682,7 +24441,6 @@
           <t>Hi there,
 I came across @herjarsa/mt5-mcp-super on npm, the one-command installer that sets up your MT5 MCP server in Claude Code, OpenCode, Codex and Gemini CLI. Making setup that easy should bring in a lot of MT5 traders.
 Many of them will soon ask for things that only work inside the terminal: custom indicator values, chart drawings from the agent, or an EA that enforces risk limits whatever the agent sends. I'm an MQL4/MQL5 developer and could build those as companion pieces for the server.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a short example?
 Best regards,
 Oseni Ibrahim
@@ -24751,7 +24509,6 @@
           <t>Hi there,
 I came across mql5-mcp on npm, which lets an agent compile and test expert advisors and indicators. Closing the loop between writing MQL5 and seeing compiler and tester output is what makes AI-assisted EA work usable.
 I'm an MQL4/MQL5 developer and could help in two ways: a set of small reference EAs and indicators with known expected results that serve as tests and docs examples, and a human review step for tricky cases the agent keeps getting wrong, such as filling modes, stop levels and multi-symbol handling.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds helpful, I can send over one reference EA to start.
 Best regards,
 Oseni Ibrahim
@@ -24820,7 +24577,6 @@
           <t>Hi there,
 I came across mql5-ea-mcp, your MCP server that indexes the MQL5 help, the Algo Book and the Neural Networks Book, with an error database for diagnosing EA problems.
 The most useful error entries usually come from live accounts rather than the docs: invalid stops from broker freeze levels, unsupported filling modes, netting account surprises, and 4756 or 10030 codes. I'm an MQL4/MQL5 developer and could contribute a set of these real cases with fixes, and I'm also open to working together on EA client projects.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a few sample entries?
 Best regards,
 Oseni Ibrahim
@@ -24894,7 +24650,6 @@
           <t>Hi IndexNano team,
 I came across @indexnano/mt5-ws on npm, the WebSocket SDK for your MT5 API with real-time orders and quotes.
 Services like this usually depend on something inside MetaTrader that has to stay reliable through terminal updates, and customers soon ask for extras such as custom EAs, trade copiers or risk guards next to their API integration. I'm an MQL4/MQL5 developer and could help with that terminal side, or take the MQL requests your customers bring in, working under your brand and to your specifications.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's relevant, I can send over a few examples of similar work.
 Best regards,
 Oseni Ibrahim
@@ -24968,7 +24723,6 @@
           <t>Hi Charles-Antoine,
 I came across tree-sitter-mql5 on npm. A proper Tree-sitter grammar for MQL5 is something the community has long lacked for editors and code tools.
 Grammars tend to break on the odd parts of the language: D'...' and C'...' literals, input groups, #property lines, templates, #import blocks and MT4-style code that still compiles in MT5. I'm an MQL4/MQL5 developer with a lot of real EA and indicator code, and I could put together a varied test corpus of these cases. I'm also open to working together on MQL-related projects.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a first batch of test files?
 Best regards,
 Oseni Ibrahim
@@ -25037,7 +24791,6 @@
           <t>Hi there,
 I came across your mql5-json, mql5-promise and mql5-timer packages. Shipping MQL5 libraries through npm, and bringing a Promise-style interface into MQL5, is an unusual approach that I liked.
 I'm also an MQL4/MQL5 developer, working on expert advisors, trade copiers, Telegram and webhook integrations. If you or the HommaTech mql-simplify project ever need extra hands, whether on client EAs or on new modules like an HTTP/WebRequest wrapper built on your promise library, I'd be glad to collaborate or take on subcontracted work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that sounds interesting, I can send over a few examples of my code.
 Best regards,
 Oseni Ibrahim
@@ -25111,7 +24864,6 @@
           <t>Hi Hristiyan,
 I came across mql5-lib on npm, the MQL5 language definitions for C++ IDEs. Being able to write MQL5 in a proper IDE with completion, instead of MetaEditor, is something many of us want.
 I'm an MQL4/MQL5 developer and could help test the definitions against real EA and indicator code, trade classes, chart objects and event handlers, and report or fix the gaps. I'm also open to collaborating or taking on overflow if you do client MQL5 work.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 If that's useful, I can send over a sample set of files to test against.
 Best regards,
 Oseni Ibrahim
@@ -25180,7 +24932,6 @@
           <t>Hi there,
 I came across mql-interpreter on npm, a TypeScript lexer, parser, semantic checker and runtime for running MQL4/5 in Node.js. That's a big undertaking.
 As the built-in stubs grow, a reliable reference helps: real EAs and scripts with known outputs from MetaTrader itself, covering OrderSend and CTrade behaviour, series indexing, ArraySetAsSeries and similar quirks. I'm an MQL4/MQL5 developer and could build a corpus like that, and help check how built-ins behave in the real terminal, including differences between MT4 and MT5 builds.
-Just so you know upfront, I work on a paid, per-project basis and can send a fixed quote once I've seen the scope.
 Would it be useful if I sent over a first set of reference scripts?
 Best regards,
 Oseni Ibrahim

</xml_diff>

<commit_message>
Outreach batch 3: 23 sent, 2 skipped
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -6535,7 +6535,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
@@ -6613,7 +6613,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -6696,7 +6696,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -6862,7 +6862,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Skipped possible sanctions (2026-09-28 20:37 UTC)</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -7247,7 +7247,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -7403,7 +7403,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -7476,7 +7476,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
@@ -7554,7 +7554,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -7715,7 +7715,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
@@ -7793,7 +7793,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -7872,7 +7872,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -7951,7 +7951,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
@@ -8030,7 +8030,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -8109,7 +8109,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -8188,7 +8188,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -8272,7 +8272,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -8350,7 +8350,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Skipped already contacted (2026-09-28 20:38 UTC)</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-28 20:38 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -24980,7 +24980,6 @@
       </c>
     </row>
     <row r="328">
-      <c r="A328" t="inlineStr"/>
       <c r="B328" t="inlineStr">
         <is>
           <t>ATJ Traders</t>
@@ -25012,7 +25011,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr"/>
       <c r="I328" t="inlineStr">
         <is>
           <t>Trading education / MT5 tooling</t>
@@ -25050,7 +25048,6 @@
       </c>
     </row>
     <row r="329">
-      <c r="A329" t="inlineStr"/>
       <c r="B329" t="inlineStr">
         <is>
           <t>PyneSys (PyneCore)</t>
@@ -25082,7 +25079,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr"/>
       <c r="I329" t="inlineStr">
         <is>
           <t>Trading technology / Pine Script tooling</t>
@@ -25120,7 +25116,6 @@
       </c>
     </row>
     <row r="330">
-      <c r="A330" t="inlineStr"/>
       <c r="B330" t="inlineStr">
         <is>
           <t>Backtest360</t>
@@ -25152,7 +25147,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr"/>
       <c r="I330" t="inlineStr">
         <is>
           <t>Backtesting SaaS / API</t>
@@ -25190,7 +25184,6 @@
       </c>
     </row>
     <row r="331">
-      <c r="A331" t="inlineStr"/>
       <c r="B331" t="inlineStr">
         <is>
           <t>AlpacaCode</t>
@@ -25222,7 +25215,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H331" t="inlineStr"/>
       <c r="I331" t="inlineStr">
         <is>
           <t>Trading software / CLI</t>
@@ -25260,7 +25252,6 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" t="inlineStr"/>
       <c r="B332" t="inlineStr">
         <is>
           <t>Bond Labs</t>
@@ -25292,7 +25283,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H332" t="inlineStr"/>
       <c r="I332" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -25330,7 +25320,6 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" t="inlineStr"/>
       <c r="B333" t="inlineStr">
         <is>
           <t>Radius Red (tradedesk)</t>
@@ -25404,7 +25393,6 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" t="inlineStr"/>
       <c r="B334" t="inlineStr">
         <is>
           <t>Alleyway Apps (Alertz Manager)</t>
@@ -25436,7 +25424,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H334" t="inlineStr"/>
       <c r="I334" t="inlineStr">
         <is>
           <t>Trading automation tools</t>
@@ -25510,7 +25497,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr"/>
       <c r="I335" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -25626,13 +25612,11 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" t="inlineStr"/>
       <c r="B337" t="inlineStr">
         <is>
           <t>v33 Systematic</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr"/>
       <c r="D337" t="inlineStr">
         <is>
           <t>btc@v33systematic.com</t>
@@ -25654,7 +25638,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H337" t="inlineStr"/>
       <c r="I337" t="inlineStr">
         <is>
           <t>Systematic crypto trading</t>
@@ -25692,7 +25675,6 @@
       </c>
     </row>
     <row r="338">
-      <c r="A338" t="inlineStr"/>
       <c r="B338" t="inlineStr">
         <is>
           <t>PineForge (4pass)</t>
@@ -25766,7 +25748,6 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="inlineStr"/>
       <c r="B339" t="inlineStr">
         <is>
           <t>Gunbot</t>
@@ -25798,7 +25779,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H339" t="inlineStr"/>
       <c r="I339" t="inlineStr">
         <is>
           <t>Trading bot software</t>
@@ -25836,7 +25816,6 @@
       </c>
     </row>
     <row r="340">
-      <c r="A340" t="inlineStr"/>
       <c r="B340" t="inlineStr">
         <is>
           <t>AlgoVault</t>
@@ -25868,7 +25847,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H340" t="inlineStr"/>
       <c r="I340" t="inlineStr">
         <is>
           <t>Crypto trading signals</t>
@@ -25906,7 +25884,6 @@
       </c>
     </row>
     <row r="341">
-      <c r="A341" t="inlineStr"/>
       <c r="B341" t="inlineStr">
         <is>
           <t>Quotient (Cassie)</t>
@@ -25938,7 +25915,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H341" t="inlineStr"/>
       <c r="I341" t="inlineStr">
         <is>
           <t>Trading bots / forecasting signals</t>
@@ -25976,7 +25952,6 @@
       </c>
     </row>
     <row r="342">
-      <c r="A342" t="inlineStr"/>
       <c r="B342" t="inlineStr">
         <is>
           <t>BlockRun (Franklin Trading)</t>
@@ -26008,7 +25983,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H342" t="inlineStr"/>
       <c r="I342" t="inlineStr">
         <is>
           <t>AI trading agent</t>
@@ -26046,7 +26020,6 @@
       </c>
     </row>
     <row r="343">
-      <c r="A343" t="inlineStr"/>
       <c r="B343" t="inlineStr">
         <is>
           <t>ProEA</t>
@@ -26078,7 +26051,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H343" t="inlineStr"/>
       <c r="I343" t="inlineStr">
         <is>
           <t>Trading tools / Pine Script</t>
@@ -26152,7 +26124,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H344" t="inlineStr"/>
       <c r="I344" t="inlineStr">
         <is>
           <t>Algorithmic trading platform</t>
@@ -26304,7 +26275,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H346" t="inlineStr"/>
       <c r="I346" t="inlineStr">
         <is>
           <t>AI agents / trading technology</t>
@@ -26342,7 +26312,6 @@
       </c>
     </row>
     <row r="347">
-      <c r="A347" t="inlineStr"/>
       <c r="B347" t="inlineStr">
         <is>
           <t>LangMart</t>
@@ -26374,7 +26343,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H347" t="inlineStr"/>
       <c r="I347" t="inlineStr">
         <is>
           <t>Trading infrastructure</t>
@@ -26412,7 +26380,6 @@
       </c>
     </row>
     <row r="348">
-      <c r="A348" t="inlineStr"/>
       <c r="B348" t="inlineStr">
         <is>
           <t>Idea Design Media</t>
@@ -26444,7 +26411,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H348" t="inlineStr"/>
       <c r="I348" t="inlineStr">
         <is>
           <t>Software development agency</t>
@@ -26519,7 +26485,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H349" t="inlineStr"/>
       <c r="I349" t="inlineStr">
         <is>
           <t>Systematic trading / validation tooling</t>
@@ -26557,7 +26522,6 @@
       </c>
     </row>
     <row r="350">
-      <c r="A350" t="inlineStr"/>
       <c r="B350" t="inlineStr">
         <is>
           <t>PineAFL</t>
@@ -26590,7 +26554,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H350" t="inlineStr"/>
       <c r="I350" t="inlineStr">
         <is>
           <t>Algo development services</t>
@@ -26744,7 +26707,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H352" t="inlineStr"/>
       <c r="I352" t="inlineStr">
         <is>
           <t>Trading analytics</t>
@@ -26782,7 +26744,6 @@
       </c>
     </row>
     <row r="353">
-      <c r="A353" t="inlineStr"/>
       <c r="B353" t="inlineStr">
         <is>
           <t>Quantiota</t>
@@ -26815,7 +26776,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H353" t="inlineStr"/>
       <c r="I353" t="inlineStr">
         <is>
           <t>Quant research / trading technology</t>
@@ -26890,7 +26850,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H354" t="inlineStr"/>
       <c r="I354" t="inlineStr">
         <is>
           <t>Software development studio</t>
@@ -26928,7 +26887,6 @@
       </c>
     </row>
     <row r="355">
-      <c r="A355" t="inlineStr"/>
       <c r="B355" t="inlineStr">
         <is>
           <t>NexusTrader (Quantweb3)</t>
@@ -26961,7 +26919,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H355" t="inlineStr"/>
       <c r="I355" t="inlineStr">
         <is>
           <t>Trading execution software</t>
@@ -26999,7 +26956,6 @@
       </c>
     </row>
     <row r="356">
-      <c r="A356" t="inlineStr"/>
       <c r="B356" t="inlineStr">
         <is>
           <t>Quvanti Labs</t>
@@ -27032,7 +26988,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H356" t="inlineStr"/>
       <c r="I356" t="inlineStr">
         <is>
           <t>Trading strategy SaaS</t>
@@ -27106,7 +27061,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H357" t="inlineStr"/>
       <c r="I357" t="inlineStr">
         <is>
           <t>Futures trading technology</t>
@@ -27180,7 +27134,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr"/>
       <c r="I358" t="inlineStr">
         <is>
           <t>Trading technology (AI research &amp; execution)</t>
@@ -27218,7 +27171,6 @@
       </c>
     </row>
     <row r="359">
-      <c r="A359" t="inlineStr"/>
       <c r="B359" t="inlineStr">
         <is>
           <t>StreamXLS</t>
@@ -27250,7 +27202,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H359" t="inlineStr"/>
       <c r="I359" t="inlineStr">
         <is>
           <t>Trading software (IBKR data to Excel)</t>
@@ -27324,7 +27275,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H360" t="inlineStr"/>
       <c r="I360" t="inlineStr">
         <is>
           <t>Trading software (multi-account IBKR)</t>
@@ -27398,7 +27348,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H361" t="inlineStr"/>
       <c r="I361" t="inlineStr">
         <is>
           <t>Prop trading tools</t>
@@ -27436,7 +27385,6 @@
       </c>
     </row>
     <row r="362">
-      <c r="A362" t="inlineStr"/>
       <c r="B362" t="inlineStr">
         <is>
           <t>Roq GmbH</t>
@@ -27468,7 +27416,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H362" t="inlineStr"/>
       <c r="I362" t="inlineStr">
         <is>
           <t>Trading technology (low-latency gateways)</t>
@@ -27506,7 +27453,6 @@
       </c>
     </row>
     <row r="363">
-      <c r="A363" t="inlineStr"/>
       <c r="B363" t="inlineStr">
         <is>
           <t>Open Byte Inc. (QuantDinger)</t>
@@ -27538,7 +27484,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H363" t="inlineStr"/>
       <c r="I363" t="inlineStr">
         <is>
           <t>Trading software (AI trading OS)</t>
@@ -27612,7 +27557,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H364" t="inlineStr"/>
       <c r="I364" t="inlineStr">
         <is>
           <t>Algorithmic trading (futures order flow)</t>
@@ -27650,7 +27594,6 @@
       </c>
     </row>
     <row r="365">
-      <c r="A365" t="inlineStr"/>
       <c r="B365" t="inlineStr">
         <is>
           <t>ATHEIST AI</t>
@@ -27682,7 +27625,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H365" t="inlineStr"/>
       <c r="I365" t="inlineStr">
         <is>
           <t>Trading technology (AI execution)</t>
@@ -27756,7 +27698,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H366" t="inlineStr"/>
       <c r="I366" t="inlineStr">
         <is>
           <t>Trading journal SaaS</t>
@@ -27794,7 +27735,6 @@
       </c>
     </row>
     <row r="367">
-      <c r="A367" t="inlineStr"/>
       <c r="B367" t="inlineStr">
         <is>
           <t>TradingApp.Store</t>
@@ -27826,7 +27766,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H367" t="inlineStr"/>
       <c r="I367" t="inlineStr">
         <is>
           <t>Trading software licensing marketplace</t>
@@ -27864,7 +27803,6 @@
       </c>
     </row>
     <row r="368">
-      <c r="A368" t="inlineStr"/>
       <c r="B368" t="inlineStr">
         <is>
           <t>Drakkar-Software (OctoBot)</t>
@@ -28016,13 +27954,11 @@
       </c>
     </row>
     <row r="370">
-      <c r="A370" t="inlineStr"/>
       <c r="B370" t="inlineStr">
         <is>
           <t>Fianchetto Labs</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr"/>
       <c r="D370" t="inlineStr">
         <is>
           <t>aleks@fianchettolabs.com</t>
@@ -28044,7 +27980,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H370" t="inlineStr"/>
       <c r="I370" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -28082,7 +28017,6 @@
       </c>
     </row>
     <row r="371">
-      <c r="A371" t="inlineStr"/>
       <c r="B371" t="inlineStr">
         <is>
           <t>Sigma Quantiphi</t>
@@ -28114,7 +28048,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H371" t="inlineStr"/>
       <c r="I371" t="inlineStr">
         <is>
           <t>Crypto trading technology</t>
@@ -28188,7 +28121,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H372" t="inlineStr"/>
       <c r="I372" t="inlineStr">
         <is>
           <t>Trading API SDKs</t>
@@ -28262,7 +28194,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H373" t="inlineStr"/>
       <c r="I373" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -28336,7 +28267,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H374" t="inlineStr"/>
       <c r="I374" t="inlineStr">
         <is>
           <t>Algorithmic trading (DeFi)</t>
@@ -28410,7 +28340,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H375" t="inlineStr"/>
       <c r="I375" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -28562,7 +28491,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H377" t="inlineStr"/>
       <c r="I377" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -28600,7 +28528,6 @@
       </c>
     </row>
     <row r="378">
-      <c r="A378" t="inlineStr"/>
       <c r="B378" t="inlineStr">
         <is>
           <t>Fugle</t>
@@ -28674,7 +28601,6 @@
       </c>
     </row>
     <row r="379">
-      <c r="A379" t="inlineStr"/>
       <c r="B379" t="inlineStr">
         <is>
           <t>Compendium (PENDAX)</t>
@@ -28706,7 +28632,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H379" t="inlineStr"/>
       <c r="I379" t="inlineStr">
         <is>
           <t>Crypto trading technology</t>
@@ -28744,7 +28669,6 @@
       </c>
     </row>
     <row r="380">
-      <c r="A380" t="inlineStr"/>
       <c r="B380" t="inlineStr">
         <is>
           <t>Takin Profit</t>
@@ -28776,7 +28700,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H380" t="inlineStr"/>
       <c r="I380" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -28850,7 +28773,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H381" t="inlineStr"/>
       <c r="I381" t="inlineStr">
         <is>
           <t>Trading software (cTrader API)</t>
@@ -28924,7 +28846,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H382" t="inlineStr"/>
       <c r="I382" t="inlineStr">
         <is>
           <t>MT5 trading tools</t>
@@ -28998,7 +28919,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H383" t="inlineStr"/>
       <c r="I383" t="inlineStr">
         <is>
           <t>Crypto trading bot</t>
@@ -29072,7 +28992,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H384" t="inlineStr"/>
       <c r="I384" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -29146,7 +29065,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H385" t="inlineStr"/>
       <c r="I385" t="inlineStr">
         <is>
           <t>Forex market data tooling</t>
@@ -29298,7 +29216,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H387" t="inlineStr"/>
       <c r="I387" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -29336,7 +29253,6 @@
       </c>
     </row>
     <row r="388">
-      <c r="A388" t="inlineStr"/>
       <c r="B388" t="inlineStr">
         <is>
           <t>Resin (nullarch)</t>
@@ -29368,7 +29284,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H388" t="inlineStr"/>
       <c r="I388" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -29442,7 +29357,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H389" t="inlineStr"/>
       <c r="I389" t="inlineStr">
         <is>
           <t>Trading bot framework</t>
@@ -29480,7 +29394,6 @@
       </c>
     </row>
     <row r="390">
-      <c r="A390" t="inlineStr"/>
       <c r="B390" t="inlineStr">
         <is>
           <t>PineAuto</t>
@@ -29512,7 +29425,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H390" t="inlineStr"/>
       <c r="I390" t="inlineStr">
         <is>
           <t>Trading automation</t>
@@ -29550,7 +29462,6 @@
       </c>
     </row>
     <row r="391">
-      <c r="A391" t="inlineStr"/>
       <c r="B391" t="inlineStr">
         <is>
           <t>Saksh Trading Bot (sakshsky)</t>
@@ -29582,7 +29493,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H391" t="inlineStr"/>
       <c r="I391" t="inlineStr">
         <is>
           <t>Trading bot development</t>
@@ -29620,7 +29530,6 @@
       </c>
     </row>
     <row r="392">
-      <c r="A392" t="inlineStr"/>
       <c r="B392" t="inlineStr">
         <is>
           <t>AutoTrade Pro</t>
@@ -29653,7 +29562,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H392" t="inlineStr"/>
       <c r="I392" t="inlineStr">
         <is>
           <t>Trading automation software</t>
@@ -29691,7 +29599,6 @@
       </c>
     </row>
     <row r="393">
-      <c r="A393" t="inlineStr"/>
       <c r="B393" t="inlineStr">
         <is>
           <t>HOOX</t>
@@ -29724,7 +29631,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H393" t="inlineStr"/>
       <c r="I393" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -29762,7 +29668,6 @@
       </c>
     </row>
     <row r="394">
-      <c r="A394" t="inlineStr"/>
       <c r="B394" t="inlineStr">
         <is>
           <t>TradeClaw</t>
@@ -29794,7 +29699,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H394" t="inlineStr"/>
       <c r="I394" t="inlineStr">
         <is>
           <t>Trading signals / research</t>
@@ -29832,7 +29736,6 @@
       </c>
     </row>
     <row r="395">
-      <c r="A395" t="inlineStr"/>
       <c r="B395" t="inlineStr">
         <is>
           <t>Capital Trader</t>
@@ -29864,7 +29767,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H395" t="inlineStr"/>
       <c r="I395" t="inlineStr">
         <is>
           <t>Trading bot software</t>
@@ -29902,7 +29804,6 @@
       </c>
     </row>
     <row r="396">
-      <c r="A396" t="inlineStr"/>
       <c r="B396" t="inlineStr">
         <is>
           <t>OpenTrader</t>
@@ -29934,7 +29835,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H396" t="inlineStr"/>
       <c r="I396" t="inlineStr">
         <is>
           <t>Crypto trading bot software</t>
@@ -29972,7 +29872,6 @@
       </c>
     </row>
     <row r="397">
-      <c r="A397" t="inlineStr"/>
       <c r="B397" t="inlineStr">
         <is>
           <t>Siebly.io</t>
@@ -30004,7 +29903,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H397" t="inlineStr"/>
       <c r="I397" t="inlineStr">
         <is>
           <t>Exchange API SDKs</t>
@@ -30042,7 +29940,6 @@
       </c>
     </row>
     <row r="398">
-      <c r="A398" t="inlineStr"/>
       <c r="B398" t="inlineStr">
         <is>
           <t>Aether Wealth</t>
@@ -30074,7 +29971,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H398" t="inlineStr"/>
       <c r="I398" t="inlineStr">
         <is>
           <t>Trading journal / trading tools</t>
@@ -30148,7 +30044,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H399" t="inlineStr"/>
       <c r="I399" t="inlineStr">
         <is>
           <t>Trading software development</t>
@@ -30186,7 +30081,6 @@
       </c>
     </row>
     <row r="400">
-      <c r="A400" t="inlineStr"/>
       <c r="B400" t="inlineStr">
         <is>
           <t>Sentinel Bot</t>
@@ -30218,7 +30112,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H400" t="inlineStr"/>
       <c r="I400" t="inlineStr">
         <is>
           <t>Crypto trading bot platform</t>
@@ -30256,7 +30149,6 @@
       </c>
     </row>
     <row r="401">
-      <c r="A401" t="inlineStr"/>
       <c r="B401" t="inlineStr">
         <is>
           <t>Bitmate</t>
@@ -30288,7 +30180,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H401" t="inlineStr"/>
       <c r="I401" t="inlineStr">
         <is>
           <t>Algorithmic trading platform</t>
@@ -30326,7 +30217,6 @@
       </c>
     </row>
     <row r="402">
-      <c r="A402" t="inlineStr"/>
       <c r="B402" t="inlineStr">
         <is>
           <t>Clodds</t>
@@ -30358,7 +30248,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H402" t="inlineStr"/>
       <c r="I402" t="inlineStr">
         <is>
           <t>Trading terminal software</t>
@@ -30396,7 +30285,6 @@
       </c>
     </row>
     <row r="403">
-      <c r="A403" t="inlineStr"/>
       <c r="B403" t="inlineStr">
         <is>
           <t>QuantToGo</t>
@@ -30428,7 +30316,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H403" t="inlineStr"/>
       <c r="I403" t="inlineStr">
         <is>
           <t>Quantitative trading signals</t>
@@ -30466,7 +30353,6 @@
       </c>
     </row>
     <row r="404">
-      <c r="A404" t="inlineStr"/>
       <c r="B404" t="inlineStr">
         <is>
           <t>ctrader-ts</t>
@@ -30498,7 +30384,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H404" t="inlineStr"/>
       <c r="I404" t="inlineStr">
         <is>
           <t>Forex trading software</t>
@@ -30536,7 +30421,6 @@
       </c>
     </row>
     <row r="405">
-      <c r="A405" t="inlineStr"/>
       <c r="B405" t="inlineStr">
         <is>
           <t>Kiploks</t>
@@ -30568,7 +30452,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H405" t="inlineStr"/>
       <c r="I405" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -30642,7 +30525,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H406" t="inlineStr"/>
       <c r="I406" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -30680,7 +30562,6 @@
       </c>
     </row>
     <row r="407">
-      <c r="A407" t="inlineStr"/>
       <c r="B407" t="inlineStr">
         <is>
           <t>BacktestJS</t>
@@ -30712,7 +30593,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H407" t="inlineStr"/>
       <c r="I407" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -30786,7 +30666,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H408" t="inlineStr"/>
       <c r="I408" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -30824,7 +30703,6 @@
       </c>
     </row>
     <row r="409">
-      <c r="A409" t="inlineStr"/>
       <c r="B409" t="inlineStr">
         <is>
           <t>TradeCanvas</t>
@@ -30856,7 +30734,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H409" t="inlineStr"/>
       <c r="I409" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -30930,7 +30807,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H410" t="inlineStr"/>
       <c r="I410" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -30968,7 +30844,6 @@
       </c>
     </row>
     <row r="411">
-      <c r="A411" t="inlineStr"/>
       <c r="B411" t="inlineStr">
         <is>
           <t>ZapCli</t>
@@ -31000,7 +30875,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H411" t="inlineStr"/>
       <c r="I411" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -31116,7 +30990,6 @@
       </c>
     </row>
     <row r="413">
-      <c r="A413" t="inlineStr"/>
       <c r="B413" t="inlineStr">
         <is>
           <t>Traseq</t>
@@ -31148,7 +31021,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H413" t="inlineStr"/>
       <c r="I413" t="inlineStr">
         <is>
           <t>Algorithmic trading platform</t>
@@ -31186,7 +31058,6 @@
       </c>
     </row>
     <row r="414">
-      <c r="A414" t="inlineStr"/>
       <c r="B414" t="inlineStr">
         <is>
           <t>Pyon</t>
@@ -31218,7 +31089,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr">
         <is>
           <t>Algorithmic trading platform</t>
@@ -31256,7 +31126,6 @@
       </c>
     </row>
     <row r="415">
-      <c r="A415" t="inlineStr"/>
       <c r="B415" t="inlineStr">
         <is>
           <t>TradeJS</t>
@@ -31288,7 +31157,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H415" t="inlineStr"/>
       <c r="I415" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -31326,7 +31194,6 @@
       </c>
     </row>
     <row r="416">
-      <c r="A416" t="inlineStr"/>
       <c r="B416" t="inlineStr">
         <is>
           <t>Wickra</t>
@@ -31358,7 +31225,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H416" t="inlineStr"/>
       <c r="I416" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -31396,7 +31262,6 @@
       </c>
     </row>
     <row r="417">
-      <c r="A417" t="inlineStr"/>
       <c r="B417" t="inlineStr">
         <is>
           <t>FXAbsolute</t>
@@ -31428,7 +31293,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H417" t="inlineStr"/>
       <c r="I417" t="inlineStr">
         <is>
           <t>Forex data &amp; analytics</t>
@@ -31502,7 +31366,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H418" t="inlineStr"/>
       <c r="I418" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -31576,7 +31439,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H419" t="inlineStr"/>
       <c r="I419" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -31614,7 +31476,6 @@
       </c>
     </row>
     <row r="420">
-      <c r="A420" t="inlineStr"/>
       <c r="B420" t="inlineStr">
         <is>
           <t>Talocode (Tradia)</t>
@@ -31646,7 +31507,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H420" t="inlineStr"/>
       <c r="I420" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -31684,7 +31544,6 @@
       </c>
     </row>
     <row r="421">
-      <c r="A421" t="inlineStr"/>
       <c r="B421" t="inlineStr">
         <is>
           <t>ig-trading-mcp</t>
@@ -31716,7 +31575,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H421" t="inlineStr"/>
       <c r="I421" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -31754,7 +31612,6 @@
       </c>
     </row>
     <row r="422">
-      <c r="A422" t="inlineStr"/>
       <c r="B422" t="inlineStr">
         <is>
           <t>node-talib / NinjaScript MCP</t>
@@ -31786,7 +31643,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H422" t="inlineStr"/>
       <c r="I422" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -31824,7 +31680,6 @@
       </c>
     </row>
     <row r="423">
-      <c r="A423" t="inlineStr"/>
       <c r="B423" t="inlineStr">
         <is>
           <t>Stoqey</t>
@@ -31856,7 +31711,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H423" t="inlineStr"/>
       <c r="I423" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -31894,7 +31748,6 @@
       </c>
     </row>
     <row r="424">
-      <c r="A424" t="inlineStr"/>
       <c r="B424" t="inlineStr">
         <is>
           <t>Swift Tech Co.</t>
@@ -32004,7 +31857,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H425" t="inlineStr"/>
       <c r="I425" t="inlineStr">
         <is>
           <t>Trading automation</t>
@@ -32042,7 +31894,6 @@
       </c>
     </row>
     <row r="426">
-      <c r="A426" t="inlineStr"/>
       <c r="B426" t="inlineStr">
         <is>
           <t>Forex Bulgaria Academy</t>
@@ -32116,7 +31967,6 @@
       </c>
     </row>
     <row r="427">
-      <c r="A427" t="inlineStr"/>
       <c r="B427" t="inlineStr">
         <is>
           <t>Prophet Forex</t>
@@ -32148,7 +31998,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H427" t="inlineStr"/>
       <c r="I427" t="inlineStr">
         <is>
           <t>Forex AI tools</t>
@@ -32186,7 +32035,6 @@
       </c>
     </row>
     <row r="428">
-      <c r="A428" t="inlineStr"/>
       <c r="B428" t="inlineStr">
         <is>
           <t>MockTrade MCP</t>
@@ -32218,7 +32066,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H428" t="inlineStr"/>
       <c r="I428" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -32256,7 +32103,6 @@
       </c>
     </row>
     <row r="429">
-      <c r="A429" t="inlineStr"/>
       <c r="B429" t="inlineStr">
         <is>
           <t>developerzava</t>
@@ -32288,7 +32134,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H429" t="inlineStr"/>
       <c r="I429" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -32362,7 +32207,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H430" t="inlineStr"/>
       <c r="I430" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -32436,7 +32280,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H431" t="inlineStr"/>
       <c r="I431" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -32510,7 +32353,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H432" t="inlineStr"/>
       <c r="I432" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -32548,7 +32390,6 @@
       </c>
     </row>
     <row r="433">
-      <c r="A433" t="inlineStr"/>
       <c r="B433" t="inlineStr">
         <is>
           <t>ibkr-client</t>
@@ -32580,7 +32421,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H433" t="inlineStr"/>
       <c r="I433" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -32654,7 +32494,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H434" t="inlineStr"/>
       <c r="I434" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -32692,7 +32531,6 @@
       </c>
     </row>
     <row r="435">
-      <c r="A435" t="inlineStr"/>
       <c r="B435" t="inlineStr">
         <is>
           <t>CandleIQ (rukkiecodes)</t>
@@ -32724,7 +32562,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H435" t="inlineStr"/>
       <c r="I435" t="inlineStr">
         <is>
           <t>Trading tools</t>
@@ -32799,7 +32636,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H436" t="inlineStr"/>
       <c r="I436" t="inlineStr">
         <is>
           <t>Trading automation / Pine Script</t>
@@ -32916,7 +32752,6 @@
       </c>
     </row>
     <row r="438">
-      <c r="A438" t="inlineStr"/>
       <c r="B438" t="inlineStr">
         <is>
           <t>MWM AI</t>
@@ -33028,7 +32863,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H439" t="inlineStr"/>
       <c r="I439" t="inlineStr">
         <is>
           <t>Pine Script developer tooling</t>
@@ -33066,7 +32900,6 @@
       </c>
     </row>
     <row r="440">
-      <c r="A440" t="inlineStr"/>
       <c r="B440" t="inlineStr">
         <is>
           <t>Blueprint Research</t>
@@ -33099,7 +32932,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H440" t="inlineStr"/>
       <c r="I440" t="inlineStr">
         <is>
           <t>Trading indicators</t>
@@ -33174,7 +33006,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H441" t="inlineStr"/>
       <c r="I441" t="inlineStr">
         <is>
           <t>Crypto bot tooling</t>
@@ -33328,7 +33159,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H443" t="inlineStr"/>
       <c r="I443" t="inlineStr">
         <is>
           <t>Algo trading development</t>
@@ -33403,7 +33233,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H444" t="inlineStr"/>
       <c r="I444" t="inlineStr">
         <is>
           <t>Trading strategy development</t>
@@ -33441,7 +33270,6 @@
       </c>
     </row>
     <row r="445">
-      <c r="A445" t="inlineStr"/>
       <c r="B445" t="inlineStr">
         <is>
           <t>Shioaji Auto-Trading API</t>
@@ -33516,7 +33344,6 @@
       </c>
     </row>
     <row r="446">
-      <c r="A446" t="inlineStr"/>
       <c r="B446" t="inlineStr">
         <is>
           <t>trade-learn</t>
@@ -33549,7 +33376,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H446" t="inlineStr"/>
       <c r="I446" t="inlineStr">
         <is>
           <t>Backtesting framework</t>
@@ -33624,7 +33450,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H447" t="inlineStr"/>
       <c r="I447" t="inlineStr">
         <is>
           <t>Trading development</t>
@@ -33699,7 +33524,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H448" t="inlineStr"/>
       <c r="I448" t="inlineStr">
         <is>
           <t>TradingView alert relay</t>
@@ -33853,7 +33677,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H450" t="inlineStr"/>
       <c r="I450" t="inlineStr">
         <is>
           <t>Trading systems development</t>
@@ -33928,7 +33751,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H451" t="inlineStr"/>
       <c r="I451" t="inlineStr">
         <is>
           <t>TradingView indicators</t>
@@ -34003,7 +33825,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H452" t="inlineStr"/>
       <c r="I452" t="inlineStr">
         <is>
           <t>TradingView to MT5 automation</t>
@@ -34078,7 +33899,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H453" t="inlineStr"/>
       <c r="I453" t="inlineStr">
         <is>
           <t>MT5 hosting / deployment</t>
@@ -34116,7 +33936,6 @@
       </c>
     </row>
     <row r="454">
-      <c r="A454" t="inlineStr"/>
       <c r="B454" t="inlineStr">
         <is>
           <t>BarashTech</t>
@@ -34149,7 +33968,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H454" t="inlineStr"/>
       <c r="I454" t="inlineStr">
         <is>
           <t>Trading bot vendor</t>
@@ -34224,7 +34042,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H455" t="inlineStr"/>
       <c r="I455" t="inlineStr">
         <is>
           <t>Indicator development freelancing</t>
@@ -34299,7 +34116,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H456" t="inlineStr"/>
       <c r="I456" t="inlineStr">
         <is>
           <t>TradingView data tools</t>
@@ -34374,7 +34190,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H457" t="inlineStr"/>
       <c r="I457" t="inlineStr">
         <is>
           <t>Quant research / trading tools</t>
@@ -34449,7 +34264,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H458" t="inlineStr"/>
       <c r="I458" t="inlineStr">
         <is>
           <t>FinTech web development</t>
@@ -34487,7 +34301,6 @@
       </c>
     </row>
     <row r="459">
-      <c r="A459" t="inlineStr"/>
       <c r="B459" t="inlineStr">
         <is>
           <t>Darth Algo</t>
@@ -34520,7 +34333,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H459" t="inlineStr"/>
       <c r="I459" t="inlineStr">
         <is>
           <t>TradingView indicator subscriptions</t>
@@ -34595,7 +34407,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H460" t="inlineStr"/>
       <c r="I460" t="inlineStr">
         <is>
           <t>Crypto trading tools</t>
@@ -34749,7 +34560,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H462" t="inlineStr"/>
       <c r="I462" t="inlineStr">
         <is>
           <t>Backtesting &amp; indicator freelancing</t>
@@ -34903,7 +34713,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H464" t="inlineStr"/>
       <c r="I464" t="inlineStr">
         <is>
           <t>Trading tools / automation</t>
@@ -34978,7 +34787,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H465" t="inlineStr"/>
       <c r="I465" t="inlineStr">
         <is>
           <t>Pine Script freelancing</t>
@@ -35053,7 +34861,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H466" t="inlineStr"/>
       <c r="I466" t="inlineStr">
         <is>
           <t>Web3 &amp; trading platform development</t>
@@ -35207,7 +35014,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H468" t="inlineStr"/>
       <c r="I468" t="inlineStr">
         <is>
           <t>Trading bots &amp; automation</t>
@@ -35282,7 +35088,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H469" t="inlineStr"/>
       <c r="I469" t="inlineStr">
         <is>
           <t>Algorithmic trading development</t>
@@ -35515,7 +35320,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H472" t="inlineStr"/>
       <c r="I472" t="inlineStr">
         <is>
           <t>Trading systems services</t>
@@ -35590,7 +35394,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H473" t="inlineStr"/>
       <c r="I473" t="inlineStr">
         <is>
           <t>Trading signal engine</t>
@@ -35665,7 +35468,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H474" t="inlineStr"/>
       <c r="I474" t="inlineStr">
         <is>
           <t>MQL5 freelancing tools</t>
@@ -35703,7 +35505,6 @@
       </c>
     </row>
     <row r="475">
-      <c r="A475" t="inlineStr"/>
       <c r="B475" t="inlineStr">
         <is>
           <t>Asterix COM Ltd</t>
@@ -35736,7 +35537,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H475" t="inlineStr"/>
       <c r="I475" t="inlineStr">
         <is>
           <t>TradingView indicators</t>
@@ -35774,7 +35574,6 @@
       </c>
     </row>
     <row r="476">
-      <c r="A476" t="inlineStr"/>
       <c r="B476" t="inlineStr">
         <is>
           <t>Kryptofly</t>
@@ -35807,7 +35606,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H476" t="inlineStr"/>
       <c r="I476" t="inlineStr">
         <is>
           <t>Indicator &amp; strategy development</t>
@@ -35882,7 +35680,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H477" t="inlineStr"/>
       <c r="I477" t="inlineStr">
         <is>
           <t>Algorithmic trading development</t>
@@ -35920,7 +35717,6 @@
       </c>
     </row>
     <row r="478">
-      <c r="A478" t="inlineStr"/>
       <c r="B478" t="inlineStr">
         <is>
           <t>ClawedBot</t>
@@ -35953,7 +35749,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H478" t="inlineStr"/>
       <c r="I478" t="inlineStr">
         <is>
           <t>AI trading bot</t>
@@ -36107,7 +35902,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H480" t="inlineStr"/>
       <c r="I480" t="inlineStr">
         <is>
           <t>Forex trading tools</t>
@@ -36145,7 +35939,6 @@
       </c>
     </row>
     <row r="481">
-      <c r="A481" t="inlineStr"/>
       <c r="B481" t="inlineStr">
         <is>
           <t>Wagmigoats Trading Firm</t>
@@ -36220,7 +36013,6 @@
       </c>
     </row>
     <row r="482">
-      <c r="A482" t="inlineStr"/>
       <c r="B482" t="inlineStr">
         <is>
           <t>Jhay-M Trading Systems</t>
@@ -36253,7 +36045,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H482" t="inlineStr"/>
       <c r="I482" t="inlineStr">
         <is>
           <t>Trading systems engineering</t>
@@ -36407,7 +36198,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H484" t="inlineStr"/>
       <c r="I484" t="inlineStr">
         <is>
           <t>Trading journal software</t>
@@ -36482,7 +36272,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H485" t="inlineStr"/>
       <c r="I485" t="inlineStr">
         <is>
           <t>Pine Script &amp; trading bots</t>
@@ -36557,7 +36346,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H486" t="inlineStr"/>
       <c r="I486" t="inlineStr">
         <is>
           <t>Trading automation development</t>
@@ -36632,7 +36420,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H487" t="inlineStr"/>
       <c r="I487" t="inlineStr">
         <is>
           <t>Trading tools / signals</t>
@@ -36786,7 +36573,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H489" t="inlineStr"/>
       <c r="I489" t="inlineStr">
         <is>
           <t>Quant trading infrastructure</t>
@@ -36824,7 +36610,6 @@
       </c>
     </row>
     <row r="490">
-      <c r="A490" t="inlineStr"/>
       <c r="B490" t="inlineStr">
         <is>
           <t>sunshine-2-me</t>
@@ -36857,7 +36642,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H490" t="inlineStr"/>
       <c r="I490" t="inlineStr">
         <is>
           <t>Trading bot development</t>
@@ -36895,7 +36679,6 @@
       </c>
     </row>
     <row r="491">
-      <c r="A491" t="inlineStr"/>
       <c r="B491" t="inlineStr">
         <is>
           <t>MJH-devTW</t>
@@ -36970,7 +36753,6 @@
       </c>
     </row>
     <row r="492">
-      <c r="A492" t="inlineStr"/>
       <c r="B492" t="inlineStr">
         <is>
           <t>YismaFX</t>
@@ -37003,7 +36785,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H492" t="inlineStr"/>
       <c r="I492" t="inlineStr">
         <is>
           <t>Trading education</t>
@@ -37236,7 +37017,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H495" t="inlineStr"/>
       <c r="I495" t="inlineStr">
         <is>
           <t>Forex EA</t>
@@ -37274,7 +37054,6 @@
       </c>
     </row>
     <row r="496">
-      <c r="A496" t="inlineStr"/>
       <c r="B496" t="inlineStr">
         <is>
           <t>Hakimi Finance</t>
@@ -37307,7 +37086,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H496" t="inlineStr"/>
       <c r="I496" t="inlineStr">
         <is>
           <t>AI trading research</t>
@@ -37382,7 +37160,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H497" t="inlineStr"/>
       <c r="I497" t="inlineStr">
         <is>
           <t>Algorithmic trading platform</t>
@@ -37457,7 +37234,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H498" t="inlineStr"/>
       <c r="I498" t="inlineStr">
         <is>
           <t>Copy-trading software</t>
@@ -37611,7 +37387,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H500" t="inlineStr"/>
       <c r="I500" t="inlineStr">
         <is>
           <t>Trading bot development</t>
@@ -37686,7 +37461,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H501" t="inlineStr"/>
       <c r="I501" t="inlineStr">
         <is>
           <t>Trading technology / fintech engineering</t>
@@ -37724,7 +37498,6 @@
       </c>
     </row>
     <row r="502">
-      <c r="A502" t="inlineStr"/>
       <c r="B502" t="inlineStr">
         <is>
           <t>vatupelage (Rawana Holdings)</t>
@@ -37799,7 +37572,6 @@
       </c>
     </row>
     <row r="503">
-      <c r="A503" t="inlineStr"/>
       <c r="B503" t="inlineStr">
         <is>
           <t>CryptoQuantix</t>
@@ -37874,7 +37646,6 @@
       </c>
     </row>
     <row r="504">
-      <c r="A504" t="inlineStr"/>
       <c r="B504" t="inlineStr">
         <is>
           <t>AI Trading Bots Pro</t>
@@ -37907,7 +37678,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H504" t="inlineStr"/>
       <c r="I504" t="inlineStr">
         <is>
           <t>Crypto trading bot development</t>
@@ -37982,7 +37752,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H505" t="inlineStr"/>
       <c r="I505" t="inlineStr">
         <is>
           <t>Futures trading bots / signals</t>
@@ -38020,7 +37789,6 @@
       </c>
     </row>
     <row r="506">
-      <c r="A506" t="inlineStr"/>
       <c r="B506" t="inlineStr">
         <is>
           <t>Akier-X (FX Adaptive Trading System)</t>
@@ -38095,7 +37863,6 @@
       </c>
     </row>
     <row r="507">
-      <c r="A507" t="inlineStr"/>
       <c r="B507" t="inlineStr">
         <is>
           <t>Polymarket Copy Trading Bot &amp; Platform (CodeX2124)</t>
@@ -38128,7 +37895,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H507" t="inlineStr"/>
       <c r="I507" t="inlineStr">
         <is>
           <t>Copy-trading software</t>
@@ -38282,7 +38048,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H509" t="inlineStr"/>
       <c r="I509" t="inlineStr">
         <is>
           <t>AI trading agents</t>
@@ -38357,7 +38122,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H510" t="inlineStr"/>
       <c r="I510" t="inlineStr">
         <is>
           <t>Exchange API libraries</t>
@@ -38432,7 +38196,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H511" t="inlineStr"/>
       <c r="I511" t="inlineStr">
         <is>
           <t>AI trading terminal</t>
@@ -38470,7 +38233,6 @@
       </c>
     </row>
     <row r="512">
-      <c r="A512" t="inlineStr"/>
       <c r="B512" t="inlineStr">
         <is>
           <t>L2 Signals</t>
@@ -38503,7 +38265,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H512" t="inlineStr"/>
       <c r="I512" t="inlineStr">
         <is>
           <t>Forex signals / trading bots</t>
@@ -38541,7 +38302,6 @@
       </c>
     </row>
     <row r="513">
-      <c r="A513" t="inlineStr"/>
       <c r="B513" t="inlineStr">
         <is>
           <t>TrendSpider001 (Crypto Trading Bot Developer)</t>
@@ -38574,7 +38334,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H513" t="inlineStr"/>
       <c r="I513" t="inlineStr">
         <is>
           <t>Trading bot development</t>
@@ -38649,7 +38408,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H514" t="inlineStr"/>
       <c r="I514" t="inlineStr">
         <is>
           <t>Trading bot development</t>
@@ -38687,7 +38445,6 @@
       </c>
     </row>
     <row r="515">
-      <c r="A515" t="inlineStr"/>
       <c r="B515" t="inlineStr">
         <is>
           <t>Koam Analytics</t>
@@ -38762,7 +38519,6 @@
       </c>
     </row>
     <row r="516">
-      <c r="A516" t="inlineStr"/>
       <c r="B516" t="inlineStr">
         <is>
           <t>IrieTrade</t>
@@ -38795,7 +38551,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H516" t="inlineStr"/>
       <c r="I516" t="inlineStr">
         <is>
           <t>Automated trading software</t>
@@ -38833,7 +38588,6 @@
       </c>
     </row>
     <row r="517">
-      <c r="A517" t="inlineStr"/>
       <c r="B517" t="inlineStr">
         <is>
           <t>CopyPump</t>
@@ -38866,7 +38620,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H517" t="inlineStr"/>
       <c r="I517" t="inlineStr">
         <is>
           <t>Copy-trading infrastructure</t>
@@ -38904,7 +38657,6 @@
       </c>
     </row>
     <row r="518">
-      <c r="A518" t="inlineStr"/>
       <c r="B518" t="inlineStr">
         <is>
           <t>AutotradeX</t>
@@ -38979,7 +38731,6 @@
       </c>
     </row>
     <row r="519">
-      <c r="A519" t="inlineStr"/>
       <c r="B519" t="inlineStr">
         <is>
           <t>Apex-prim (freqtrade strategy audit)</t>
@@ -39012,7 +38763,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H519" t="inlineStr"/>
       <c r="I519" t="inlineStr">
         <is>
           <t>Strategy auditing</t>
@@ -39050,7 +38800,6 @@
       </c>
     </row>
     <row r="520">
-      <c r="A520" t="inlineStr"/>
       <c r="B520" t="inlineStr">
         <is>
           <t>NinjaTrader Smart Money Concept Bot</t>
@@ -39083,7 +38832,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H520" t="inlineStr"/>
       <c r="I520" t="inlineStr">
         <is>
           <t>Futures trading bots</t>
@@ -39121,7 +38869,6 @@
       </c>
     </row>
     <row r="521">
-      <c r="A521" t="inlineStr"/>
       <c r="B521" t="inlineStr">
         <is>
           <t>KERRIGAN Trading Lab</t>
@@ -39154,7 +38901,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H521" t="inlineStr"/>
       <c r="I521" t="inlineStr">
         <is>
           <t>Trading research software</t>
@@ -39192,7 +38938,6 @@
       </c>
     </row>
     <row r="522">
-      <c r="A522" t="inlineStr"/>
       <c r="B522" t="inlineStr">
         <is>
           <t>WIQON Lab</t>
@@ -39225,7 +38970,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H522" t="inlineStr"/>
       <c r="I522" t="inlineStr">
         <is>
           <t>Crypto strategy audits / custom bots</t>
@@ -39300,7 +39044,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H523" t="inlineStr"/>
       <c r="I523" t="inlineStr">
         <is>
           <t>Trading infrastructure engineering</t>
@@ -39375,7 +39118,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H524" t="inlineStr"/>
       <c r="I524" t="inlineStr">
         <is>
           <t>Grid bot tooling</t>
@@ -39492,7 +39234,6 @@
       </c>
     </row>
     <row r="526">
-      <c r="A526" t="inlineStr"/>
       <c r="B526" t="inlineStr">
         <is>
           <t>AxTrader (Asterix)</t>
@@ -39525,7 +39266,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H526" t="inlineStr"/>
       <c r="I526" t="inlineStr">
         <is>
           <t>Trading signals / education</t>
@@ -39563,7 +39303,6 @@
       </c>
     </row>
     <row r="527">
-      <c r="A527" t="inlineStr"/>
       <c r="B527" t="inlineStr">
         <is>
           <t>Profit Hub Expert (Benadesigns)</t>
@@ -39638,7 +39377,6 @@
       </c>
     </row>
     <row r="528">
-      <c r="A528" t="inlineStr"/>
       <c r="B528" t="inlineStr">
         <is>
           <t>CEX Option Futures Quant Trading Bot (yeahrb)</t>
@@ -39671,7 +39409,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H528" t="inlineStr"/>
       <c r="I528" t="inlineStr">
         <is>
           <t>Crypto trading bots</t>
@@ -39709,7 +39446,6 @@
       </c>
     </row>
     <row r="529">
-      <c r="A529" t="inlineStr"/>
       <c r="B529" t="inlineStr">
         <is>
           <t>Metadevxi</t>
@@ -39742,7 +39478,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H529" t="inlineStr"/>
       <c r="I529" t="inlineStr">
         <is>
           <t>Web3 / trading bot development</t>
@@ -39780,7 +39515,6 @@
       </c>
     </row>
     <row r="530">
-      <c r="A530" t="inlineStr"/>
       <c r="B530" t="inlineStr">
         <is>
           <t>bl0ckchaindev</t>
@@ -39813,7 +39547,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H530" t="inlineStr"/>
       <c r="I530" t="inlineStr">
         <is>
           <t>Trading bot development</t>
@@ -39930,7 +39663,6 @@
       </c>
     </row>
     <row r="532">
-      <c r="A532" t="inlineStr"/>
       <c r="B532" t="inlineStr">
         <is>
           <t>Sarff (freelance developer)</t>
@@ -40005,7 +39737,6 @@
       </c>
     </row>
     <row r="533">
-      <c r="A533" t="inlineStr"/>
       <c r="B533" t="inlineStr">
         <is>
           <t>fahamgeer177 (freelance AI/ML &amp; algo-trading)</t>
@@ -40117,7 +39848,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H534" t="inlineStr"/>
       <c r="I534" t="inlineStr">
         <is>
           <t>API integration / automation development</t>
@@ -40155,7 +39885,6 @@
       </c>
     </row>
     <row r="535">
-      <c r="A535" t="inlineStr"/>
       <c r="B535" t="inlineStr">
         <is>
           <t>Shtenco (Forex Arbitrage System for MT5)</t>
@@ -40188,7 +39917,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H535" t="inlineStr"/>
       <c r="I535" t="inlineStr">
         <is>
           <t>Forex algorithmic trading</t>
@@ -40226,7 +39954,6 @@
       </c>
     </row>
     <row r="536">
-      <c r="A536" t="inlineStr"/>
       <c r="B536" t="inlineStr">
         <is>
           <t>Portfolio Tracker 2.0</t>
@@ -40259,7 +39986,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H536" t="inlineStr"/>
       <c r="I536" t="inlineStr">
         <is>
           <t>Algo portfolio software</t>
@@ -40297,7 +40023,6 @@
       </c>
     </row>
     <row r="537">
-      <c r="A537" t="inlineStr"/>
       <c r="B537" t="inlineStr">
         <is>
           <t>AgentFxTrading</t>
@@ -40372,7 +40097,6 @@
       </c>
     </row>
     <row r="538">
-      <c r="A538" t="inlineStr"/>
       <c r="B538" t="inlineStr">
         <is>
           <t>La Brújula del Trader</t>
@@ -40405,7 +40129,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H538" t="inlineStr"/>
       <c r="I538" t="inlineStr">
         <is>
           <t>Trading journal / analytics</t>
@@ -40443,7 +40166,6 @@
       </c>
     </row>
     <row r="539">
-      <c r="A539" t="inlineStr"/>
       <c r="B539" t="inlineStr">
         <is>
           <t>Benjamin-cup (Polymarket bot developer)</t>
@@ -40476,7 +40198,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H539" t="inlineStr"/>
       <c r="I539" t="inlineStr">
         <is>
           <t>Prediction-market bot development</t>
@@ -40551,7 +40272,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H540" t="inlineStr"/>
       <c r="I540" t="inlineStr">
         <is>
           <t>Trading analysis bots</t>
@@ -40626,7 +40346,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H541" t="inlineStr"/>
       <c r="I541" t="inlineStr">
         <is>
           <t>Independent development (Web3 / trading systems)</t>
@@ -40664,7 +40383,6 @@
       </c>
     </row>
     <row r="542">
-      <c r="A542" t="inlineStr"/>
       <c r="B542" t="inlineStr">
         <is>
           <t>xyts (univquant)</t>
@@ -40697,7 +40415,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H542" t="inlineStr"/>
       <c r="I542" t="inlineStr">
         <is>
           <t>Low-latency trading frameworks</t>
@@ -40735,7 +40452,6 @@
       </c>
     </row>
     <row r="543">
-      <c r="A543" t="inlineStr"/>
       <c r="B543" t="inlineStr">
         <is>
           <t>Zerodha Market Connect Pro</t>
@@ -40810,7 +40526,6 @@
       </c>
     </row>
     <row r="544">
-      <c r="A544" t="inlineStr"/>
       <c r="B544" t="inlineStr">
         <is>
           <t>Arsenal VPS Trading System (precision9)</t>
@@ -40843,7 +40558,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H544" t="inlineStr"/>
       <c r="I544" t="inlineStr">
         <is>
           <t>Crypto futures trading systems</t>
@@ -40995,7 +40709,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H546" t="inlineStr"/>
       <c r="I546" t="inlineStr">
         <is>
           <t>Trading software (risk / discipline)</t>
@@ -41303,7 +41016,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H550" t="inlineStr"/>
       <c r="I550" t="inlineStr">
         <is>
           <t>Trading technology (futures research)</t>
@@ -41377,7 +41089,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H551" t="inlineStr"/>
       <c r="I551" t="inlineStr">
         <is>
           <t>Trading tools (futures API monitoring)</t>
@@ -41493,7 +41204,6 @@
       </c>
     </row>
     <row r="553">
-      <c r="A553" t="inlineStr"/>
       <c r="B553" t="inlineStr">
         <is>
           <t>Futures Edge Trade (Prop Firm Rules Dataset)</t>
@@ -41525,7 +41235,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H553" t="inlineStr"/>
       <c r="I553" t="inlineStr">
         <is>
           <t>Prop trading tools</t>
@@ -41599,7 +41308,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H554" t="inlineStr"/>
       <c r="I554" t="inlineStr">
         <is>
           <t>Quant research / futures</t>
@@ -41829,7 +41537,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H557" t="inlineStr"/>
       <c r="I557" t="inlineStr">
         <is>
           <t>Trading indicators (order flow)</t>
@@ -41903,7 +41610,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H558" t="inlineStr"/>
       <c r="I558" t="inlineStr">
         <is>
           <t>Trading software (charting &amp; setups)</t>
@@ -42019,7 +41725,6 @@
       </c>
     </row>
     <row r="560">
-      <c r="A560" t="inlineStr"/>
       <c r="B560" t="inlineStr">
         <is>
           <t>OTC Predictor</t>
@@ -42051,7 +41756,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H560" t="inlineStr"/>
       <c r="I560" t="inlineStr">
         <is>
           <t>Trading tools (Deriv synthetic indices)</t>
@@ -42125,7 +41829,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H561" t="inlineStr"/>
       <c r="I561" t="inlineStr">
         <is>
           <t>Trading tools (position sizing)</t>
@@ -42163,7 +41866,6 @@
       </c>
     </row>
     <row r="562">
-      <c r="A562" t="inlineStr"/>
       <c r="B562" t="inlineStr">
         <is>
           <t>ReeseLimitedLLC (Keystone AI &amp; ML)</t>
@@ -42237,7 +41939,6 @@
       </c>
     </row>
     <row r="563">
-      <c r="A563" t="inlineStr"/>
       <c r="B563" t="inlineStr">
         <is>
           <t>TuBot LATAM</t>
@@ -42269,7 +41970,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H563" t="inlineStr"/>
       <c r="I563" t="inlineStr">
         <is>
           <t>Trading indicators (NinjaTrader sales)</t>
@@ -42463,7 +42163,6 @@
       </c>
     </row>
     <row r="566">
-      <c r="A566" t="inlineStr"/>
       <c r="B566" t="inlineStr">
         <is>
           <t>Senior Trading &amp; Web Developer (Copytrading Bot Platform)</t>
@@ -42495,7 +42194,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H566" t="inlineStr"/>
       <c r="I566" t="inlineStr">
         <is>
           <t>Trade copier development</t>
@@ -42569,7 +42267,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H567" t="inlineStr"/>
       <c r="I567" t="inlineStr">
         <is>
           <t>Trading tools (spread research, cTrader)</t>
@@ -42643,7 +42340,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H568" t="inlineStr"/>
       <c r="I568" t="inlineStr">
         <is>
           <t>Trading automation (cTrader/AI)</t>
@@ -42717,7 +42413,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H569" t="inlineStr"/>
       <c r="I569" t="inlineStr">
         <is>
           <t>Trading signal automation (n8n/TradingView)</t>
@@ -42833,7 +42528,6 @@
       </c>
     </row>
     <row r="571">
-      <c r="A571" t="inlineStr"/>
       <c r="B571" t="inlineStr">
         <is>
           <t>Binary Bot &amp; Deriv Bot (Tr-reny)</t>
@@ -42865,7 +42559,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H571" t="inlineStr"/>
       <c r="I571" t="inlineStr">
         <is>
           <t>Trading bots (Deriv)</t>
@@ -42939,7 +42632,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H572" t="inlineStr"/>
       <c r="I572" t="inlineStr">
         <is>
           <t>Trading platform (Deriv)</t>
@@ -42977,7 +42669,6 @@
       </c>
     </row>
     <row r="573">
-      <c r="A573" t="inlineStr"/>
       <c r="B573" t="inlineStr">
         <is>
           <t>Deriv_Pro (Deriv Bots XML Collection)</t>
@@ -43009,7 +42700,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H573" t="inlineStr"/>
       <c r="I573" t="inlineStr">
         <is>
           <t>Trading bots (Deriv)</t>
@@ -43047,7 +42737,6 @@
       </c>
     </row>
     <row r="574">
-      <c r="A574" t="inlineStr"/>
       <c r="B574" t="inlineStr">
         <is>
           <t>Deriv Bot Academy (FrankFx)</t>
@@ -43079,7 +42768,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H574" t="inlineStr"/>
       <c r="I574" t="inlineStr">
         <is>
           <t>Trading bots (Deriv)</t>
@@ -43153,7 +42841,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H575" t="inlineStr"/>
       <c r="I575" t="inlineStr">
         <is>
           <t>Trading software (Alpaca starter)</t>
@@ -43227,7 +42914,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H576" t="inlineStr"/>
       <c r="I576" t="inlineStr">
         <is>
           <t>Algorithmic trading strategy development</t>
@@ -43301,7 +42987,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H577" t="inlineStr"/>
       <c r="I577" t="inlineStr">
         <is>
           <t>Futures research &amp; execution (Sierra Chart)</t>
@@ -43417,7 +43102,6 @@
       </c>
     </row>
     <row r="579">
-      <c r="A579" t="inlineStr"/>
       <c r="B579" t="inlineStr">
         <is>
           <t>QuantDIY (QuantX)</t>
@@ -43449,7 +43133,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H579" t="inlineStr"/>
       <c r="I579" t="inlineStr">
         <is>
           <t>Trading software (prop/futures)</t>
@@ -43487,7 +43170,6 @@
       </c>
     </row>
     <row r="580">
-      <c r="A580" t="inlineStr"/>
       <c r="B580" t="inlineStr">
         <is>
           <t>QuantForge IO</t>
@@ -43519,7 +43201,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H580" t="inlineStr"/>
       <c r="I580" t="inlineStr">
         <is>
           <t>cTrader development</t>
@@ -43593,7 +43274,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H581" t="inlineStr"/>
       <c r="I581" t="inlineStr">
         <is>
           <t>Trading automation (IBKR equities)</t>
@@ -43631,7 +43311,6 @@
       </c>
     </row>
     <row r="582">
-      <c r="A582" t="inlineStr"/>
       <c r="B582" t="inlineStr">
         <is>
           <t>AI FIX Parser</t>
@@ -43663,7 +43342,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H582" t="inlineStr"/>
       <c r="I582" t="inlineStr">
         <is>
           <t>Trading technology (FIX tooling)</t>
@@ -43737,7 +43415,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H583" t="inlineStr"/>
       <c r="I583" t="inlineStr">
         <is>
           <t>Prop trading tools (discipline app)</t>
@@ -43775,7 +43452,6 @@
       </c>
     </row>
     <row r="584">
-      <c r="A584" t="inlineStr"/>
       <c r="B584" t="inlineStr">
         <is>
           <t>ToolFleet</t>
@@ -43807,7 +43483,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H584" t="inlineStr"/>
       <c r="I584" t="inlineStr">
         <is>
           <t>Prop trading tools</t>
@@ -43881,7 +43556,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H585" t="inlineStr"/>
       <c r="I585" t="inlineStr">
         <is>
           <t>Trading bot development (crypto/forex)</t>
@@ -43919,7 +43593,6 @@
       </c>
     </row>
     <row r="586">
-      <c r="A586" t="inlineStr"/>
       <c r="B586" t="inlineStr">
         <is>
           <t>Bouchane (cTrader tools)</t>
@@ -43951,7 +43624,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H586" t="inlineStr"/>
       <c r="I586" t="inlineStr">
         <is>
           <t>Trading tools (cTrader)</t>
@@ -44025,7 +43697,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H587" t="inlineStr"/>
       <c r="I587" t="inlineStr">
         <is>
           <t>Algorithmic trading development</t>
@@ -44063,7 +43734,6 @@
       </c>
     </row>
     <row r="588">
-      <c r="A588" t="inlineStr"/>
       <c r="B588" t="inlineStr">
         <is>
           <t>IBF Trading (IBF Copy)</t>
@@ -44095,7 +43765,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H588" t="inlineStr"/>
       <c r="I588" t="inlineStr">
         <is>
           <t>Copy trading app (cTrader)</t>
@@ -44133,7 +43802,6 @@
       </c>
     </row>
     <row r="589">
-      <c r="A589" t="inlineStr"/>
       <c r="B589" t="inlineStr">
         <is>
           <t>Empire Noble North (Trading Journal Platform)</t>
@@ -44165,7 +43833,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H589" t="inlineStr"/>
       <c r="I589" t="inlineStr">
         <is>
           <t>Trading journal (cTrader Open API)</t>
@@ -44317,7 +43984,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H591" t="inlineStr"/>
       <c r="I591" t="inlineStr">
         <is>
           <t>Trading platform development (ProfitChart/NTSL)</t>
@@ -44391,7 +44057,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H592" t="inlineStr"/>
       <c r="I592" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -44465,7 +44130,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H593" t="inlineStr"/>
       <c r="I593" t="inlineStr">
         <is>
           <t>Trading software (IBKR)</t>
@@ -44503,7 +44167,6 @@
       </c>
     </row>
     <row r="594">
-      <c r="A594" t="inlineStr"/>
       <c r="B594" t="inlineStr">
         <is>
           <t>IBKR Trade AI</t>
@@ -44535,7 +44198,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H594" t="inlineStr"/>
       <c r="I594" t="inlineStr">
         <is>
           <t>Trading software (IBKR)</t>
@@ -44609,7 +44271,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H595" t="inlineStr"/>
       <c r="I595" t="inlineStr">
         <is>
           <t>Trading software (IBKR / TradingView)</t>
@@ -44683,7 +44344,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H596" t="inlineStr"/>
       <c r="I596" t="inlineStr">
         <is>
           <t>Crypto trading tooling</t>
@@ -44721,7 +44381,6 @@
       </c>
     </row>
     <row r="597">
-      <c r="A597" t="inlineStr"/>
       <c r="B597" t="inlineStr">
         <is>
           <t>topstep-backtest</t>
@@ -44753,7 +44412,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H597" t="inlineStr"/>
       <c r="I597" t="inlineStr">
         <is>
           <t>Prop-firm futures tooling</t>
@@ -44827,7 +44485,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H598" t="inlineStr"/>
       <c r="I598" t="inlineStr">
         <is>
           <t>Trading API tooling</t>
@@ -44865,7 +44522,6 @@
       </c>
     </row>
     <row r="599">
-      <c r="A599" t="inlineStr"/>
       <c r="B599" t="inlineStr">
         <is>
           <t>quantform</t>
@@ -44897,7 +44553,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H599" t="inlineStr"/>
       <c r="I599" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -45049,7 +44704,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H601" t="inlineStr"/>
       <c r="I601" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -45123,7 +44777,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H602" t="inlineStr"/>
       <c r="I602" t="inlineStr">
         <is>
           <t>Futures trading software</t>
@@ -45161,7 +44814,6 @@
       </c>
     </row>
     <row r="603">
-      <c r="A603" t="inlineStr"/>
       <c r="B603" t="inlineStr">
         <is>
           <t>StratEvo</t>
@@ -45193,7 +44845,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H603" t="inlineStr"/>
       <c r="I603" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -45231,7 +44882,6 @@
       </c>
     </row>
     <row r="604">
-      <c r="A604" t="inlineStr"/>
       <c r="B604" t="inlineStr">
         <is>
           <t>nsekit</t>
@@ -45305,7 +44955,6 @@
       </c>
     </row>
     <row r="605">
-      <c r="A605" t="inlineStr"/>
       <c r="B605" t="inlineStr">
         <is>
           <t>2oolkit (pacifica-cli)</t>
@@ -45337,7 +44986,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H605" t="inlineStr"/>
       <c r="I605" t="inlineStr">
         <is>
           <t>Crypto/derivatives trading tools</t>
@@ -45412,7 +45060,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H606" t="inlineStr"/>
       <c r="I606" t="inlineStr">
         <is>
           <t>Crypto trading bot</t>
@@ -45687,7 +45334,6 @@
       </c>
     </row>
     <row r="610">
-      <c r="A610" t="inlineStr"/>
       <c r="B610" t="inlineStr">
         <is>
           <t>dearolaf (Polymarket BTC 5-Minute Trading Bot)</t>
@@ -45720,7 +45366,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H610" t="inlineStr"/>
       <c r="I610" t="inlineStr">
         <is>
           <t>Prediction-market trading bots</t>
@@ -45758,7 +45403,6 @@
       </c>
     </row>
     <row r="611">
-      <c r="A611" t="inlineStr"/>
       <c r="B611" t="inlineStr">
         <is>
           <t>Barter (barter-rs)</t>
@@ -45791,7 +45435,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H611" t="inlineStr"/>
       <c r="I611" t="inlineStr">
         <is>
           <t>Algorithmic trading software</t>
@@ -45829,7 +45472,6 @@
       </c>
     </row>
     <row r="612">
-      <c r="A612" t="inlineStr"/>
       <c r="B612" t="inlineStr">
         <is>
           <t>Crypto Trade (the-crypto-trade)</t>
@@ -45862,7 +45504,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H612" t="inlineStr"/>
       <c r="I612" t="inlineStr">
         <is>
           <t>Crypto trading software</t>
@@ -45900,7 +45541,6 @@
       </c>
     </row>
     <row r="613">
-      <c r="A613" t="inlineStr"/>
       <c r="B613" t="inlineStr">
         <is>
           <t>Grid Manual Bot</t>
@@ -45933,7 +45573,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H613" t="inlineStr"/>
       <c r="I613" t="inlineStr">
         <is>
           <t>Crypto grid trading bots</t>
@@ -45971,7 +45610,6 @@
       </c>
     </row>
     <row r="614">
-      <c r="A614" t="inlineStr"/>
       <c r="B614" t="inlineStr">
         <is>
           <t>Nous Platform</t>
@@ -46004,7 +45642,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H614" t="inlineStr"/>
       <c r="I614" t="inlineStr">
         <is>
           <t>Crypto trading terminal</t>
@@ -46042,7 +45679,6 @@
       </c>
     </row>
     <row r="615">
-      <c r="A615" t="inlineStr"/>
       <c r="B615" t="inlineStr">
         <is>
           <t>Kinetix AI Trading Terminal (masanidev)</t>
@@ -46075,7 +45711,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H615" t="inlineStr"/>
       <c r="I615" t="inlineStr">
         <is>
           <t>Crypto trading SaaS</t>
@@ -46113,7 +45748,6 @@
       </c>
     </row>
     <row r="616">
-      <c r="A616" t="inlineStr"/>
       <c r="B616" t="inlineStr">
         <is>
           <t>Ares Aegis</t>
@@ -46146,7 +45780,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H616" t="inlineStr"/>
       <c r="I616" t="inlineStr">
         <is>
           <t>Crypto futures trading platform</t>
@@ -46221,7 +45854,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H617" t="inlineStr"/>
       <c r="I617" t="inlineStr">
         <is>
           <t>Crypto quant SaaS</t>
@@ -46259,7 +45891,6 @@
       </c>
     </row>
     <row r="618">
-      <c r="A618" t="inlineStr"/>
       <c r="B618" t="inlineStr">
         <is>
           <t>Crypto Autotrader</t>
@@ -46292,7 +45923,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H618" t="inlineStr"/>
       <c r="I618" t="inlineStr">
         <is>
           <t>Crypto trading bots</t>
@@ -46367,7 +45997,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H619" t="inlineStr"/>
       <c r="I619" t="inlineStr">
         <is>
           <t>Freqtrade tooling</t>
@@ -46442,7 +46071,6 @@
 Trading Bot Developer</t>
         </is>
       </c>
-      <c r="H620" t="inlineStr"/>
       <c r="I620" t="inlineStr">
         <is>
           <t>Broker API tooling</t>
@@ -46558,7 +46186,6 @@
       </c>
     </row>
     <row r="622">
-      <c r="A622" t="inlineStr"/>
       <c r="B622" t="inlineStr">
         <is>
           <t>Marc (MNQ systematic trading)</t>

</xml_diff>

<commit_message>
Outreach batch 4: final 12 sent, queue complete
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -8502,7 +8502,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -8585,7 +8585,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -8668,7 +8668,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -8997,7 +8997,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -9075,7 +9075,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -9149,7 +9149,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -9222,7 +9222,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -9300,7 +9300,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Queued (round 2)</t>
+          <t>Sent 2026-09-29 00:37 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">

</xml_diff>

<commit_message>
Outreach batch: 24 sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -9450,6 +9450,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H116" t="inlineStr">
         <is>
           <t>Estonia</t>
@@ -9528,6 +9533,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H117" t="inlineStr">
         <is>
           <t>Brazil</t>
@@ -9604,6 +9614,11 @@
 Best regards,
 Oseni Ibrahim
 Trading Bot Developer</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -9675,6 +9690,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H119" t="inlineStr">
         <is>
           <t>Cambodia</t>
@@ -9754,6 +9774,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I120" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -9827,6 +9852,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I121" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -9900,6 +9930,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I122" t="inlineStr">
         <is>
           <t>Fintech / blockchain development</t>
@@ -9973,6 +10008,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H123" t="inlineStr">
         <is>
           <t>Indonesia</t>
@@ -10051,6 +10091,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H124" t="inlineStr">
         <is>
           <t>Brazil</t>
@@ -10124,6 +10169,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I125" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -10197,6 +10247,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I126" t="inlineStr">
         <is>
           <t>Software / trading tools</t>
@@ -10265,6 +10320,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I127" t="inlineStr">
         <is>
           <t>Proprietary quantitative trading</t>
@@ -10333,6 +10393,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H128" t="inlineStr">
         <is>
           <t>India</t>
@@ -10406,6 +10471,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I129" t="inlineStr">
         <is>
           <t>Trading tools / custom development</t>
@@ -10474,6 +10544,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H130" t="inlineStr">
         <is>
           <t>Italy</t>
@@ -10547,6 +10622,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I131" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10615,6 +10695,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I132" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10683,6 +10768,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10751,6 +10841,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Skipped already contacted (2026-09-29 17:01 UTC)</t>
+        </is>
+      </c>
       <c r="H134" t="inlineStr">
         <is>
           <t>United States</t>
@@ -10829,6 +10924,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H135" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -10902,6 +11002,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -10970,6 +11075,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I137" t="inlineStr">
         <is>
           <t>Forex brokerage technology</t>
@@ -11038,6 +11148,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -11106,6 +11221,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I139" t="inlineStr">
         <is>
           <t>AI trading systems</t>
@@ -11177,6 +11297,11 @@
 Best regards,
 Oseni Ibrahim
 Trading Bot Developer</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">

</xml_diff>

<commit_message>
Outreach batch: 25 sent; 1 bounce recorded
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -9452,7 +9452,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Sent 2026-09-29 17:01 UTC from oseniibrahim845@gmail.com</t>
+          <t>Bounced (2026-09-30 01:27 UTC)</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -11382,6 +11382,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I141" t="inlineStr">
         <is>
           <t>Trading systems</t>
@@ -11455,6 +11460,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I142" t="inlineStr">
         <is>
           <t>Trading software</t>
@@ -11528,6 +11538,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H143" t="inlineStr">
         <is>
           <t>United Arab Emirates</t>
@@ -11606,6 +11621,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H144" t="inlineStr">
         <is>
           <t>Indonesia</t>
@@ -11684,6 +11704,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H145" t="inlineStr">
         <is>
           <t>Oman</t>
@@ -11762,6 +11787,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H146" t="inlineStr">
         <is>
           <t>India</t>
@@ -11840,6 +11870,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I147" t="inlineStr">
         <is>
           <t>Software development</t>
@@ -11913,6 +11948,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I148" t="inlineStr">
         <is>
           <t>Trading framework</t>
@@ -11981,6 +12021,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I149" t="inlineStr">
         <is>
           <t>MT5 trade management tools</t>
@@ -12054,6 +12099,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H150" t="inlineStr">
         <is>
           <t>Brazil</t>
@@ -12132,6 +12182,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H151" t="inlineStr">
         <is>
           <t>Ukraine</t>
@@ -12205,6 +12260,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I152" t="inlineStr">
         <is>
           <t>Freelance trading software</t>
@@ -12278,6 +12338,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H153" t="inlineStr">
         <is>
           <t>Colombia</t>
@@ -12351,6 +12416,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I154" t="inlineStr">
         <is>
           <t>Freelance software development</t>
@@ -12424,6 +12494,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I155" t="inlineStr">
         <is>
           <t>Trading indicators</t>
@@ -12497,6 +12572,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I156" t="inlineStr">
         <is>
           <t>Trading education</t>
@@ -12570,6 +12650,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H157" t="inlineStr">
         <is>
           <t>Indonesia</t>
@@ -12648,6 +12733,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I158" t="inlineStr">
         <is>
           <t>MQL developer tooling</t>
@@ -12716,6 +12806,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I159" t="inlineStr">
         <is>
           <t>MQL5 libraries</t>
@@ -12789,6 +12884,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I160" t="inlineStr">
         <is>
           <t>Trading strategy development</t>
@@ -12862,6 +12962,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I161" t="inlineStr">
         <is>
           <t>Software development</t>
@@ -12935,6 +13040,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I162" t="inlineStr">
         <is>
           <t>Quant research</t>
@@ -13008,6 +13118,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H163" t="inlineStr">
         <is>
           <t>Kenya</t>
@@ -13081,6 +13196,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I164" t="inlineStr">
         <is>
           <t>AI trading systems</t>
@@ -13147,6 +13267,11 @@
 Best regards,
 Oseni Ibrahim
 Trading Bot Developer</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 01:28 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">

</xml_diff>

<commit_message>
Outreach batch: 25 sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NzbUqn2rPYzKggdY77vhWH
</commit_message>
<xml_diff>
--- a/EA_Trading_Bot_Prospects_500.xlsx
+++ b/EA_Trading_Bot_Prospects_500.xlsx
@@ -13352,6 +13352,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I166" t="inlineStr">
         <is>
           <t>Algorithmic trading</t>
@@ -13425,6 +13430,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H167" t="inlineStr">
         <is>
           <t>United States</t>
@@ -13496,6 +13506,11 @@
 Best regards,
 Oseni Ibrahim
 Trading Bot Developer</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -13572,6 +13587,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I169" t="inlineStr">
         <is>
           <t>Trading technology</t>
@@ -13646,6 +13666,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H170" t="inlineStr">
         <is>
           <t>Zimbabwe</t>
@@ -13725,6 +13750,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H171" t="inlineStr">
         <is>
           <t>Pakistan</t>
@@ -13804,6 +13834,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H172" t="inlineStr">
         <is>
           <t>Dominican Republic</t>
@@ -13883,6 +13918,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H173" t="inlineStr">
         <is>
           <t>Canada</t>
@@ -13962,6 +14002,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H174" t="inlineStr">
         <is>
           <t>Indonesia</t>
@@ -14036,6 +14081,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H175" t="inlineStr">
         <is>
           <t>Russia</t>
@@ -14110,6 +14160,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I176" t="inlineStr">
         <is>
           <t>Forex EA software</t>
@@ -14183,6 +14238,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H177" t="inlineStr">
         <is>
           <t>Indonesia</t>
@@ -14261,6 +14321,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H178" t="inlineStr">
         <is>
           <t>Tanzania</t>
@@ -14339,6 +14404,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H179" t="inlineStr">
         <is>
           <t>Argentina</t>
@@ -14417,6 +14487,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H180" t="inlineStr">
         <is>
           <t>Lebanon</t>
@@ -14495,6 +14570,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H181" t="inlineStr">
         <is>
           <t>Colombia</t>
@@ -14573,6 +14653,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H182" t="inlineStr">
         <is>
           <t>Azerbaijan</t>
@@ -14651,6 +14736,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I183" t="inlineStr">
         <is>
           <t>Trading software / fintech UI</t>
@@ -14724,6 +14814,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H184" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -14802,6 +14897,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H185" t="inlineStr">
         <is>
           <t>Nigeria</t>
@@ -14880,6 +14980,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H186" t="inlineStr">
         <is>
           <t>Spain</t>
@@ -14958,6 +15063,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I187" t="inlineStr">
         <is>
           <t>Quantitative trading</t>
@@ -15031,6 +15141,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="H188" t="inlineStr">
         <is>
           <t>India</t>
@@ -15104,6 +15219,11 @@
 Trading Bot Developer</t>
         </is>
       </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
+        </is>
+      </c>
       <c r="I189" t="inlineStr">
         <is>
           <t>Trading software / backtesting</t>
@@ -15175,6 +15295,11 @@
 Best regards,
 Oseni Ibrahim
 Trading Bot Developer</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Sent 2026-09-30 05:00 UTC from oseniibrahim845@gmail.com</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">

</xml_diff>